<commit_message>
Fix Spanish category labels leaking into an Italian catalog
CATEGORY_RULES stored the internal matching label (e.g. "sofás",
"sillones", "mesas") directly as product.category and
alternatives_group - Spanish, even though prompt.md forces the
assistant's own prose to Italian. Client feedback (Andrea, Febal
Casa): a client testing the assistant saw Spanish words and asked why.

Relabeled every category to Italian (divani, poltrone, tavoli, ...).
Multilingual search coverage (a visitor typing "sofa" or "sillón")
still works exactly as before via CATEGORY_SYNONYMS, now keyed by the
Italian label instead of mixing languages into the stored value
itself. Regenerated clients/febal-casa/catalog.json(.full)/.xlsx via
build-febal-catalog.mjs - all 95 records rebuilt, same coordinates and
images, only the category strings changed.
</commit_message>
<xml_diff>
--- a/clients/febal-casa/catalog.xlsx
+++ b/clients/febal-casa/catalog.xlsx
@@ -463,10 +463,10 @@
         <v>Boiserie camino</v>
       </c>
       <c r="C2" t="str">
-        <v>paneles decorativos</v>
+        <v>boiserie</v>
       </c>
       <c r="D2" t="str">
-        <v>La parete attrezzata boiserie è concepita come un sistema in grado di dialogare con tutti gli altri arredi della gamma Febal Casa</v>
+        <v>La boiserie è concepita come un sistema in grado di dialogare con tutti gli altri arredi della gamma Febal Casa, un elemento versatile che si innesta con soluzione di continuità arrivando fino a terra.</v>
       </c>
       <c r="E2" t="str">
         <v/>
@@ -475,7 +475,7 @@
         <v/>
       </c>
       <c r="G2" t="str">
-        <v>boiserie, camino, paneles decorativos, panel, revestimiento, pared, decorativo, columna, vertical, parete, attrezzata, concepita, sistema, grado, dialogare, tutti, altri, arredi, gamma, febal</v>
+        <v>boiserie, camino, panel, paneles decorativos, revestimiento, pared, decorativo, columna, vertical, concepita, sistema, grado, dialogare, tutti, altri, arredi, gamma, febal, casa, elemento</v>
       </c>
       <c r="H2" t="str">
         <v/>
@@ -505,7 +505,7 @@
         <v>https://www.febalcasa.com/it/prodotti/boiserie/</v>
       </c>
       <c r="Q2" t="str">
-        <v>paneles-decorativos</v>
+        <v>boiserie</v>
       </c>
       <c r="R2" t="str">
         <v>TRUE</v>
@@ -519,10 +519,10 @@
         <v>Boiserie</v>
       </c>
       <c r="C3" t="str">
-        <v>paneles decorativos</v>
+        <v>boiserie</v>
       </c>
       <c r="D3" t="str">
-        <v>La parete attrezzata boiserie è concepita come un sistema in grado di dialogare con tutti gli altri arredi della gamma Febal Casa</v>
+        <v>La boiserie è concepita come un sistema in grado di dialogare con tutti gli altri arredi della gamma Febal Casa, un elemento versatile che si innesta con soluzione di continuità arrivando fino a terra.</v>
       </c>
       <c r="E3" t="str">
         <v/>
@@ -531,7 +531,7 @@
         <v/>
       </c>
       <c r="G3" t="str">
-        <v>boiserie, paneles decorativos, panel, revestimiento, pared, decorativo, columna, vertical, parete, attrezzata, concepita, sistema, grado, dialogare, tutti, altri, arredi, gamma, febal</v>
+        <v>boiserie, panel, paneles decorativos, revestimiento, pared, decorativo, columna, vertical, concepita, sistema, grado, dialogare, tutti, altri, arredi, gamma, febal, casa, elemento</v>
       </c>
       <c r="H3" t="str">
         <v/>
@@ -561,7 +561,7 @@
         <v>https://www.febalcasa.com/it/prodotti/boiserie/</v>
       </c>
       <c r="Q3" t="str">
-        <v>paneles-decorativos</v>
+        <v>boiserie</v>
       </c>
       <c r="R3" t="str">
         <v>TRUE</v>
@@ -575,7 +575,7 @@
         <v>Divano Balmoral</v>
       </c>
       <c r="C4" t="str">
-        <v>sofás</v>
+        <v>divani</v>
       </c>
       <c r="D4" t="str">
         <v>Un divano componibile pensato per interpretare le esigenze abitative contemporanee, coniugando estetica, ergonomia e versatilità. La scelta ideale per un soggiorno elegante, accogliente e su misura.</v>
@@ -587,7 +587,7 @@
         <v/>
       </c>
       <c r="G4" t="str">
-        <v>divano, balmoral, sofás, sofa, sofá, couch, asiento, componibile, pensato, interpretare, esigenze, abitative, contemporanee, coniugando, estetica, ergonomia, versatilita, scelta</v>
+        <v>divano, balmoral, divani, sofa, sofá, sofás, couch, asiento, componibile, pensato, interpretare, esigenze, abitative, contemporanee, coniugando, estetica, ergonomia, versatilita, scelta</v>
       </c>
       <c r="H4" t="str">
         <v/>
@@ -617,7 +617,7 @@
         <v>https://www.febalcasa.com/it/prodotti/balmoral/</v>
       </c>
       <c r="Q4" t="str">
-        <v>sofas</v>
+        <v>divani</v>
       </c>
       <c r="R4" t="str">
         <v>TRUE</v>
@@ -631,10 +631,10 @@
         <v>Tavolino Rio</v>
       </c>
       <c r="C5" t="str">
-        <v>mesas de centro</v>
+        <v>tavolini</v>
       </c>
       <c r="D5" t="str">
-        <v>Il tavolino Rio è contraddistinto da una struttura in metallo che presenta la particolarità di poter accogliere riviste e giornali. Una funzione che lo rende</v>
+        <v>Il tavolino Rio è contraddistinto da una struttura in metallo che presenta la particolarità di poter accogliere riviste e giornali. Una funzione che lo rende il compagno ideale nei momenti di relax. Il piano può essere configurato a seconda del proprio gusto in finitura laccata opaca o impiallacciata.</v>
       </c>
       <c r="E5" t="str">
         <v/>
@@ -643,7 +643,7 @@
         <v/>
       </c>
       <c r="G5" t="str">
-        <v>tavolino, rio, mesas de centro, mesa de centro, mesita, coffee table, contraddistinto, struttura, metallo, presenta, particolarita, poter, accogliere, riviste, giornali, funzione, rende</v>
+        <v>tavolino, rio, tavolini, mesa de centro, mesita, coffee table, contraddistinto, struttura, metallo, presenta, particolarita, poter, accogliere, riviste, giornali, funzione, rende</v>
       </c>
       <c r="H5" t="str">
         <v/>
@@ -673,7 +673,7 @@
         <v>https://www.febalcasa.com/it/prodotti/rio/</v>
       </c>
       <c r="Q5" t="str">
-        <v>mesas-de-centro</v>
+        <v>tavolini</v>
       </c>
       <c r="R5" t="str">
         <v>TRUE</v>
@@ -687,10 +687,10 @@
         <v>Tavolino Rio</v>
       </c>
       <c r="C6" t="str">
-        <v>mesas de centro</v>
+        <v>tavolini</v>
       </c>
       <c r="D6" t="str">
-        <v>Il tavolino Rio è contraddistinto da una struttura in metallo che presenta la particolarità di poter accogliere riviste e giornali. Una funzione che lo rende</v>
+        <v>Il tavolino Rio è contraddistinto da una struttura in metallo che presenta la particolarità di poter accogliere riviste e giornali. Una funzione che lo rende il compagno ideale nei momenti di relax. Il piano può essere configurato a seconda del proprio gusto in finitura laccata opaca o impiallacciata.</v>
       </c>
       <c r="E6" t="str">
         <v/>
@@ -699,7 +699,7 @@
         <v/>
       </c>
       <c r="G6" t="str">
-        <v>tavolino, rio, mesas de centro, mesa de centro, mesita, coffee table, contraddistinto, struttura, metallo, presenta, particolarita, poter, accogliere, riviste, giornali, funzione, rende</v>
+        <v>tavolino, rio, tavolini, mesa de centro, mesita, coffee table, contraddistinto, struttura, metallo, presenta, particolarita, poter, accogliere, riviste, giornali, funzione, rende</v>
       </c>
       <c r="H6" t="str">
         <v/>
@@ -729,7 +729,7 @@
         <v>https://www.febalcasa.com/it/prodotti/rio/</v>
       </c>
       <c r="Q6" t="str">
-        <v>mesas-de-centro</v>
+        <v>tavolini</v>
       </c>
       <c r="R6" t="str">
         <v>TRUE</v>
@@ -743,10 +743,10 @@
         <v>Boiserie</v>
       </c>
       <c r="C7" t="str">
-        <v>paneles decorativos</v>
+        <v>boiserie</v>
       </c>
       <c r="D7" t="str">
-        <v>La parete attrezzata boiserie è concepita come un sistema in grado di dialogare con tutti gli altri arredi della gamma Febal Casa</v>
+        <v>La boiserie è concepita come un sistema in grado di dialogare con tutti gli altri arredi della gamma Febal Casa, un elemento versatile che si innesta con soluzione di continuità arrivando fino a terra.</v>
       </c>
       <c r="E7" t="str">
         <v/>
@@ -755,7 +755,7 @@
         <v/>
       </c>
       <c r="G7" t="str">
-        <v>boiserie, paneles decorativos, panel, revestimiento, pared, decorativo, columna, vertical, parete, attrezzata, concepita, sistema, grado, dialogare, tutti, altri, arredi, gamma, febal</v>
+        <v>boiserie, panel, paneles decorativos, revestimiento, pared, decorativo, columna, vertical, concepita, sistema, grado, dialogare, tutti, altri, arredi, gamma, febal, casa, elemento</v>
       </c>
       <c r="H7" t="str">
         <v/>
@@ -785,7 +785,7 @@
         <v>https://www.febalcasa.com/it/prodotti/boiserie/</v>
       </c>
       <c r="Q7" t="str">
-        <v>paneles-decorativos</v>
+        <v>boiserie</v>
       </c>
       <c r="R7" t="str">
         <v>TRUE</v>
@@ -799,7 +799,7 @@
         <v>Cucina Origina Anta Square Cannettato</v>
       </c>
       <c r="C8" t="str">
-        <v>cocinas</v>
+        <v>cucine</v>
       </c>
       <c r="D8" t="str">
         <v>Cucina Origina Anta Square Cannettato — pieza de la colección Febal Casa, sección CASA 01 - AUTENTICA.</v>
@@ -811,7 +811,7 @@
         <v/>
       </c>
       <c r="G8" t="str">
-        <v>cucina, origina, anta, square, cannettato, cocinas, cocina, kitchen, isla, casa, pieza, coleccion, febal, seccion, autentica</v>
+        <v>cucina, origina, anta, square, cannettato, cucine, cocina, cocinas, kitchen, isla, casa, pieza, coleccion, febal, seccion, autentica</v>
       </c>
       <c r="H8" t="str">
         <v/>
@@ -841,7 +841,7 @@
         <v>https://www.febalcasa.com/it/prodotti/origina-anta-square-cannettato/</v>
       </c>
       <c r="Q8" t="str">
-        <v>cocinas</v>
+        <v>cucine</v>
       </c>
       <c r="R8" t="str">
         <v>TRUE</v>
@@ -855,7 +855,7 @@
         <v>Sistema Origina</v>
       </c>
       <c r="C9" t="str">
-        <v>sistemas modulares</v>
+        <v>sistemi modulari</v>
       </c>
       <c r="D9" t="str">
         <v>Sistema Origina — pieza de la colección Febal Casa, sección CASA 01 - AUTENTICA.</v>
@@ -867,7 +867,7 @@
         <v/>
       </c>
       <c r="G9" t="str">
-        <v>sistema, origina, sistemas modulares, sistema modular, modular, casa, pieza, coleccion, febal, seccion, autentica</v>
+        <v>sistema, origina, sistemi modulari, sistema modular, sistemas modulares, modular, casa, pieza, coleccion, febal, seccion, autentica</v>
       </c>
       <c r="H9" t="str">
         <v/>
@@ -897,7 +897,7 @@
         <v>https://www.febalcasa.com/it/prodotti/origina-anta-square-cannettato/</v>
       </c>
       <c r="Q9" t="str">
-        <v>sistemas-modulares</v>
+        <v>sistemi-modulari</v>
       </c>
       <c r="R9" t="str">
         <v>TRUE</v>
@@ -911,7 +911,7 @@
         <v>Sistema Origina</v>
       </c>
       <c r="C10" t="str">
-        <v>sistemas modulares</v>
+        <v>sistemi modulari</v>
       </c>
       <c r="D10" t="str">
         <v>Sistema Origina — pieza de la colección Febal Casa, sección CASA 01 - AUTENTICA.</v>
@@ -923,7 +923,7 @@
         <v/>
       </c>
       <c r="G10" t="str">
-        <v>sistema, origina, sistemas modulares, sistema modular, modular, casa, pieza, coleccion, febal, seccion, autentica</v>
+        <v>sistema, origina, sistemi modulari, sistema modular, sistemas modulares, modular, casa, pieza, coleccion, febal, seccion, autentica</v>
       </c>
       <c r="H10" t="str">
         <v/>
@@ -953,7 +953,7 @@
         <v>https://www.febalcasa.com/it/prodotti/origina-anta-square-cannettato/</v>
       </c>
       <c r="Q10" t="str">
-        <v>sistemas-modulares</v>
+        <v>sistemi-modulari</v>
       </c>
       <c r="R10" t="str">
         <v>TRUE</v>
@@ -967,7 +967,7 @@
         <v>Sistema Diciotto</v>
       </c>
       <c r="C11" t="str">
-        <v>sistemas modulares</v>
+        <v>sistemi modulari</v>
       </c>
       <c r="D11" t="str">
         <v>Diciotto è una parete attrezzata per la zona living di design: pratico, versatile e funzionale permette una modularità altissima.</v>
@@ -979,7 +979,7 @@
         <v/>
       </c>
       <c r="G11" t="str">
-        <v>sistema, diciotto, sistemas modulares, sistema modular, modular, parete, attrezzata, zona, living, design, pratico, versatile, funzionale, permette, modularita, altissima</v>
+        <v>sistema, diciotto, sistemi modulari, sistema modular, sistemas modulares, modular, parete, attrezzata, zona, living, design, pratico, versatile, funzionale, permette, modularita, altissima</v>
       </c>
       <c r="H11" t="str">
         <v/>
@@ -1009,7 +1009,7 @@
         <v>https://www.febalcasa.com/it/prodotti/diciotto/</v>
       </c>
       <c r="Q11" t="str">
-        <v>sistemas-modulares</v>
+        <v>sistemi-modulari</v>
       </c>
       <c r="R11" t="str">
         <v>TRUE</v>
@@ -1023,7 +1023,7 @@
         <v>Libreria Trenta</v>
       </c>
       <c r="C12" t="str">
-        <v>librerías</v>
+        <v>librerie</v>
       </c>
       <c r="D12" t="str">
         <v>Trenta è la libreria interpretata da Febal Casa come elemento chiave intorno cui viene progettata la zona giorno.</v>
@@ -1035,7 +1035,7 @@
         <v/>
       </c>
       <c r="G12" t="str">
-        <v>libreria, trenta, librerías, librería, estanteria, estantería, bookshelf, estante, interpretata, febal, casa, elemento, chiave, intorno, viene, progettata, zona, giorno</v>
+        <v>libreria, trenta, librerie, librería, librerías, estanteria, estantería, bookshelf, estante, interpretata, febal, casa, elemento, chiave, intorno, viene, progettata, zona, giorno</v>
       </c>
       <c r="H12" t="str">
         <v/>
@@ -1065,7 +1065,7 @@
         <v>https://www.febalcasa.com/it/prodotti/trenta/</v>
       </c>
       <c r="Q12" t="str">
-        <v>librerias</v>
+        <v>librerie</v>
       </c>
       <c r="R12" t="str">
         <v>TRUE</v>
@@ -1079,7 +1079,7 @@
         <v>Libreria Trenta</v>
       </c>
       <c r="C13" t="str">
-        <v>librerías</v>
+        <v>librerie</v>
       </c>
       <c r="D13" t="str">
         <v>Trenta è la libreria interpretata da Febal Casa come elemento chiave intorno cui viene progettata la zona giorno.</v>
@@ -1091,7 +1091,7 @@
         <v/>
       </c>
       <c r="G13" t="str">
-        <v>libreria, trenta, librerías, librería, estanteria, estantería, bookshelf, estante, interpretata, febal, casa, elemento, chiave, intorno, viene, progettata, zona, giorno</v>
+        <v>libreria, trenta, librerie, librería, librerías, estanteria, estantería, bookshelf, estante, interpretata, febal, casa, elemento, chiave, intorno, viene, progettata, zona, giorno</v>
       </c>
       <c r="H13" t="str">
         <v/>
@@ -1121,7 +1121,7 @@
         <v>https://www.febalcasa.com/it/prodotti/trenta/</v>
       </c>
       <c r="Q13" t="str">
-        <v>librerias</v>
+        <v>librerie</v>
       </c>
       <c r="R13" t="str">
         <v>TRUE</v>
@@ -1135,7 +1135,7 @@
         <v>Madie Aurora</v>
       </c>
       <c r="C14" t="str">
-        <v>aparadores</v>
+        <v>madie</v>
       </c>
       <c r="D14" t="str">
         <v>La madia Aurora si distingue per la leggerezza dei volumi e l’estetica ricercata. Arreda la tua Casa con Febal Casa.</v>
@@ -1147,7 +1147,7 @@
         <v/>
       </c>
       <c r="G14" t="str">
-        <v>madie, aurora, aparadores, aparador, madia, credenza, sideboard, buffet, casa, distingue, leggerezza, volumi, estetica, ricercata, arreda, febal</v>
+        <v>madie, aurora, aparador, aparadores, madia, credenza, sideboard, buffet, casa, distingue, leggerezza, volumi, estetica, ricercata, arreda, febal</v>
       </c>
       <c r="H14" t="str">
         <v/>
@@ -1177,7 +1177,7 @@
         <v>https://www.febalcasa.com/it/prodotti/aurora/</v>
       </c>
       <c r="Q14" t="str">
-        <v>aparadores</v>
+        <v>madie</v>
       </c>
       <c r="R14" t="str">
         <v>TRUE</v>
@@ -1191,10 +1191,10 @@
         <v>Tavolino Rio</v>
       </c>
       <c r="C15" t="str">
-        <v>mesas de centro</v>
+        <v>tavolini</v>
       </c>
       <c r="D15" t="str">
-        <v>Il tavolino Rio è contraddistinto da una struttura in metallo che presenta la particolarità di poter accogliere riviste e giornali. Una funzione che lo rende</v>
+        <v>Il tavolino Rio è contraddistinto da una struttura in metallo che presenta la particolarità di poter accogliere riviste e giornali. Una funzione che lo rende il compagno ideale nei momenti di relax. Il piano può essere configurato a seconda del proprio gusto in finitura laccata opaca o impiallacciata.</v>
       </c>
       <c r="E15" t="str">
         <v/>
@@ -1203,7 +1203,7 @@
         <v/>
       </c>
       <c r="G15" t="str">
-        <v>tavolino, rio, mesas de centro, mesa de centro, mesita, coffee table, contraddistinto, struttura, metallo, presenta, particolarita, poter, accogliere, riviste, giornali, funzione, rende</v>
+        <v>tavolino, rio, tavolini, mesa de centro, mesita, coffee table, contraddistinto, struttura, metallo, presenta, particolarita, poter, accogliere, riviste, giornali, funzione, rende</v>
       </c>
       <c r="H15" t="str">
         <v/>
@@ -1233,7 +1233,7 @@
         <v>https://www.febalcasa.com/it/prodotti/rio/</v>
       </c>
       <c r="Q15" t="str">
-        <v>mesas-de-centro</v>
+        <v>tavolini</v>
       </c>
       <c r="R15" t="str">
         <v>TRUE</v>
@@ -1247,7 +1247,7 @@
         <v>Armadio Profile/ Block</v>
       </c>
       <c r="C16" t="str">
-        <v>armarios</v>
+        <v>armadi</v>
       </c>
       <c r="D16" t="str">
         <v>L'armadio con anta battente Profile Block si distingue per le sue linee nette e moderne, perfetta per un armadio dal carattere deciso.</v>
@@ -1259,7 +1259,7 @@
         <v/>
       </c>
       <c r="G16" t="str">
-        <v>armadio, profile/, block, armarios, armario, closet, ropero, wardrobe, cabina armadio, vestidor, anta, battente, profile, distingue, linee, nette, moderne, perfetta, carattere, deciso</v>
+        <v>armadio, profile/, block, armadi, armario, armarios, closet, ropero, wardrobe, cabina armadio, vestidor, anta, battente, profile, distingue, linee, nette, moderne, perfetta, carattere, deciso</v>
       </c>
       <c r="H16" t="str">
         <v/>
@@ -1289,7 +1289,7 @@
         <v>https://www.febalcasa.com/it/tipologia/armadi/ante/battente/profile-block/</v>
       </c>
       <c r="Q16" t="str">
-        <v>armarios</v>
+        <v>armadi</v>
       </c>
       <c r="R16" t="str">
         <v>TRUE</v>
@@ -1303,10 +1303,10 @@
         <v>Libreria Lapis</v>
       </c>
       <c r="C17" t="str">
-        <v>librerías</v>
+        <v>librerie</v>
       </c>
       <c r="D17" t="str">
-        <v>Il sistema libreria Lapis, configurabile a parete e centro stanza, si adatta perfettamente anche ad ambienti giorno e notte regalando estremo rigore e</v>
+        <v>Il sistema libreria Lapis, configurabile a parete e centro stanza, si adatta perfettamente anche ad ambienti giorno e notte regalando estremo rigore e contenimento. Il suo design inedito è personalizzabile grazie a diversi elementi compositivi: ripiani in vetro, in metallo o in pannello, pensili e basi in differenti modularità per soddisfare qualsiasi esigenza.</v>
       </c>
       <c r="E17" t="str">
         <v/>
@@ -1315,7 +1315,7 @@
         <v/>
       </c>
       <c r="G17" t="str">
-        <v>libreria, lapis, librerías, librería, estanteria, estantería, bookshelf, estante, sistema, configurabile, parete, centro, stanza, adatta, perfettamente, ambienti, giorno, notte</v>
+        <v>libreria, lapis, librerie, librería, librerías, estanteria, estantería, bookshelf, estante, sistema, configurabile, parete, centro, stanza, adatta, perfettamente, ambienti, giorno, notte</v>
       </c>
       <c r="H17" t="str">
         <v/>
@@ -1345,7 +1345,7 @@
         <v>https://www.febalcasa.com/it/prodotti/lapis/</v>
       </c>
       <c r="Q17" t="str">
-        <v>librerias</v>
+        <v>librerie</v>
       </c>
       <c r="R17" t="str">
         <v>TRUE</v>
@@ -1359,10 +1359,10 @@
         <v>Pouff Windsor</v>
       </c>
       <c r="C18" t="str">
-        <v>puffs</v>
+        <v>pouf</v>
       </c>
       <c r="D18" t="str">
-        <v>Il pouf Windsor completa la gamma dei pouf della collezione divani Febal Casa. Grazie alle dimensioni e ai rivestimenti in cui è disponibile, è un elemento</v>
+        <v>Il pouf Windsor completa la gamma dei pouf della collezione divani Febal Casa. Grazie alle dimensioni e ai rivestimenti in cui è disponibile, è un elemento estremamente versatile che risponde a qualsiasi esigenza. La sua leggerezza permette di offrire soluzioni dinamiche per ogni stile di vita.</v>
       </c>
       <c r="E18" t="str">
         <v/>
@@ -1371,7 +1371,7 @@
         <v/>
       </c>
       <c r="G18" t="str">
-        <v>pouff, windsor, puffs, puff, puf, ottoman, reposapies, pouf, completa, gamma, collezione, divani, febal, casa, grazie, dimensioni, rivestimenti, disponibile</v>
+        <v>pouff, windsor, pouf, puff, puffs, puf, ottoman, reposapies, completa, gamma, collezione, divani, febal, casa, grazie, dimensioni, rivestimenti, disponibile</v>
       </c>
       <c r="H18" t="str">
         <v/>
@@ -1401,7 +1401,7 @@
         <v>https://www.febalcasa.com/it/prodotti/windsor/</v>
       </c>
       <c r="Q18" t="str">
-        <v>puffs</v>
+        <v>pouf</v>
       </c>
       <c r="R18" t="str">
         <v>TRUE</v>
@@ -1415,10 +1415,10 @@
         <v>Boiserie TV</v>
       </c>
       <c r="C19" t="str">
-        <v>paneles decorativos</v>
+        <v>boiserie</v>
       </c>
       <c r="D19" t="str">
-        <v>La parete attrezzata boiserie è concepita come un sistema in grado di dialogare con tutti gli altri arredi della gamma Febal Casa</v>
+        <v>La boiserie è concepita come un sistema in grado di dialogare con tutti gli altri arredi della gamma Febal Casa, un elemento versatile che si innesta con soluzione di continuità arrivando fino a terra.</v>
       </c>
       <c r="E19" t="str">
         <v/>
@@ -1427,7 +1427,7 @@
         <v/>
       </c>
       <c r="G19" t="str">
-        <v>boiserie, paneles decorativos, panel, revestimiento, pared, decorativo, columna, vertical, parete, attrezzata, concepita, sistema, grado, dialogare, tutti, altri, arredi, gamma, febal</v>
+        <v>boiserie, panel, paneles decorativos, revestimiento, pared, decorativo, columna, vertical, concepita, sistema, grado, dialogare, tutti, altri, arredi, gamma, febal, casa, elemento</v>
       </c>
       <c r="H19" t="str">
         <v/>
@@ -1457,7 +1457,7 @@
         <v>https://www.febalcasa.com/it/prodotti/boiserie/</v>
       </c>
       <c r="Q19" t="str">
-        <v>paneles-decorativos</v>
+        <v>boiserie</v>
       </c>
       <c r="R19" t="str">
         <v>TRUE</v>
@@ -1471,7 +1471,7 @@
         <v>Sistema Origina</v>
       </c>
       <c r="C20" t="str">
-        <v>sistemas modulares</v>
+        <v>sistemi modulari</v>
       </c>
       <c r="D20" t="str">
         <v>L’anta a telaio è simbolo di un uno stile classico che può essere abbinato a aperture a gola, a maniglie e a pomoli.</v>
@@ -1483,7 +1483,7 @@
         <v/>
       </c>
       <c r="G20" t="str">
-        <v>sistema, origina, sistemas modulares, sistema modular, modular, anta, telaio, simbolo, stile, classico, abbinato, aperture, gola, maniglie, pomoli</v>
+        <v>sistema, origina, sistemi modulari, sistema modular, sistemas modulares, modular, anta, telaio, simbolo, stile, classico, abbinato, aperture, gola, maniglie, pomoli</v>
       </c>
       <c r="H20" t="str">
         <v/>
@@ -1513,7 +1513,7 @@
         <v>https://www.febalcasa.com/it/prodotti/origina-anta-telaio-legno/</v>
       </c>
       <c r="Q20" t="str">
-        <v>sistemas-modulares</v>
+        <v>sistemi-modulari</v>
       </c>
       <c r="R20" t="str">
         <v>TRUE</v>
@@ -1527,7 +1527,7 @@
         <v>Sistema Origina</v>
       </c>
       <c r="C21" t="str">
-        <v>sistemas modulares</v>
+        <v>sistemi modulari</v>
       </c>
       <c r="D21" t="str">
         <v>L’anta a telaio è simbolo di un uno stile classico che può essere abbinato a aperture a gola, a maniglie e a pomoli.</v>
@@ -1539,7 +1539,7 @@
         <v/>
       </c>
       <c r="G21" t="str">
-        <v>sistema, origina, sistemas modulares, sistema modular, modular, anta, telaio, simbolo, stile, classico, abbinato, aperture, gola, maniglie, pomoli</v>
+        <v>sistema, origina, sistemi modulari, sistema modular, sistemas modulares, modular, anta, telaio, simbolo, stile, classico, abbinato, aperture, gola, maniglie, pomoli</v>
       </c>
       <c r="H21" t="str">
         <v/>
@@ -1569,7 +1569,7 @@
         <v>https://www.febalcasa.com/it/prodotti/origina-anta-telaio-legno/</v>
       </c>
       <c r="Q21" t="str">
-        <v>sistemas-modulares</v>
+        <v>sistemi-modulari</v>
       </c>
       <c r="R21" t="str">
         <v>TRUE</v>
@@ -1583,7 +1583,7 @@
         <v>Sistema Origina</v>
       </c>
       <c r="C22" t="str">
-        <v>sistemas modulares</v>
+        <v>sistemi modulari</v>
       </c>
       <c r="D22" t="str">
         <v>L’anta a telaio è simbolo di un uno stile classico che può essere abbinato a aperture a gola, a maniglie e a pomoli.</v>
@@ -1595,7 +1595,7 @@
         <v/>
       </c>
       <c r="G22" t="str">
-        <v>sistema, origina, sistemas modulares, sistema modular, modular, anta, telaio, simbolo, stile, classico, abbinato, aperture, gola, maniglie, pomoli</v>
+        <v>sistema, origina, sistemi modulari, sistema modular, sistemas modulares, modular, anta, telaio, simbolo, stile, classico, abbinato, aperture, gola, maniglie, pomoli</v>
       </c>
       <c r="H22" t="str">
         <v/>
@@ -1625,7 +1625,7 @@
         <v>https://www.febalcasa.com/it/prodotti/origina-anta-telaio-legno/</v>
       </c>
       <c r="Q22" t="str">
-        <v>sistemas-modulares</v>
+        <v>sistemi-modulari</v>
       </c>
       <c r="R22" t="str">
         <v>TRUE</v>
@@ -1639,7 +1639,7 @@
         <v>Armadio Barret con Portale</v>
       </c>
       <c r="C23" t="str">
-        <v>armarios</v>
+        <v>armadi</v>
       </c>
       <c r="D23" t="str">
         <v>Scopri gli armadi a ponte con passaggio Febal Casa: soluzioni architettoniche che ottimizzano lo spazio con stile e funzionalità.</v>
@@ -1651,7 +1651,7 @@
         <v/>
       </c>
       <c r="G23" t="str">
-        <v>armadio, barret, portale, armarios, armario, closet, ropero, wardrobe, cabina armadio, vestidor, scopri, armadi, ponte, passaggio, febal, casa, soluzioni, architettoniche, ottimizzano, spazio, stile, funzionalita</v>
+        <v>armadio, barret, portale, armadi, armario, armarios, closet, ropero, wardrobe, cabina armadio, vestidor, scopri, ponte, passaggio, febal, casa, soluzioni, architettoniche, ottimizzano, spazio, stile, funzionalita</v>
       </c>
       <c r="H23" t="str">
         <v/>
@@ -1681,7 +1681,7 @@
         <v>https://www.febalcasa.com/it/tipologia/armadi/ispirazioni/armadio-con-passaggio-con-ponte/</v>
       </c>
       <c r="Q23" t="str">
-        <v>armarios</v>
+        <v>armadi</v>
       </c>
       <c r="R23" t="str">
         <v>TRUE</v>
@@ -1695,7 +1695,7 @@
         <v>Libreria Trenta</v>
       </c>
       <c r="C24" t="str">
-        <v>librerías</v>
+        <v>librerie</v>
       </c>
       <c r="D24" t="str">
         <v>Trenta è la libreria interpretata da Febal Casa come elemento chiave intorno cui viene progettata la zona giorno.</v>
@@ -1707,7 +1707,7 @@
         <v/>
       </c>
       <c r="G24" t="str">
-        <v>libreria, trenta, librerías, librería, estanteria, estantería, bookshelf, estante, interpretata, febal, casa, elemento, chiave, intorno, viene, progettata, zona, giorno</v>
+        <v>libreria, trenta, librerie, librería, librerías, estanteria, estantería, bookshelf, estante, interpretata, febal, casa, elemento, chiave, intorno, viene, progettata, zona, giorno</v>
       </c>
       <c r="H24" t="str">
         <v/>
@@ -1737,7 +1737,7 @@
         <v>https://www.febalcasa.com/it/prodotti/trenta/</v>
       </c>
       <c r="Q24" t="str">
-        <v>librerias</v>
+        <v>librerie</v>
       </c>
       <c r="R24" t="str">
         <v>TRUE</v>
@@ -1751,10 +1751,10 @@
         <v>Boiserie</v>
       </c>
       <c r="C25" t="str">
-        <v>paneles decorativos</v>
+        <v>boiserie</v>
       </c>
       <c r="D25" t="str">
-        <v>La parete attrezzata boiserie è concepita come un sistema in grado di dialogare con tutti gli altri arredi della gamma Febal Casa</v>
+        <v>La boiserie è concepita come un sistema in grado di dialogare con tutti gli altri arredi della gamma Febal Casa, un elemento versatile che si innesta con soluzione di continuità arrivando fino a terra.</v>
       </c>
       <c r="E25" t="str">
         <v/>
@@ -1763,7 +1763,7 @@
         <v/>
       </c>
       <c r="G25" t="str">
-        <v>boiserie, paneles decorativos, panel, revestimiento, pared, decorativo, columna, vertical, parete, attrezzata, concepita, sistema, grado, dialogare, tutti, altri, arredi, gamma, febal</v>
+        <v>boiserie, panel, paneles decorativos, revestimiento, pared, decorativo, columna, vertical, concepita, sistema, grado, dialogare, tutti, altri, arredi, gamma, febal, casa, elemento</v>
       </c>
       <c r="H25" t="str">
         <v/>
@@ -1793,7 +1793,7 @@
         <v>https://www.febalcasa.com/it/prodotti/boiserie/</v>
       </c>
       <c r="Q25" t="str">
-        <v>paneles-decorativos</v>
+        <v>boiserie</v>
       </c>
       <c r="R25" t="str">
         <v>TRUE</v>
@@ -1807,7 +1807,7 @@
         <v>Libreria Trenta Anta Libeskind022</v>
       </c>
       <c r="C26" t="str">
-        <v>librerías</v>
+        <v>librerie</v>
       </c>
       <c r="D26" t="str">
         <v>Trenta è la libreria interpretata da Febal Casa come elemento chiave intorno cui viene progettata la zona giorno.</v>
@@ -1819,7 +1819,7 @@
         <v/>
       </c>
       <c r="G26" t="str">
-        <v>libreria, trenta, anta, libeskind022, librerías, librería, estanteria, estantería, bookshelf, estante, interpretata, febal, casa, elemento, chiave, intorno, viene, progettata, zona, giorno</v>
+        <v>libreria, trenta, anta, libeskind022, librerie, librería, librerías, estanteria, estantería, bookshelf, estante, interpretata, febal, casa, elemento, chiave, intorno, viene, progettata, zona, giorno</v>
       </c>
       <c r="H26" t="str">
         <v/>
@@ -1849,7 +1849,7 @@
         <v>https://www.febalcasa.com/it/prodotti/trenta/</v>
       </c>
       <c r="Q26" t="str">
-        <v>librerias</v>
+        <v>librerie</v>
       </c>
       <c r="R26" t="str">
         <v>TRUE</v>
@@ -1863,7 +1863,7 @@
         <v>Divano Camden</v>
       </c>
       <c r="C27" t="str">
-        <v>sofás</v>
+        <v>divani</v>
       </c>
       <c r="D27" t="str">
         <v>Camden unisce eleganza e comfort in un design armonioso e avvolgente. Personalizzabile nei rivestimenti, si adatta a spazi classici e moderni, offrendo stile, calore e funzionalità a ogni ambiente living.</v>
@@ -1875,7 +1875,7 @@
         <v/>
       </c>
       <c r="G27" t="str">
-        <v>divano, camden, sofás, sofa, sofá, couch, asiento, unisce, eleganza, comfort, design, armonioso, avvolgente, personalizzabile, rivestimenti, adatta, spazi, classici</v>
+        <v>divano, camden, divani, sofa, sofá, sofás, couch, asiento, unisce, eleganza, comfort, design, armonioso, avvolgente, personalizzabile, rivestimenti, adatta, spazi, classici</v>
       </c>
       <c r="H27" t="str">
         <v/>
@@ -1905,7 +1905,7 @@
         <v>https://www.febalcasa.com/it/prodotti/camden/</v>
       </c>
       <c r="Q27" t="str">
-        <v>sofas</v>
+        <v>divani</v>
       </c>
       <c r="R27" t="str">
         <v>TRUE</v>
@@ -1919,7 +1919,7 @@
         <v>Divano Camden</v>
       </c>
       <c r="C28" t="str">
-        <v>sofás</v>
+        <v>divani</v>
       </c>
       <c r="D28" t="str">
         <v>Camden unisce eleganza e comfort in un design armonioso e avvolgente. Personalizzabile nei rivestimenti, si adatta a spazi classici e moderni, offrendo stile, calore e funzionalità a ogni ambiente living.</v>
@@ -1931,7 +1931,7 @@
         <v/>
       </c>
       <c r="G28" t="str">
-        <v>divano, camden, sofás, sofa, sofá, couch, asiento, unisce, eleganza, comfort, design, armonioso, avvolgente, personalizzabile, rivestimenti, adatta, spazi, classici</v>
+        <v>divano, camden, divani, sofa, sofá, sofás, couch, asiento, unisce, eleganza, comfort, design, armonioso, avvolgente, personalizzabile, rivestimenti, adatta, spazi, classici</v>
       </c>
       <c r="H28" t="str">
         <v/>
@@ -1961,7 +1961,7 @@
         <v>https://www.febalcasa.com/it/prodotti/camden/</v>
       </c>
       <c r="Q28" t="str">
-        <v>sofas</v>
+        <v>divani</v>
       </c>
       <c r="R28" t="str">
         <v>TRUE</v>
@@ -1975,10 +1975,10 @@
         <v>Poltrone Astor</v>
       </c>
       <c r="C29" t="str">
-        <v>sillones</v>
+        <v>poltrone</v>
       </c>
       <c r="D29" t="str">
-        <v>Astor, la poltrona elegante e confortevole per arredare il soggiorno con stile. La poltrona Astor rappresenta una perfetta sintesi tra estetica e</v>
+        <v>La poltrona Astor rappresenta una perfetta sintesi tra estetica e funzionalità. Dotata di un'ampia seduta ergonomica e una struttura solida, offre il massimo del comfort per il relax quotidiano. La base girevole, disponibile in versione circolare o a raggiera, aggiunge praticità e movimento, rendendola ideale anche per ambienti dinamici. Il design pulito e contemporaneo la rende un complemento perfetto per soggiorni moderni o salotti raffinati. Astor è disponibile in una selezione di tessuti di alta qualità e tonalità neutre o vivaci, per adattarsi con eleganza a ogni stile d'arredo. Una poltrona confortevole, di design, progettata per chi desidera un ambiente accogliente e ricercato.</v>
       </c>
       <c r="E29" t="str">
         <v/>
@@ -1987,7 +1987,7 @@
         <v/>
       </c>
       <c r="G29" t="str">
-        <v>poltrone, astor, sillones, sillon, sillón, poltrona, armchair, elegante, confortevole, arredare, soggiorno, stile, rappresenta, perfetta, sintesi, estetica</v>
+        <v>poltrone, astor, sillon, sillón, sillones, poltrona, armchair, disponibile, design, rappresenta, perfetta, sintesi, estetica, funzionalita, dotata, ampia, seduta</v>
       </c>
       <c r="H29" t="str">
         <v/>
@@ -2017,7 +2017,7 @@
         <v>https://www.febalcasa.com/it/prodotti/astor/</v>
       </c>
       <c r="Q29" t="str">
-        <v>sillones</v>
+        <v>poltrone</v>
       </c>
       <c r="R29" t="str">
         <v>TRUE</v>
@@ -2031,10 +2031,10 @@
         <v>Tavolini Ink</v>
       </c>
       <c r="C30" t="str">
-        <v>otros</v>
+        <v>altro</v>
       </c>
       <c r="D30" t="str">
-        <v>Elegante e funzionale, il coffee table Ink è adatto a qualsiasi stile. E' il complemento perfetto per accogliere una tazza di caffè durante una conversazione</v>
+        <v>Elegante e funzionale, il coffee table Ink è adatto a qualsiasi stile. E' il complemento perfetto per accogliere una tazza di caffè durante una conversazione o per esporre una selezione di oggetti preziosi in occasione di ospiti.</v>
       </c>
       <c r="E30" t="str">
         <v/>
@@ -2043,7 +2043,7 @@
         <v/>
       </c>
       <c r="G30" t="str">
-        <v>tavolini, ink, otros, elegante, funzionale, coffee, table, adatto, qualsiasi, stile, complemento, perfetto, accogliere, tazza, caffe</v>
+        <v>tavolini, ink, altro, elegante, funzionale, coffee, table, adatto, qualsiasi, stile, complemento, perfetto, accogliere, tazza, caffe</v>
       </c>
       <c r="H30" t="str">
         <v/>
@@ -2073,7 +2073,7 @@
         <v>https://www.febalcasa.com/it/prodotti/ink/</v>
       </c>
       <c r="Q30" t="str">
-        <v>otros</v>
+        <v>altro</v>
       </c>
       <c r="R30" t="str">
         <v>TRUE</v>
@@ -2087,7 +2087,7 @@
         <v>Cucina Origina Anta Libeskind022</v>
       </c>
       <c r="C31" t="str">
-        <v>cocinas</v>
+        <v>cucine</v>
       </c>
       <c r="D31" t="str">
         <v>Cucina Origina Anta Libeskind022 — pieza de la colección Febal Casa, sección CASA 02 - PERFETTA.</v>
@@ -2099,7 +2099,7 @@
         <v/>
       </c>
       <c r="G31" t="str">
-        <v>cucina, origina, anta, libeskind022, cocinas, cocina, kitchen, isla, casa, libeskind, pieza, coleccion, febal, seccion, perfetta</v>
+        <v>cucina, origina, anta, libeskind022, cucine, cocina, cocinas, kitchen, isla, casa, libeskind, pieza, coleccion, febal, seccion, perfetta</v>
       </c>
       <c r="H31" t="str">
         <v/>
@@ -2129,7 +2129,7 @@
         <v>https://www.febalcasa.com/it/prodotti/origina-anta-libeskind/</v>
       </c>
       <c r="Q31" t="str">
-        <v>cocinas</v>
+        <v>cucine</v>
       </c>
       <c r="R31" t="str">
         <v>TRUE</v>
@@ -2143,7 +2143,7 @@
         <v>Sistema Origina</v>
       </c>
       <c r="C32" t="str">
-        <v>sistemas modulares</v>
+        <v>sistemi modulari</v>
       </c>
       <c r="D32" t="str">
         <v>Sistema Origina — pieza de la colección Febal Casa, sección CASA 02 - PERFETTA.</v>
@@ -2155,7 +2155,7 @@
         <v/>
       </c>
       <c r="G32" t="str">
-        <v>sistema, origina, sistemas modulares, sistema modular, modular, casa, pieza, coleccion, febal, seccion, perfetta</v>
+        <v>sistema, origina, sistemi modulari, sistema modular, sistemas modulares, modular, casa, pieza, coleccion, febal, seccion, perfetta</v>
       </c>
       <c r="H32" t="str">
         <v/>
@@ -2185,7 +2185,7 @@
         <v>https://www.febalcasa.com/it/prodotti/origina-anta-libeskind/</v>
       </c>
       <c r="Q32" t="str">
-        <v>sistemas-modulares</v>
+        <v>sistemi-modulari</v>
       </c>
       <c r="R32" t="str">
         <v>TRUE</v>
@@ -2199,10 +2199,10 @@
         <v>Pouff Windsor</v>
       </c>
       <c r="C33" t="str">
-        <v>puffs</v>
+        <v>pouf</v>
       </c>
       <c r="D33" t="str">
-        <v>Il pouf Windsor completa la gamma dei pouf della collezione divani Febal Casa. Grazie alle dimensioni e ai rivestimenti in cui è disponibile, è un elemento</v>
+        <v>Il pouf Windsor completa la gamma dei pouf della collezione divani Febal Casa. Grazie alle dimensioni e ai rivestimenti in cui è disponibile, è un elemento estremamente versatile che risponde a qualsiasi esigenza. La sua leggerezza permette di offrire soluzioni dinamiche per ogni stile di vita.</v>
       </c>
       <c r="E33" t="str">
         <v/>
@@ -2211,7 +2211,7 @@
         <v/>
       </c>
       <c r="G33" t="str">
-        <v>pouff, windsor, puffs, puff, puf, ottoman, reposapies, pouf, completa, gamma, collezione, divani, febal, casa, grazie, dimensioni, rivestimenti, disponibile</v>
+        <v>pouff, windsor, pouf, puff, puffs, puf, ottoman, reposapies, completa, gamma, collezione, divani, febal, casa, grazie, dimensioni, rivestimenti, disponibile</v>
       </c>
       <c r="H33" t="str">
         <v/>
@@ -2241,7 +2241,7 @@
         <v>https://www.febalcasa.com/it/prodotti/windsor/</v>
       </c>
       <c r="Q33" t="str">
-        <v>puffs</v>
+        <v>pouf</v>
       </c>
       <c r="R33" t="str">
         <v>TRUE</v>
@@ -2255,7 +2255,7 @@
         <v>Libreria Trenta</v>
       </c>
       <c r="C34" t="str">
-        <v>librerías</v>
+        <v>librerie</v>
       </c>
       <c r="D34" t="str">
         <v>Trenta è la libreria interpretata da Febal Casa come elemento chiave intorno cui viene progettata la zona giorno.</v>
@@ -2267,7 +2267,7 @@
         <v/>
       </c>
       <c r="G34" t="str">
-        <v>libreria, trenta, librerías, librería, estanteria, estantería, bookshelf, estante, interpretata, febal, casa, elemento, chiave, intorno, viene, progettata, zona, giorno</v>
+        <v>libreria, trenta, librerie, librería, librerías, estanteria, estantería, bookshelf, estante, interpretata, febal, casa, elemento, chiave, intorno, viene, progettata, zona, giorno</v>
       </c>
       <c r="H34" t="str">
         <v/>
@@ -2297,7 +2297,7 @@
         <v>https://www.febalcasa.com/it/prodotti/trenta/</v>
       </c>
       <c r="Q34" t="str">
-        <v>librerias</v>
+        <v>librerie</v>
       </c>
       <c r="R34" t="str">
         <v>TRUE</v>
@@ -2311,10 +2311,10 @@
         <v>Tavolo Phoenix</v>
       </c>
       <c r="C35" t="str">
-        <v>mesas</v>
+        <v>tavoli</v>
       </c>
       <c r="D35" t="str">
-        <v>Un’armonia di forme per il tavolo Phoenix, caratterizzato da un’imponente base geometrica e dal piano configurabile secondo il proprio stile. Il suggestivo</v>
+        <v>Un'armonia di forme per il tavolo Phoenix, caratterizzato da un'imponente base geometrica e dal piano configurabile secondo il proprio stile. Il suggestivo accostamento di materiali e finiture e l'equilibrio tra le proporzioni ne fanno un complemento di grande impatto estetico, in grado di donare prestigio a ogni ambiente. Il tavolo Phoenix è proposto con piani di varie dimensioni di forma rettangolare in variabile fissa o allungabile. I piani sono in Cristallo Lucido, Cristallo Velvet, Superceramica, Supermarmo Opaco, Supermarmo Lucido e Impiallacciato. La struttura è in metallo finitura Ottone scuro, Nero, Antracite o Sabbia.</v>
       </c>
       <c r="E35" t="str">
         <v/>
@@ -2323,7 +2323,7 @@
         <v/>
       </c>
       <c r="G35" t="str">
-        <v>tavolo, phoenix, mesas, mesa, table, comedor, armonia, forme, caratterizzato, imponente, base, geometrica, piano, configurabile, secondo, proprio</v>
+        <v>tavolo, phoenix, tavoli, mesa, mesas, table, comedor, piani, cristallo, lucido, supermarmo, armonia, forme, caratterizzato, imponente, base, geometrica</v>
       </c>
       <c r="H35" t="str">
         <v/>
@@ -2353,7 +2353,7 @@
         <v>https://www.febalcasa.com/it/prodotti/phoenix/</v>
       </c>
       <c r="Q35" t="str">
-        <v>mesas</v>
+        <v>tavoli</v>
       </c>
       <c r="R35" t="str">
         <v>TRUE</v>
@@ -2367,10 +2367,10 @@
         <v>Madia Libeskind022</v>
       </c>
       <c r="C36" t="str">
-        <v>aparadores</v>
+        <v>madie</v>
       </c>
       <c r="D36" t="str">
-        <v>Il design è minimale e al contempo complesso: a seconda di come viene colpito dalla luce muta costantemente creando una superficie dinamica che si integra</v>
+        <v>Il design è minimale e al contempo complesso: a seconda di come viene colpito dalla luce muta costantemente creando una superficie dinamica che si integra allo stile di vita contemporaneo. Ad impreziosire il living e il dining, la madia LIBESKIND022 può essere configurata in 3 diverse tipologie: altezza H 75 cm in versione 3 ante o 4 ante e altezza H 154 cm in versione 2 ante. Oltre a poter essere configurata con ripiani interni in pannello o vetro e con un top laccato opaco o gres, la madia prevede la possibilità di inserire una cassettiera interna con maniglia integrata in legno per la versione H 75 cm e un kit allestimento bar per la versione H 154 cm con cassetto e un comodo piano estraibile.</v>
       </c>
       <c r="E36" t="str">
         <v/>
@@ -2379,7 +2379,7 @@
         <v/>
       </c>
       <c r="G36" t="str">
-        <v>madia, libeskind022, aparadores, aparador, credenza, sideboard, buffet, design, minimale, contempo, complesso, seconda, viene, colpito, luce, muta, costantemente, creando, superficie</v>
+        <v>madia, libeskind022, madie, aparador, aparadores, credenza, sideboard, buffet, versione, ante, configurata, altezza, design, minimale, contempo, complesso, seconda, viene, colpito</v>
       </c>
       <c r="H36" t="str">
         <v/>
@@ -2409,7 +2409,7 @@
         <v>https://www.febalcasa.com/it/prodotti/libeskind022/</v>
       </c>
       <c r="Q36" t="str">
-        <v>aparadores</v>
+        <v>madie</v>
       </c>
       <c r="R36" t="str">
         <v>TRUE</v>
@@ -2423,10 +2423,10 @@
         <v>Poltrona Vivienne</v>
       </c>
       <c r="C37" t="str">
-        <v>sillones</v>
+        <v>poltrone</v>
       </c>
       <c r="D37" t="str">
-        <v>Poltrona Vivienne, il perfetto equilibrio tra design moderno e comfort avvolgente. La poltrona Vivienne è la scelta ideale per chi cerca un elemento d’arredo</v>
+        <v>La poltrona Vivienne è la scelta ideale per chi cerca un elemento d'arredo elegante e versatile per il soggiorno o la zona lettura. Il suo design raffinato e contemporaneo si distingue per linee morbide e proporzioni equilibrate, mentre la possibilità di scegliere tra base girevole a raggiera o circolare la rende funzionale e personalizzabile. Perfetta in contesti moderni o classici, Vivienne è realizzata con tessuti pregiati e finiture curate nei minimi dettagli. Una poltrona di design che coniuga estetica e benessere, pensata per completare con stile ogni ambiente living. Disponibile in diversi colori e rivestimenti, si adatta facilmente ad arredi contemporanei, diventando un'icona di comfort senza tempo.</v>
       </c>
       <c r="E37" t="str">
         <v/>
@@ -2435,7 +2435,7 @@
         <v/>
       </c>
       <c r="G37" t="str">
-        <v>poltrona, vivienne, sillones, sillon, sillón, armchair, perfetto, equilibrio, design, moderno, comfort, avvolgente, scelta, ideale, cerca, elemento</v>
+        <v>poltrona, vivienne, poltrone, sillon, sillón, sillones, armchair, design, scelta, ideale, cerca, elemento, arredo, elegante, versatile, soggiorno, zona</v>
       </c>
       <c r="H37" t="str">
         <v/>
@@ -2465,7 +2465,7 @@
         <v>https://www.febalcasa.com/it/prodotti/vivienne/</v>
       </c>
       <c r="Q37" t="str">
-        <v>sillones</v>
+        <v>poltrone</v>
       </c>
       <c r="R37" t="str">
         <v>TRUE</v>
@@ -2479,7 +2479,7 @@
         <v>Armadio Collezione Momenti.</v>
       </c>
       <c r="C38" t="str">
-        <v>armarios</v>
+        <v>armadi</v>
       </c>
       <c r="D38" t="str">
         <v>La lavanderia è l'ambiente della casa che richiede un occhio di riguardo, non solo dal punto di vista estetico, ma anche da quello pratico.</v>
@@ -2491,7 +2491,7 @@
         <v/>
       </c>
       <c r="G38" t="str">
-        <v>armadio, collezione, momenti., armarios, armario, closet, ropero, wardrobe, cabina armadio, vestidor, lavanderia, ambiente, casa, richiede, occhio, riguardo, solo, punto, vista, estetico, quello, pratico</v>
+        <v>armadio, collezione, momenti., armadi, armario, armarios, closet, ropero, wardrobe, cabina armadio, vestidor, lavanderia, ambiente, casa, richiede, occhio, riguardo, solo, punto, vista, estetico, quello, pratico</v>
       </c>
       <c r="H38" t="str">
         <v/>
@@ -2521,7 +2521,7 @@
         <v>https://www.febalcasa.com/it/tipologia/mobili-di-servizi/mobili-di-servizi-laundry/</v>
       </c>
       <c r="Q38" t="str">
-        <v>armarios</v>
+        <v>armadi</v>
       </c>
       <c r="R38" t="str">
         <v>TRUE</v>
@@ -2535,10 +2535,10 @@
         <v>Boiserie</v>
       </c>
       <c r="C39" t="str">
-        <v>paneles decorativos</v>
+        <v>boiserie</v>
       </c>
       <c r="D39" t="str">
-        <v>La parete attrezzata boiserie è concepita come un sistema in grado di dialogare con tutti gli altri arredi della gamma Febal Casa</v>
+        <v>La boiserie è concepita come un sistema in grado di dialogare con tutti gli altri arredi della gamma Febal Casa, un elemento versatile che si innesta con soluzione di continuità arrivando fino a terra.</v>
       </c>
       <c r="E39" t="str">
         <v/>
@@ -2547,7 +2547,7 @@
         <v/>
       </c>
       <c r="G39" t="str">
-        <v>boiserie, paneles decorativos, panel, revestimiento, pared, decorativo, columna, vertical, parete, attrezzata, concepita, sistema, grado, dialogare, tutti, altri, arredi, gamma, febal</v>
+        <v>boiserie, panel, paneles decorativos, revestimiento, pared, decorativo, columna, vertical, concepita, sistema, grado, dialogare, tutti, altri, arredi, gamma, febal, casa, elemento</v>
       </c>
       <c r="H39" t="str">
         <v/>
@@ -2577,7 +2577,7 @@
         <v>https://www.febalcasa.com/it/prodotti/boiserie/</v>
       </c>
       <c r="Q39" t="str">
-        <v>paneles-decorativos</v>
+        <v>boiserie</v>
       </c>
       <c r="R39" t="str">
         <v>TRUE</v>
@@ -2591,7 +2591,7 @@
         <v>Letto Couple</v>
       </c>
       <c r="C40" t="str">
-        <v>dormitorio</v>
+        <v>camera da letto</v>
       </c>
       <c r="D40" t="str">
         <v>Letto Couple — pieza de la colección Febal Casa, sección CASA 02 - PERFETTA.</v>
@@ -2603,7 +2603,7 @@
         <v/>
       </c>
       <c r="G40" t="str">
-        <v>letto, couple, dormitorio, cama, bed, recamara, recámara, habitacion, gruppo notte, casa, pieza, coleccion, febal, seccion, perfetta</v>
+        <v>letto, couple, camera da letto, cama, dormitorio, bed, recamara, recámara, habitacion, gruppo notte, casa, pieza, coleccion, febal, seccion, perfetta</v>
       </c>
       <c r="H40" t="str">
         <v/>
@@ -2633,7 +2633,7 @@
         <v/>
       </c>
       <c r="Q40" t="str">
-        <v>dormitorio</v>
+        <v>camera-da-letto</v>
       </c>
       <c r="R40" t="str">
         <v>TRUE</v>
@@ -2647,10 +2647,10 @@
         <v>Poltrona Isabelle</v>
       </c>
       <c r="C41" t="str">
-        <v>sillones</v>
+        <v>poltrone</v>
       </c>
       <c r="D41" t="str">
-        <v>Isabelle, la poltroncina elegante e compatta per ambienti raffinati. Le poltroncine Isabelle sono la scelta ideale per chi desidera aggiungere un tocco di</v>
+        <v>Le poltroncine Isabelle sono la scelta ideale per chi desidera aggiungere un tocco di stile e comfort agli interni più curati. Compatte e raffinate, sono perfette per soggiorni eleganti, ingressi o angoli lettura. La loro forma armoniosa e i dettagli sartoriali valorizzano ogni ambiente, mentre i rivestimenti in tessuti di pregio ne esaltano il carattere ricercato. Isabelle si adatta facilmente a contesti moderni o classici, offrendo una soluzione versatile per chi cerca una poltroncina di design, comoda e dallo stile senza tempo. Disponibile in una gamma di finiture eleganti, è la poltroncina perfetta per completare il tuo arredamento con grazia e funzionalità.</v>
       </c>
       <c r="E41" t="str">
         <v/>
@@ -2659,7 +2659,7 @@
         <v/>
       </c>
       <c r="G41" t="str">
-        <v>poltrona, isabelle, sillones, sillon, sillón, armchair, poltroncina, elegante, compatta, ambienti, raffinati, poltroncine, scelta, ideale, desidera, aggiungere, tocco</v>
+        <v>poltrona, isabelle, poltrone, sillon, sillón, sillones, armchair, stile, eleganti, poltroncina, poltroncine, scelta, ideale, desidera, aggiungere, tocco, comfort, interni</v>
       </c>
       <c r="H41" t="str">
         <v/>
@@ -2689,7 +2689,7 @@
         <v>https://www.febalcasa.com/it/prodotti/isabelle/</v>
       </c>
       <c r="Q41" t="str">
-        <v>sillones</v>
+        <v>poltrone</v>
       </c>
       <c r="R41" t="str">
         <v>TRUE</v>
@@ -2703,10 +2703,10 @@
         <v>Specchio Polar</v>
       </c>
       <c r="C42" t="str">
-        <v>otros</v>
+        <v>altro</v>
       </c>
       <c r="D42" t="str">
-        <v>La specchiera Polar è progettata per essere posizionata a terra e offrire una visione completa della figura. Inoltre, può essere spostata agilmente e trovare</v>
+        <v>La specchiera Polar è progettata per essere posizionata a terra e offrire una visione completa della figura. Inoltre, può essere spostata agilmente e trovare posto in più ambienti della casa in base alle necessità del momento.</v>
       </c>
       <c r="E42" t="str">
         <v/>
@@ -2715,7 +2715,7 @@
         <v/>
       </c>
       <c r="G42" t="str">
-        <v>specchio, polar, otros, specchiera, progettata, posizionata, terra, offrire, visione, completa, figura, inoltre, spostata, agilmente</v>
+        <v>specchio, polar, altro, specchiera, progettata, posizionata, terra, offrire, visione, completa, figura, inoltre, spostata, agilmente</v>
       </c>
       <c r="H42" t="str">
         <v/>
@@ -2745,7 +2745,7 @@
         <v>https://www.febalcasa.com/it/prodotti/polar/</v>
       </c>
       <c r="Q42" t="str">
-        <v>otros</v>
+        <v>altro</v>
       </c>
       <c r="R42" t="str">
         <v>TRUE</v>
@@ -2759,10 +2759,10 @@
         <v>Boiserie</v>
       </c>
       <c r="C43" t="str">
-        <v>paneles decorativos</v>
+        <v>boiserie</v>
       </c>
       <c r="D43" t="str">
-        <v>La parete attrezzata boiserie è concepita come un sistema in grado di dialogare con tutti gli altri arredi della gamma Febal Casa</v>
+        <v>La boiserie è concepita come un sistema in grado di dialogare con tutti gli altri arredi della gamma Febal Casa, un elemento versatile che si innesta con soluzione di continuità arrivando fino a terra.</v>
       </c>
       <c r="E43" t="str">
         <v/>
@@ -2771,7 +2771,7 @@
         <v/>
       </c>
       <c r="G43" t="str">
-        <v>boiserie, paneles decorativos, panel, revestimiento, pared, decorativo, columna, vertical, parete, attrezzata, concepita, sistema, grado, dialogare, tutti, altri, arredi, gamma, febal</v>
+        <v>boiserie, panel, paneles decorativos, revestimiento, pared, decorativo, columna, vertical, concepita, sistema, grado, dialogare, tutti, altri, arredi, gamma, febal, casa, elemento</v>
       </c>
       <c r="H43" t="str">
         <v/>
@@ -2801,7 +2801,7 @@
         <v>https://www.febalcasa.com/it/prodotti/boiserie/</v>
       </c>
       <c r="Q43" t="str">
-        <v>paneles-decorativos</v>
+        <v>boiserie</v>
       </c>
       <c r="R43" t="str">
         <v>TRUE</v>
@@ -2815,7 +2815,7 @@
         <v>Cabina Armadio Lapis</v>
       </c>
       <c r="C44" t="str">
-        <v>armarios</v>
+        <v>armadi</v>
       </c>
       <c r="D44" t="str">
         <v>Il sistema Lapis, configurabile a parete o a centro stanza, si integra perfettamente nella cabina armadio su misura e, grazie alla sua struttura, lascia filtrare la luce.</v>
@@ -2827,7 +2827,7 @@
         <v/>
       </c>
       <c r="G44" t="str">
-        <v>cabina, armadio, lapis, armarios, armario, closet, ropero, wardrobe, cabina armadio, vestidor, sistema, configurabile, parete, centro, stanza, integra, perfettamente, misura, grazie</v>
+        <v>cabina, armadio, lapis, armadi, armario, armarios, closet, ropero, wardrobe, cabina armadio, vestidor, sistema, configurabile, parete, centro, stanza, integra, perfettamente, misura, grazie</v>
       </c>
       <c r="H44" t="str">
         <v/>
@@ -2857,7 +2857,7 @@
         <v>https://www.febalcasa.com/it/tipologia/cabine-armadio/lapis/</v>
       </c>
       <c r="Q44" t="str">
-        <v>armarios</v>
+        <v>armadi</v>
       </c>
       <c r="R44" t="str">
         <v>TRUE</v>
@@ -2871,10 +2871,10 @@
         <v>Boiserie</v>
       </c>
       <c r="C45" t="str">
-        <v>paneles decorativos</v>
+        <v>boiserie</v>
       </c>
       <c r="D45" t="str">
-        <v>La parete attrezzata boiserie è concepita come un sistema in grado di dialogare con tutti gli altri arredi della gamma Febal Casa</v>
+        <v>La boiserie è concepita come un sistema in grado di dialogare con tutti gli altri arredi della gamma Febal Casa, un elemento versatile che si innesta con soluzione di continuità arrivando fino a terra.</v>
       </c>
       <c r="E45" t="str">
         <v/>
@@ -2883,7 +2883,7 @@
         <v/>
       </c>
       <c r="G45" t="str">
-        <v>boiserie, paneles decorativos, panel, revestimiento, pared, decorativo, columna, vertical, parete, attrezzata, concepita, sistema, grado, dialogare, tutti, altri, arredi, gamma, febal</v>
+        <v>boiserie, panel, paneles decorativos, revestimiento, pared, decorativo, columna, vertical, concepita, sistema, grado, dialogare, tutti, altri, arredi, gamma, febal, casa, elemento</v>
       </c>
       <c r="H45" t="str">
         <v/>
@@ -2913,7 +2913,7 @@
         <v>https://www.febalcasa.com/it/prodotti/boiserie/</v>
       </c>
       <c r="Q45" t="str">
-        <v>paneles-decorativos</v>
+        <v>boiserie</v>
       </c>
       <c r="R45" t="str">
         <v>TRUE</v>
@@ -2927,7 +2927,7 @@
         <v>Armadio Lewitt Plus</v>
       </c>
       <c r="C46" t="str">
-        <v>armarios</v>
+        <v>armadi</v>
       </c>
       <c r="D46" t="str">
         <v>L'armadio con anta battente Lewitt Plus con presa a gola continua unisce design e massima personalizzazione, ideale per ambienti contemporanei.</v>
@@ -2939,7 +2939,7 @@
         <v/>
       </c>
       <c r="G46" t="str">
-        <v>armadio, lewitt, plus, armarios, armario, closet, ropero, wardrobe, cabina armadio, vestidor, anta, battente, presa, gola, continua, unisce, design, massima, personalizzazione</v>
+        <v>armadio, lewitt, plus, armadi, armario, armarios, closet, ropero, wardrobe, cabina armadio, vestidor, anta, battente, presa, gola, continua, unisce, design, massima, personalizzazione</v>
       </c>
       <c r="H46" t="str">
         <v/>
@@ -2969,7 +2969,7 @@
         <v>https://www.febalcasa.com/it/prodotti/lewitt-plus/</v>
       </c>
       <c r="Q46" t="str">
-        <v>armarios</v>
+        <v>armadi</v>
       </c>
       <c r="R46" t="str">
         <v>TRUE</v>
@@ -2983,7 +2983,7 @@
         <v>Sistema Diciotto</v>
       </c>
       <c r="C47" t="str">
-        <v>sistemas modulares</v>
+        <v>sistemi modulari</v>
       </c>
       <c r="D47" t="str">
         <v>Diciotto è una parete attrezzata per la zona living di design: pratico, versatile e funzionale permette una modularità altissima.</v>
@@ -2995,7 +2995,7 @@
         <v/>
       </c>
       <c r="G47" t="str">
-        <v>sistema, diciotto, sistemas modulares, sistema modular, modular, parete, attrezzata, zona, living, design, pratico, versatile, funzionale, permette, modularita, altissima</v>
+        <v>sistema, diciotto, sistemi modulari, sistema modular, sistemas modulares, modular, parete, attrezzata, zona, living, design, pratico, versatile, funzionale, permette, modularita, altissima</v>
       </c>
       <c r="H47" t="str">
         <v/>
@@ -3025,7 +3025,7 @@
         <v>https://www.febalcasa.com/it/prodotti/diciotto/</v>
       </c>
       <c r="Q47" t="str">
-        <v>sistemas-modulares</v>
+        <v>sistemi-modulari</v>
       </c>
       <c r="R47" t="str">
         <v>TRUE</v>
@@ -3039,7 +3039,7 @@
         <v>Libreria Trenta</v>
       </c>
       <c r="C48" t="str">
-        <v>librerías</v>
+        <v>librerie</v>
       </c>
       <c r="D48" t="str">
         <v>Trenta è la libreria interpretata da Febal Casa come elemento chiave intorno cui viene progettata la zona giorno.</v>
@@ -3051,7 +3051,7 @@
         <v/>
       </c>
       <c r="G48" t="str">
-        <v>libreria, trenta, librerías, librería, estanteria, estantería, bookshelf, estante, interpretata, febal, casa, elemento, chiave, intorno, viene, progettata, zona, giorno</v>
+        <v>libreria, trenta, librerie, librería, librerías, estanteria, estantería, bookshelf, estante, interpretata, febal, casa, elemento, chiave, intorno, viene, progettata, zona, giorno</v>
       </c>
       <c r="H48" t="str">
         <v/>
@@ -3081,7 +3081,7 @@
         <v>https://www.febalcasa.com/it/prodotti/trenta/</v>
       </c>
       <c r="Q48" t="str">
-        <v>librerias</v>
+        <v>librerie</v>
       </c>
       <c r="R48" t="str">
         <v>TRUE</v>
@@ -3095,7 +3095,7 @@
         <v>Divano Melrose</v>
       </c>
       <c r="C49" t="str">
-        <v>sofás</v>
+        <v>divani</v>
       </c>
       <c r="D49" t="str">
         <v>Melrose è un divano modulare dal design moderno e accogliente, pensato per unire stile, comfort e versatilità. Le linee morbide e i rivestimenti sartoriali lo rendono ideale per arredare con eleganza ogni spazio living contemporaneo.</v>
@@ -3107,7 +3107,7 @@
         <v/>
       </c>
       <c r="G49" t="str">
-        <v>divano, melrose, sofás, sofa, sofá, couch, asiento, modulare, design, moderno, accogliente, pensato, unire, stile, comfort, versatilita, linee</v>
+        <v>divano, melrose, divani, sofa, sofá, sofás, couch, asiento, modulare, design, moderno, accogliente, pensato, unire, stile, comfort, versatilita, linee</v>
       </c>
       <c r="H49" t="str">
         <v/>
@@ -3137,7 +3137,7 @@
         <v>https://www.febalcasa.com/it/prodotti/melrose/</v>
       </c>
       <c r="Q49" t="str">
-        <v>sofas</v>
+        <v>divani</v>
       </c>
       <c r="R49" t="str">
         <v>TRUE</v>
@@ -3151,10 +3151,10 @@
         <v>Poltrona Andy</v>
       </c>
       <c r="C50" t="str">
-        <v>sillones</v>
+        <v>poltrone</v>
       </c>
       <c r="D50" t="str">
-        <v>Moderna e contemporanea, la nuova poltrona Andy presenta un design distintivo e allo stesso tempo confortevole per la vita di tutti i giorni. Le sue geometrie</v>
+        <v>Moderna e contemporanea, la nuova poltrona Andy presenta un design distintivo e allo stesso tempo confortevole per la vita di tutti i giorni. Le sue geometrie catturano l'attenzione e la rendono la protagonista dell'ambiente.</v>
       </c>
       <c r="E50" t="str">
         <v/>
@@ -3163,7 +3163,7 @@
         <v/>
       </c>
       <c r="G50" t="str">
-        <v>poltrona, andy, sillones, sillon, sillón, armchair, moderna, contemporanea, nuova, presenta, design, distintivo, stesso, tempo, confortevole, vita</v>
+        <v>poltrona, andy, poltrone, sillon, sillón, sillones, armchair, moderna, contemporanea, nuova, presenta, design, distintivo, stesso, tempo, confortevole, vita</v>
       </c>
       <c r="H50" t="str">
         <v/>
@@ -3193,7 +3193,7 @@
         <v>https://www.febalcasa.com/it/prodotti/andy/</v>
       </c>
       <c r="Q50" t="str">
-        <v>sillones</v>
+        <v>poltrone</v>
       </c>
       <c r="R50" t="str">
         <v>TRUE</v>
@@ -3207,7 +3207,7 @@
         <v>Gruppo Notte Marlene</v>
       </c>
       <c r="C51" t="str">
-        <v>dormitorio</v>
+        <v>camera da letto</v>
       </c>
       <c r="D51" t="str">
         <v>Marlene di Febal Casa: gruppo notte dalle forme curvilinee, disponibile con maniglia verticale in metallo e inserto in pelle. Top in gres e ampie opzioni di personalizzazione.</v>
@@ -3219,7 +3219,7 @@
         <v/>
       </c>
       <c r="G51" t="str">
-        <v>gruppo, notte, marlene, dormitorio, cama, letto, bed, recamara, recámara, habitacion, gruppo notte, febal, casa, forme, curvilinee, disponibile, maniglia, verticale, metallo, inserto</v>
+        <v>gruppo, notte, marlene, camera da letto, cama, dormitorio, letto, bed, recamara, recámara, habitacion, gruppo notte, febal, casa, forme, curvilinee, disponibile, maniglia, verticale, metallo, inserto</v>
       </c>
       <c r="H51" t="str">
         <v/>
@@ -3249,7 +3249,7 @@
         <v>https://www.febalcasa.com/it/prodotti/febal-notte-gruppo-como-e-comodino-marlene/</v>
       </c>
       <c r="Q51" t="str">
-        <v>dormitorio</v>
+        <v>camera-da-letto</v>
       </c>
       <c r="R51" t="str">
         <v>TRUE</v>
@@ -3263,7 +3263,7 @@
         <v>Cucina Modula anta Square</v>
       </c>
       <c r="C52" t="str">
-        <v>cocinas</v>
+        <v>cucine</v>
       </c>
       <c r="D52" t="str">
         <v>Cucina Modula anta Square — pieza de la colección Febal Casa, sección CASA 03 - AUDACE.</v>
@@ -3275,7 +3275,7 @@
         <v/>
       </c>
       <c r="G52" t="str">
-        <v>cucina, modula, anta, square, cocinas, cocina, kitchen, isla, casa, pieza, coleccion, febal, seccion, audace</v>
+        <v>cucina, modula, anta, square, cucine, cocina, cocinas, kitchen, isla, casa, pieza, coleccion, febal, seccion, audace</v>
       </c>
       <c r="H52" t="str">
         <v/>
@@ -3305,7 +3305,7 @@
         <v>https://www.febalcasa.com/it/prodotti/modula-anta-square/</v>
       </c>
       <c r="Q52" t="str">
-        <v>cocinas</v>
+        <v>cucine</v>
       </c>
       <c r="R52" t="str">
         <v>TRUE</v>
@@ -3319,7 +3319,7 @@
         <v>Tavolo Madeira</v>
       </c>
       <c r="C53" t="str">
-        <v>mesas</v>
+        <v>tavoli</v>
       </c>
       <c r="D53" t="str">
         <v>Tavolo Madeira — pieza de la colección Febal Casa, sección CASA 03 - AUDACE.</v>
@@ -3331,7 +3331,7 @@
         <v/>
       </c>
       <c r="G53" t="str">
-        <v>tavolo, madeira, mesas, mesa, table, comedor, casa, pieza, coleccion, febal, seccion, audace</v>
+        <v>tavolo, madeira, tavoli, mesa, mesas, table, comedor, casa, pieza, coleccion, febal, seccion, audace</v>
       </c>
       <c r="H53" t="str">
         <v/>
@@ -3361,7 +3361,7 @@
         <v xml:space="preserve">https://www.febalcasa.com/it/prodotti/madeira/ </v>
       </c>
       <c r="Q53" t="str">
-        <v>mesas</v>
+        <v>tavoli</v>
       </c>
       <c r="R53" t="str">
         <v>TRUE</v>
@@ -3375,10 +3375,10 @@
         <v>Sedia Nina</v>
       </c>
       <c r="C54" t="str">
-        <v>sillas</v>
+        <v>sedie</v>
       </c>
       <c r="D54" t="str">
-        <v>La sedia Nina può essere personalizzata con struttura in metallo oppure rivestita in abbinamento alla scocca. Il design è studiato per offrire una seduta</v>
+        <v>La sedia Nina può essere personalizzata con struttura in metallo oppure rivestita in abbinamento alla scocca. Il design è studiato per offrire una seduta confortevole e, se lo si desidera, aggiungere un tocco di colore alla zona dining.</v>
       </c>
       <c r="E54" t="str">
         <v/>
@@ -3387,7 +3387,7 @@
         <v/>
       </c>
       <c r="G54" t="str">
-        <v>sedia, nina, sillas, silla, chair, asiento, personalizzata, struttura, metallo, oppure, rivestita, abbinamento, scocca, design, studiato, offrire</v>
+        <v>sedia, nina, sedie, silla, sillas, chair, asiento, personalizzata, struttura, metallo, oppure, rivestita, abbinamento, scocca, design, studiato, offrire</v>
       </c>
       <c r="H54" t="str">
         <v/>
@@ -3417,7 +3417,7 @@
         <v>https://www.febalcasa.com/it/prodotti/nina/</v>
       </c>
       <c r="Q54" t="str">
-        <v>sillas</v>
+        <v>sedie</v>
       </c>
       <c r="R54" t="str">
         <v>TRUE</v>
@@ -3431,7 +3431,7 @@
         <v>Madia Leaf</v>
       </c>
       <c r="C55" t="str">
-        <v>aparadores</v>
+        <v>madie</v>
       </c>
       <c r="D55" t="str">
         <v>La madia Leaf, disponibile in due diverse altezze, si caratterizza per il suo disegno razionale impreziosito dalla maniglia incassata.</v>
@@ -3443,7 +3443,7 @@
         <v/>
       </c>
       <c r="G55" t="str">
-        <v>madia, leaf, aparadores, aparador, credenza, sideboard, buffet, disponibile, diverse, altezze, caratterizza, disegno, razionale, impreziosito, maniglia, incassata</v>
+        <v>madia, leaf, madie, aparador, aparadores, credenza, sideboard, buffet, disponibile, diverse, altezze, caratterizza, disegno, razionale, impreziosito, maniglia, incassata</v>
       </c>
       <c r="H55" t="str">
         <v/>
@@ -3473,7 +3473,7 @@
         <v>https://www.febalcasa.com/it/prodotti/leaf/</v>
       </c>
       <c r="Q55" t="str">
-        <v>aparadores</v>
+        <v>madie</v>
       </c>
       <c r="R55" t="str">
         <v>TRUE</v>
@@ -3487,7 +3487,7 @@
         <v>Libreria Trenta</v>
       </c>
       <c r="C56" t="str">
-        <v>librerías</v>
+        <v>librerie</v>
       </c>
       <c r="D56" t="str">
         <v>Trenta è la libreria interpretata da Febal Casa come elemento chiave intorno cui viene progettata la zona giorno.</v>
@@ -3499,7 +3499,7 @@
         <v/>
       </c>
       <c r="G56" t="str">
-        <v>libreria, trenta, librerías, librería, estanteria, estantería, bookshelf, estante, interpretata, febal, casa, elemento, chiave, intorno, viene, progettata, zona, giorno</v>
+        <v>libreria, trenta, librerie, librería, librerías, estanteria, estantería, bookshelf, estante, interpretata, febal, casa, elemento, chiave, intorno, viene, progettata, zona, giorno</v>
       </c>
       <c r="H56" t="str">
         <v/>
@@ -3529,7 +3529,7 @@
         <v>https://www.febalcasa.com/it/prodotti/trenta/</v>
       </c>
       <c r="Q56" t="str">
-        <v>librerias</v>
+        <v>librerie</v>
       </c>
       <c r="R56" t="str">
         <v>TRUE</v>
@@ -3543,7 +3543,7 @@
         <v>Gruppo Notte Marlene</v>
       </c>
       <c r="C57" t="str">
-        <v>dormitorio</v>
+        <v>camera da letto</v>
       </c>
       <c r="D57" t="str">
         <v>Astrid di Febal Casa: gruppo notte con vassoio superiore in cristallo e maniglie integrate nel disegno. Eleganza trasparente per la camera da letto contemporanea.</v>
@@ -3555,7 +3555,7 @@
         <v/>
       </c>
       <c r="G57" t="str">
-        <v>gruppo, notte, marlene, dormitorio, cama, letto, bed, recamara, recámara, habitacion, gruppo notte, astrid, febal, casa, vassoio, superiore, cristallo, maniglie, integrate, disegno, eleganza</v>
+        <v>gruppo, notte, marlene, camera da letto, cama, dormitorio, letto, bed, recamara, recámara, habitacion, gruppo notte, astrid, febal, casa, vassoio, superiore, cristallo, maniglie, integrate, disegno, eleganza</v>
       </c>
       <c r="H57" t="str">
         <v/>
@@ -3585,7 +3585,7 @@
         <v>https://www.febalcasa.com/it/prodotti/astrid/</v>
       </c>
       <c r="Q57" t="str">
-        <v>dormitorio</v>
+        <v>camera-da-letto</v>
       </c>
       <c r="R57" t="str">
         <v>TRUE</v>
@@ -3599,10 +3599,10 @@
         <v>Boiserie</v>
       </c>
       <c r="C58" t="str">
-        <v>paneles decorativos</v>
+        <v>boiserie</v>
       </c>
       <c r="D58" t="str">
-        <v>La parete attrezzata boiserie è concepita come un sistema in grado di dialogare con tutti gli altri arredi della gamma Febal Casa</v>
+        <v>La boiserie è concepita come un sistema in grado di dialogare con tutti gli altri arredi della gamma Febal Casa, un elemento versatile che si innesta con soluzione di continuità arrivando fino a terra.</v>
       </c>
       <c r="E58" t="str">
         <v/>
@@ -3611,7 +3611,7 @@
         <v/>
       </c>
       <c r="G58" t="str">
-        <v>boiserie, paneles decorativos, panel, revestimiento, pared, decorativo, columna, vertical, parete, attrezzata, concepita, sistema, grado, dialogare, tutti, altri, arredi, gamma, febal</v>
+        <v>boiserie, panel, paneles decorativos, revestimiento, pared, decorativo, columna, vertical, concepita, sistema, grado, dialogare, tutti, altri, arredi, gamma, febal, casa, elemento</v>
       </c>
       <c r="H58" t="str">
         <v/>
@@ -3641,7 +3641,7 @@
         <v>https://www.febalcasa.com/it/prodotti/boiserie/</v>
       </c>
       <c r="Q58" t="str">
-        <v>paneles-decorativos</v>
+        <v>boiserie</v>
       </c>
       <c r="R58" t="str">
         <v>TRUE</v>
@@ -3655,7 +3655,7 @@
         <v>Armadio Collezione Momenti.</v>
       </c>
       <c r="C59" t="str">
-        <v>armarios</v>
+        <v>armadi</v>
       </c>
       <c r="D59" t="str">
         <v>Armadio Collezione Momenti. — pieza de la colección Febal Casa, sección CASA 03 - AUDACE.</v>
@@ -3667,7 +3667,7 @@
         <v/>
       </c>
       <c r="G59" t="str">
-        <v>armadio, collezione, momenti., armarios, armario, closet, ropero, wardrobe, cabina armadio, vestidor, casa, momenti, pieza, coleccion, febal, seccion, audace</v>
+        <v>armadio, collezione, momenti., armadi, armario, armarios, closet, ropero, wardrobe, cabina armadio, vestidor, casa, momenti, pieza, coleccion, febal, seccion, audace</v>
       </c>
       <c r="H59" t="str">
         <v/>
@@ -3697,7 +3697,7 @@
         <v>https://www.febalcasa.com/it/tipologia/momenti/cameretta/</v>
       </c>
       <c r="Q59" t="str">
-        <v>armarios</v>
+        <v>armadi</v>
       </c>
       <c r="R59" t="str">
         <v>TRUE</v>
@@ -3711,7 +3711,7 @@
         <v>Letto Collezione Momenti.</v>
       </c>
       <c r="C60" t="str">
-        <v>dormitorio</v>
+        <v>camera da letto</v>
       </c>
       <c r="D60" t="str">
         <v>Letto Collezione Momenti. — pieza de la colección Febal Casa, sección CASA 03 - AUDACE.</v>
@@ -3723,7 +3723,7 @@
         <v/>
       </c>
       <c r="G60" t="str">
-        <v>letto, collezione, momenti., dormitorio, cama, bed, recamara, recámara, habitacion, gruppo notte, casa, momenti, pieza, coleccion, febal, seccion, audace</v>
+        <v>letto, collezione, momenti., camera da letto, cama, dormitorio, bed, recamara, recámara, habitacion, gruppo notte, casa, momenti, pieza, coleccion, febal, seccion, audace</v>
       </c>
       <c r="H60" t="str">
         <v/>
@@ -3753,7 +3753,7 @@
         <v>https://www.febalcasa.com/it/tipologia/momenti/cameretta/</v>
       </c>
       <c r="Q60" t="str">
-        <v>dormitorio</v>
+        <v>camera-da-letto</v>
       </c>
       <c r="R60" t="str">
         <v>TRUE</v>
@@ -3767,7 +3767,7 @@
         <v>Libreria Collezione Momenti.</v>
       </c>
       <c r="C61" t="str">
-        <v>librerías</v>
+        <v>librerie</v>
       </c>
       <c r="D61" t="str">
         <v>Libreria Collezione Momenti. — pieza de la colección Febal Casa, sección CASA 03 - AUDACE.</v>
@@ -3779,7 +3779,7 @@
         <v/>
       </c>
       <c r="G61" t="str">
-        <v>libreria, collezione, momenti., librerías, librería, estanteria, estantería, bookshelf, estante, casa, momenti, pieza, coleccion, febal, seccion, audace</v>
+        <v>libreria, collezione, momenti., librerie, librería, librerías, estanteria, estantería, bookshelf, estante, casa, momenti, pieza, coleccion, febal, seccion, audace</v>
       </c>
       <c r="H61" t="str">
         <v/>
@@ -3809,7 +3809,7 @@
         <v>https://www.febalcasa.com/it/tipologia/momenti/cameretta/</v>
       </c>
       <c r="Q61" t="str">
-        <v>librerias</v>
+        <v>librerie</v>
       </c>
       <c r="R61" t="str">
         <v>TRUE</v>
@@ -3823,10 +3823,10 @@
         <v>Pouff Windsor</v>
       </c>
       <c r="C62" t="str">
-        <v>puffs</v>
+        <v>pouf</v>
       </c>
       <c r="D62" t="str">
-        <v>Il pouf Windsor completa la gamma dei pouf della collezione divani Febal Casa. Grazie alle dimensioni e ai rivestimenti in cui è disponibile, è un elemento</v>
+        <v>Il pouf Windsor completa la gamma dei pouf della collezione divani Febal Casa. Grazie alle dimensioni e ai rivestimenti in cui è disponibile, è un elemento estremamente versatile che risponde a qualsiasi esigenza. La sua leggerezza permette di offrire soluzioni dinamiche per ogni stile di vita.</v>
       </c>
       <c r="E62" t="str">
         <v/>
@@ -3835,7 +3835,7 @@
         <v/>
       </c>
       <c r="G62" t="str">
-        <v>pouff, windsor, puffs, puff, puf, ottoman, reposapies, pouf, completa, gamma, collezione, divani, febal, casa, grazie, dimensioni, rivestimenti, disponibile</v>
+        <v>pouff, windsor, pouf, puff, puffs, puf, ottoman, reposapies, completa, gamma, collezione, divani, febal, casa, grazie, dimensioni, rivestimenti, disponibile</v>
       </c>
       <c r="H62" t="str">
         <v/>
@@ -3865,7 +3865,7 @@
         <v>https://www.febalcasa.com/it/prodotti/windsor/</v>
       </c>
       <c r="Q62" t="str">
-        <v>puffs</v>
+        <v>pouf</v>
       </c>
       <c r="R62" t="str">
         <v>TRUE</v>
@@ -3879,7 +3879,7 @@
         <v>Armadio  Collezione Momenti.</v>
       </c>
       <c r="C63" t="str">
-        <v>armarios</v>
+        <v>armadi</v>
       </c>
       <c r="D63" t="str">
         <v>Armadio  Collezione Momenti. — pieza de la colección Febal Casa, sección CASA 03 - AUDACE.</v>
@@ -3891,7 +3891,7 @@
         <v/>
       </c>
       <c r="G63" t="str">
-        <v>armadio, collezione, momenti., armarios, armario, closet, ropero, wardrobe, cabina armadio, vestidor, casa, momenti, pieza, coleccion, febal, seccion, audace</v>
+        <v>armadio, collezione, momenti., armadi, armario, armarios, closet, ropero, wardrobe, cabina armadio, vestidor, casa, momenti, pieza, coleccion, febal, seccion, audace</v>
       </c>
       <c r="H63" t="str">
         <v/>
@@ -3921,7 +3921,7 @@
         <v>https://www.febalcasa.com/it/tipologia/momenti/cameretta/</v>
       </c>
       <c r="Q63" t="str">
-        <v>armarios</v>
+        <v>armadi</v>
       </c>
       <c r="R63" t="str">
         <v>TRUE</v>
@@ -3935,10 +3935,10 @@
         <v>Boiserie</v>
       </c>
       <c r="C64" t="str">
-        <v>paneles decorativos</v>
+        <v>boiserie</v>
       </c>
       <c r="D64" t="str">
-        <v>La parete attrezzata boiserie è concepita come un sistema in grado di dialogare con tutti gli altri arredi della gamma Febal Casa</v>
+        <v>La boiserie è concepita come un sistema in grado di dialogare con tutti gli altri arredi della gamma Febal Casa, un elemento versatile che si innesta con soluzione di continuità arrivando fino a terra.</v>
       </c>
       <c r="E64" t="str">
         <v/>
@@ -3947,7 +3947,7 @@
         <v/>
       </c>
       <c r="G64" t="str">
-        <v>boiserie, paneles decorativos, panel, revestimiento, pared, decorativo, columna, vertical, parete, attrezzata, concepita, sistema, grado, dialogare, tutti, altri, arredi, gamma, febal</v>
+        <v>boiserie, panel, paneles decorativos, revestimiento, pared, decorativo, columna, vertical, concepita, sistema, grado, dialogare, tutti, altri, arredi, gamma, febal, casa, elemento</v>
       </c>
       <c r="H64" t="str">
         <v/>
@@ -3977,7 +3977,7 @@
         <v>https://www.febalcasa.com/it/prodotti/boiserie/</v>
       </c>
       <c r="Q64" t="str">
-        <v>paneles-decorativos</v>
+        <v>boiserie</v>
       </c>
       <c r="R64" t="str">
         <v>TRUE</v>
@@ -3991,7 +3991,7 @@
         <v>Libreria Trenta</v>
       </c>
       <c r="C65" t="str">
-        <v>librerías</v>
+        <v>librerie</v>
       </c>
       <c r="D65" t="str">
         <v>Trenta è la libreria interpretata da Febal Casa come elemento chiave intorno cui viene progettata la zona giorno.</v>
@@ -4003,7 +4003,7 @@
         <v/>
       </c>
       <c r="G65" t="str">
-        <v>libreria, trenta, librerías, librería, estanteria, estantería, bookshelf, estante, interpretata, febal, casa, elemento, chiave, intorno, viene, progettata, zona, giorno</v>
+        <v>libreria, trenta, librerie, librería, librerías, estanteria, estantería, bookshelf, estante, interpretata, febal, casa, elemento, chiave, intorno, viene, progettata, zona, giorno</v>
       </c>
       <c r="H65" t="str">
         <v/>
@@ -4033,7 +4033,7 @@
         <v>https://www.febalcasa.com/it/prodotti/trenta/</v>
       </c>
       <c r="Q65" t="str">
-        <v>librerias</v>
+        <v>librerie</v>
       </c>
       <c r="R65" t="str">
         <v>TRUE</v>
@@ -4047,7 +4047,7 @@
         <v>Madia Onda - Zaha Hadid Architects</v>
       </c>
       <c r="C66" t="str">
-        <v>aparadores</v>
+        <v>madie</v>
       </c>
       <c r="D66" t="str">
         <v>Madia Onda - Zaha Hadid Architects — pieza de la colección Febal Casa, sección CASA 04 - A-MARE.</v>
@@ -4059,7 +4059,7 @@
         <v/>
       </c>
       <c r="G66" t="str">
-        <v>madia, onda, zaha, hadid, architects, aparadores, aparador, credenza, sideboard, buffet, casa, pieza, coleccion, febal, seccion, mare</v>
+        <v>madia, onda, zaha, hadid, architects, madie, aparador, aparadores, credenza, sideboard, buffet, casa, pieza, coleccion, febal, seccion, mare</v>
       </c>
       <c r="H66" t="str">
         <v/>
@@ -4089,7 +4089,7 @@
         <v>https://www.febalcasa.com/it/prodotti/madia-onda/</v>
       </c>
       <c r="Q66" t="str">
-        <v>aparadores</v>
+        <v>madie</v>
       </c>
       <c r="R66" t="str">
         <v>TRUE</v>
@@ -4103,7 +4103,7 @@
         <v>Divano Navigli</v>
       </c>
       <c r="C67" t="str">
-        <v>sofás</v>
+        <v>divani</v>
       </c>
       <c r="D67" t="str">
         <v>Disponibile in diverse tonalità e rivestimenti, il Divano Navigli è caratterizzato dall’ampiezza della seduta e dall’effetto trapuntatura continua.</v>
@@ -4115,7 +4115,7 @@
         <v/>
       </c>
       <c r="G67" t="str">
-        <v>divano, navigli, sofás, sofa, sofá, couch, asiento, dall, disponibile, diverse, tonalita, rivestimenti, caratterizzato, ampiezza, seduta, effetto, trapuntatura</v>
+        <v>divano, navigli, divani, sofa, sofá, sofás, couch, asiento, dall, disponibile, diverse, tonalita, rivestimenti, caratterizzato, ampiezza, seduta, effetto, trapuntatura</v>
       </c>
       <c r="H67" t="str">
         <v/>
@@ -4145,7 +4145,7 @@
         <v>https://www.febalcasa.com/it/prodotti/navigli/</v>
       </c>
       <c r="Q67" t="str">
-        <v>sofas</v>
+        <v>divani</v>
       </c>
       <c r="R67" t="str">
         <v>TRUE</v>
@@ -4159,10 +4159,10 @@
         <v>Libreria Lapis</v>
       </c>
       <c r="C68" t="str">
-        <v>librerías</v>
+        <v>librerie</v>
       </c>
       <c r="D68" t="str">
-        <v>Il sistema libreria Lapis, configurabile a parete e centro stanza, si adatta perfettamente anche ad ambienti giorno e notte regalando estremo rigore e</v>
+        <v>Il sistema libreria Lapis, configurabile a parete e centro stanza, si adatta perfettamente anche ad ambienti giorno e notte regalando estremo rigore e contenimento. Il suo design inedito è personalizzabile grazie a diversi elementi compositivi: ripiani in vetro, in metallo o in pannello, pensili e basi in differenti modularità per soddisfare qualsiasi esigenza.</v>
       </c>
       <c r="E68" t="str">
         <v/>
@@ -4171,7 +4171,7 @@
         <v/>
       </c>
       <c r="G68" t="str">
-        <v>libreria, lapis, librerías, librería, estanteria, estantería, bookshelf, estante, sistema, configurabile, parete, centro, stanza, adatta, perfettamente, ambienti, giorno, notte</v>
+        <v>libreria, lapis, librerie, librería, librerías, estanteria, estantería, bookshelf, estante, sistema, configurabile, parete, centro, stanza, adatta, perfettamente, ambienti, giorno, notte</v>
       </c>
       <c r="H68" t="str">
         <v/>
@@ -4201,7 +4201,7 @@
         <v>https://www.febalcasa.com/it/prodotti/lapis/</v>
       </c>
       <c r="Q68" t="str">
-        <v>librerias</v>
+        <v>librerie</v>
       </c>
       <c r="R68" t="str">
         <v>TRUE</v>
@@ -4215,7 +4215,7 @@
         <v>Sistema Origina</v>
       </c>
       <c r="C69" t="str">
-        <v>sistemas modulares</v>
+        <v>sistemi modulari</v>
       </c>
       <c r="D69" t="str">
         <v>Il design dell'anta sagoma37 è caratterizzato da una lavorazione inclinata a 37 gradi, scopri tutta la linea di mobili.</v>
@@ -4227,7 +4227,7 @@
         <v/>
       </c>
       <c r="G69" t="str">
-        <v>sistema, origina, sistemas modulares, sistema modular, modular, design, dell, anta, sagoma, caratterizzato, lavorazione, inclinata, gradi, scopri, tutta, linea, mobili</v>
+        <v>sistema, origina, sistemi modulari, sistema modular, sistemas modulares, modular, design, dell, anta, sagoma, caratterizzato, lavorazione, inclinata, gradi, scopri, tutta, linea, mobili</v>
       </c>
       <c r="H69" t="str">
         <v/>
@@ -4257,7 +4257,7 @@
         <v>https://www.febalcasa.com/it/prodotti/origina-anta-sagoma37/</v>
       </c>
       <c r="Q69" t="str">
-        <v>sistemas-modulares</v>
+        <v>sistemi-modulari</v>
       </c>
       <c r="R69" t="str">
         <v>TRUE</v>
@@ -4271,7 +4271,7 @@
         <v>Cucina Origina Anta Sagoma 37</v>
       </c>
       <c r="C70" t="str">
-        <v>cocinas</v>
+        <v>cucine</v>
       </c>
       <c r="D70" t="str">
         <v>Il design dell'anta sagoma37 è caratterizzato da una lavorazione inclinata a 37 gradi, scopri tutta la linea di mobili.</v>
@@ -4283,7 +4283,7 @@
         <v/>
       </c>
       <c r="G70" t="str">
-        <v>cucina, origina, anta, sagoma, cocinas, cocina, kitchen, isla, design, dell, caratterizzato, lavorazione, inclinata, gradi, scopri, tutta, linea, mobili</v>
+        <v>cucina, origina, anta, sagoma, cucine, cocina, cocinas, kitchen, isla, design, dell, caratterizzato, lavorazione, inclinata, gradi, scopri, tutta, linea, mobili</v>
       </c>
       <c r="H70" t="str">
         <v/>
@@ -4313,7 +4313,7 @@
         <v>https://www.febalcasa.com/it/prodotti/origina-anta-sagoma37/</v>
       </c>
       <c r="Q70" t="str">
-        <v>cocinas</v>
+        <v>cucine</v>
       </c>
       <c r="R70" t="str">
         <v>TRUE</v>
@@ -4327,7 +4327,7 @@
         <v>Cucina Origina Anta Sagoma 37</v>
       </c>
       <c r="C71" t="str">
-        <v>cocinas</v>
+        <v>cucine</v>
       </c>
       <c r="D71" t="str">
         <v>Il design dell'anta sagoma37 è caratterizzato da una lavorazione inclinata a 37 gradi, scopri tutta la linea di mobili.</v>
@@ -4339,7 +4339,7 @@
         <v/>
       </c>
       <c r="G71" t="str">
-        <v>cucina, origina, anta, sagoma, cocinas, cocina, kitchen, isla, design, dell, caratterizzato, lavorazione, inclinata, gradi, scopri, tutta, linea, mobili</v>
+        <v>cucina, origina, anta, sagoma, cucine, cocina, cocinas, kitchen, isla, design, dell, caratterizzato, lavorazione, inclinata, gradi, scopri, tutta, linea, mobili</v>
       </c>
       <c r="H71" t="str">
         <v/>
@@ -4369,7 +4369,7 @@
         <v>https://www.febalcasa.com/it/prodotti/origina-anta-sagoma37/</v>
       </c>
       <c r="Q71" t="str">
-        <v>cocinas</v>
+        <v>cucine</v>
       </c>
       <c r="R71" t="str">
         <v>TRUE</v>
@@ -4383,10 +4383,10 @@
         <v>Boiserie</v>
       </c>
       <c r="C72" t="str">
-        <v>paneles decorativos</v>
+        <v>boiserie</v>
       </c>
       <c r="D72" t="str">
-        <v>La parete attrezzata boiserie è concepita come un sistema in grado di dialogare con tutti gli altri arredi della gamma Febal Casa</v>
+        <v>La boiserie è concepita come un sistema in grado di dialogare con tutti gli altri arredi della gamma Febal Casa, un elemento versatile che si innesta con soluzione di continuità arrivando fino a terra.</v>
       </c>
       <c r="E72" t="str">
         <v/>
@@ -4395,7 +4395,7 @@
         <v/>
       </c>
       <c r="G72" t="str">
-        <v>boiserie, paneles decorativos, panel, revestimiento, pared, decorativo, columna, vertical, parete, attrezzata, concepita, sistema, grado, dialogare, tutti, altri, arredi, gamma, febal</v>
+        <v>boiserie, panel, paneles decorativos, revestimiento, pared, decorativo, columna, vertical, concepita, sistema, grado, dialogare, tutti, altri, arredi, gamma, febal, casa, elemento</v>
       </c>
       <c r="H72" t="str">
         <v/>
@@ -4425,7 +4425,7 @@
         <v>https://www.febalcasa.com/it/prodotti/boiserie/</v>
       </c>
       <c r="Q72" t="str">
-        <v>paneles-decorativos</v>
+        <v>boiserie</v>
       </c>
       <c r="R72" t="str">
         <v>TRUE</v>
@@ -4439,10 +4439,10 @@
         <v>Tavolo Leeds</v>
       </c>
       <c r="C73" t="str">
-        <v>mesas</v>
+        <v>tavoli</v>
       </c>
       <c r="D73" t="str">
-        <v>Il tavolo Leeds è disponibile in versione fissa e allungabile e in forma rettangolare o a botte per incontrare ogni esigenza di stile e spazio. La base</v>
+        <v>Il tavolo Leeds è disponibile in versione fissa e allungabile e in forma rettangolare o a botte per incontrare ogni esigenza di stile e spazio. La base scultorea è la caratteristica distintiva del modello: personalizzabile in cinque finiture metallo è in grado di abbinarsi perfettamente con i materiali del piano e dare vita a composizioni uniche.</v>
       </c>
       <c r="E73" t="str">
         <v/>
@@ -4451,7 +4451,7 @@
         <v/>
       </c>
       <c r="G73" t="str">
-        <v>tavolo, leeds, mesas, mesa, table, comedor, disponibile, versione, fissa, allungabile, forma, rettangolare, botte, incontrare, ogni, esigenza</v>
+        <v>tavolo, leeds, tavoli, mesa, mesas, table, comedor, disponibile, versione, fissa, allungabile, forma, rettangolare, botte, incontrare, ogni, esigenza</v>
       </c>
       <c r="H73" t="str">
         <v/>
@@ -4481,7 +4481,7 @@
         <v>https://www.febalcasa.com/it/prodotti/leeds/</v>
       </c>
       <c r="Q73" t="str">
-        <v>mesas</v>
+        <v>tavoli</v>
       </c>
       <c r="R73" t="str">
         <v>TRUE</v>
@@ -4495,10 +4495,10 @@
         <v>Sedia Nives con braccioli</v>
       </c>
       <c r="C74" t="str">
-        <v>sillas</v>
+        <v>sedie</v>
       </c>
       <c r="D74" t="str">
-        <v>Eleganti e di design la sedia e la poltroncina Nives sono anche estremamente accoglienti grazie alla seduta imbottita e ai braccioli che assicurano avvolgenza</v>
+        <v>Eleganti e di design la sedia e la poltroncina Nives sono anche estremamente accoglienti grazie alla seduta imbottita e ai braccioli che assicurano avvolgenza e comodità. Le linee dolci e sinuose, la versatilità, l'ergonomia della seduta e dello schienale rendono Nives una vera e propria icona di comfort. L'alta qualità dei materiali, la cura sartoriale della realizzazione e i numerosi rivestimenti e finiture fanno di Nives l'elemento d'arredo giusto per conferire eleganza e forte personalità a qualsiasi ambiente. Le gambe sono personalizzabili in metallo verniciato nelle finiture Ottone scuro, Nero, Antracite e Sabbia per incontrare ogni esigenza.</v>
       </c>
       <c r="E74" t="str">
         <v/>
@@ -4507,7 +4507,7 @@
         <v/>
       </c>
       <c r="G74" t="str">
-        <v>sedia, nives, braccioli, sillas, silla, chair, asiento, eleganti, design, poltroncina, estremamente, accoglienti, grazie, seduta, imbottita, assicurano</v>
+        <v>sedia, nives, braccioli, sedie, silla, sillas, chair, asiento, seduta, finiture, eleganti, design, poltroncina, estremamente, accoglienti, grazie, imbottita</v>
       </c>
       <c r="H74" t="str">
         <v/>
@@ -4537,7 +4537,7 @@
         <v>https://www.febalcasa.com/it/prodotti/nives/</v>
       </c>
       <c r="Q74" t="str">
-        <v>sillas</v>
+        <v>sedie</v>
       </c>
       <c r="R74" t="str">
         <v>TRUE</v>
@@ -4551,7 +4551,7 @@
         <v>Armadio Scorrevole Rodin</v>
       </c>
       <c r="C75" t="str">
-        <v>armarios</v>
+        <v>armadi</v>
       </c>
       <c r="D75" t="str">
         <v>L’armadio con anta scorrevole Rodin si distingue per la maniglia orizzontale con LED integrato, regolabile via app o telecomando.</v>
@@ -4563,7 +4563,7 @@
         <v/>
       </c>
       <c r="G75" t="str">
-        <v>armadio, scorrevole, rodin, armarios, armario, closet, ropero, wardrobe, cabina armadio, vestidor, anta, distingue, maniglia, orizzontale, integrato, regolabile, telecomando</v>
+        <v>armadio, scorrevole, rodin, armadi, armario, armarios, closet, ropero, wardrobe, cabina armadio, vestidor, anta, distingue, maniglia, orizzontale, integrato, regolabile, telecomando</v>
       </c>
       <c r="H75" t="str">
         <v/>
@@ -4593,7 +4593,7 @@
         <v>https://www.febalcasa.com/it/prodotti/rodin/</v>
       </c>
       <c r="Q75" t="str">
-        <v>armarios</v>
+        <v>armadi</v>
       </c>
       <c r="R75" t="str">
         <v>TRUE</v>
@@ -4607,7 +4607,7 @@
         <v>Cabina Armadio Hype</v>
       </c>
       <c r="C76" t="str">
-        <v>armarios</v>
+        <v>armadi</v>
       </c>
       <c r="D76" t="str">
         <v>Hype è un sistema modulare per cabine armadio con struttura a cremagliera, pensato per soluzioni lineari, angolari o su misura.</v>
@@ -4619,7 +4619,7 @@
         <v/>
       </c>
       <c r="G76" t="str">
-        <v>cabina, armadio, hype, armarios, armario, closet, ropero, wardrobe, cabina armadio, vestidor, sistema, modulare, cabine, struttura, cremagliera, pensato, soluzioni, lineari, angolari, misura</v>
+        <v>cabina, armadio, hype, armadi, armario, armarios, closet, ropero, wardrobe, cabina armadio, vestidor, sistema, modulare, cabine, struttura, cremagliera, pensato, soluzioni, lineari, angolari, misura</v>
       </c>
       <c r="H76" t="str">
         <v/>
@@ -4649,7 +4649,7 @@
         <v>https://www.febalcasa.com/it/prodotti/hype/</v>
       </c>
       <c r="Q76" t="str">
-        <v>armarios</v>
+        <v>armadi</v>
       </c>
       <c r="R76" t="str">
         <v>TRUE</v>
@@ -4663,7 +4663,7 @@
         <v>Isola Onda - Zaha Hadid Architects</v>
       </c>
       <c r="C77" t="str">
-        <v>cocinas</v>
+        <v>cucine</v>
       </c>
       <c r="D77" t="str">
         <v>Isola Onda - Zaha Hadid Architects — pieza de la colección Febal Casa, sección CASA 04 - A-MARE.</v>
@@ -4675,7 +4675,7 @@
         <v/>
       </c>
       <c r="G77" t="str">
-        <v>isola, onda, zaha, hadid, architects, cocinas, cocina, cucina, kitchen, isla, casa, pieza, coleccion, febal, seccion, mare</v>
+        <v>isola, onda, zaha, hadid, architects, cucine, cocina, cocinas, cucina, kitchen, isla, casa, pieza, coleccion, febal, seccion, mare</v>
       </c>
       <c r="H77" t="str">
         <v/>
@@ -4705,7 +4705,7 @@
         <v>https://www.febalcasa.com/it/prodotti/origina-isola-onda/</v>
       </c>
       <c r="Q77" t="str">
-        <v>cocinas</v>
+        <v>cucine</v>
       </c>
       <c r="R77" t="str">
         <v>TRUE</v>
@@ -4719,7 +4719,7 @@
         <v>Sistema Origina anta Square</v>
       </c>
       <c r="C78" t="str">
-        <v>sistemas modulares</v>
+        <v>sistemi modulari</v>
       </c>
       <c r="D78" t="str">
         <v>L’anta square, disponibile con maniglia o con gola sagomata, integra perfettamente ambiente cucina e living creando spazi unici e multifunzionali.</v>
@@ -4731,7 +4731,7 @@
         <v/>
       </c>
       <c r="G78" t="str">
-        <v>sistema, origina, anta, square, sistemas modulares, sistema modular, modular, disponibile, maniglia, gola, sagomata, integra, perfettamente, ambiente, cucina, living, creando</v>
+        <v>sistema, origina, anta, square, sistemi modulari, sistema modular, sistemas modulares, modular, disponibile, maniglia, gola, sagomata, integra, perfettamente, ambiente, cucina, living, creando</v>
       </c>
       <c r="H78" t="str">
         <v/>
@@ -4761,7 +4761,7 @@
         <v>https://www.febalcasa.com/it/prodotti/origina-anta-square/</v>
       </c>
       <c r="Q78" t="str">
-        <v>sistemas-modulares</v>
+        <v>sistemi-modulari</v>
       </c>
       <c r="R78" t="str">
         <v>TRUE</v>
@@ -4775,7 +4775,7 @@
         <v>Sistema Origina anta Square</v>
       </c>
       <c r="C79" t="str">
-        <v>sistemas modulares</v>
+        <v>sistemi modulari</v>
       </c>
       <c r="D79" t="str">
         <v>L’anta square, disponibile con maniglia o con gola sagomata, integra perfettamente ambiente cucina e living creando spazi unici e multifunzionali.</v>
@@ -4787,7 +4787,7 @@
         <v/>
       </c>
       <c r="G79" t="str">
-        <v>sistema, origina, anta, square, sistemas modulares, sistema modular, modular, disponibile, maniglia, gola, sagomata, integra, perfettamente, ambiente, cucina, living, creando</v>
+        <v>sistema, origina, anta, square, sistemi modulari, sistema modular, sistemas modulares, modular, disponibile, maniglia, gola, sagomata, integra, perfettamente, ambiente, cucina, living, creando</v>
       </c>
       <c r="H79" t="str">
         <v/>
@@ -4817,7 +4817,7 @@
         <v>https://www.febalcasa.com/it/prodotti/origina-anta-square/</v>
       </c>
       <c r="Q79" t="str">
-        <v>sistemas-modulares</v>
+        <v>sistemi-modulari</v>
       </c>
       <c r="R79" t="str">
         <v>TRUE</v>
@@ -4831,7 +4831,7 @@
         <v>Armadio Profile/ Leather</v>
       </c>
       <c r="C80" t="str">
-        <v>armarios</v>
+        <v>armadi</v>
       </c>
       <c r="D80" t="str">
         <v>L'armadio con anta battente Profile Leather di Febal Casa combina eleganza materica e funzionalità per un arredo raffinato.</v>
@@ -4843,7 +4843,7 @@
         <v/>
       </c>
       <c r="G80" t="str">
-        <v>armadio, profile/, leather, armarios, armario, closet, ropero, wardrobe, cabina armadio, vestidor, anta, battente, profile, febal, casa, combina, eleganza, materica, funzionalita, arredo</v>
+        <v>armadio, profile/, leather, armadi, armario, armarios, closet, ropero, wardrobe, cabina armadio, vestidor, anta, battente, profile, febal, casa, combina, eleganza, materica, funzionalita, arredo</v>
       </c>
       <c r="H80" t="str">
         <v/>
@@ -4873,7 +4873,7 @@
         <v>https://www.febalcasa.com/it/tipologia/armadi/ante/battente/profile-leather/</v>
       </c>
       <c r="Q80" t="str">
-        <v>armarios</v>
+        <v>armadi</v>
       </c>
       <c r="R80" t="str">
         <v>TRUE</v>
@@ -4887,7 +4887,7 @@
         <v>Armadio Profile/ Leather</v>
       </c>
       <c r="C81" t="str">
-        <v>armarios</v>
+        <v>armadi</v>
       </c>
       <c r="D81" t="str">
         <v>L'armadio con anta battente Profile Leather di Febal Casa combina eleganza materica e funzionalità per un arredo raffinato.</v>
@@ -4899,7 +4899,7 @@
         <v/>
       </c>
       <c r="G81" t="str">
-        <v>armadio, profile/, leather, armarios, armario, closet, ropero, wardrobe, cabina armadio, vestidor, anta, battente, profile, febal, casa, combina, eleganza, materica, funzionalita, arredo</v>
+        <v>armadio, profile/, leather, armadi, armario, armarios, closet, ropero, wardrobe, cabina armadio, vestidor, anta, battente, profile, febal, casa, combina, eleganza, materica, funzionalita, arredo</v>
       </c>
       <c r="H81" t="str">
         <v/>
@@ -4929,7 +4929,7 @@
         <v>https://www.febalcasa.com/it/tipologia/armadi/ante/battente/profile-leather/</v>
       </c>
       <c r="Q81" t="str">
-        <v>armarios</v>
+        <v>armadi</v>
       </c>
       <c r="R81" t="str">
         <v>TRUE</v>
@@ -4943,7 +4943,7 @@
         <v>Armadio Profile/ Solid</v>
       </c>
       <c r="C82" t="str">
-        <v>armarios</v>
+        <v>armadi</v>
       </c>
       <c r="D82" t="str">
         <v>Solidità e design si incontrano nell’anta Profile Solid, per armadi battenti dal carattere moderno e di design.</v>
@@ -4955,7 +4955,7 @@
         <v/>
       </c>
       <c r="G82" t="str">
-        <v>armadio, profile/, solid, armarios, armario, closet, ropero, wardrobe, cabina armadio, vestidor, design, solidita, incontrano, nell, anta, profile, armadi, battenti, carattere, moderno</v>
+        <v>armadio, profile/, solid, armadi, armario, armarios, closet, ropero, wardrobe, cabina armadio, vestidor, design, solidita, incontrano, nell, anta, profile, battenti, carattere, moderno</v>
       </c>
       <c r="H82" t="str">
         <v/>
@@ -4985,7 +4985,7 @@
         <v>https://www.febalcasa.com/it/tipologia/armadi/ante/battente/profile-solid/</v>
       </c>
       <c r="Q82" t="str">
-        <v>armarios</v>
+        <v>armadi</v>
       </c>
       <c r="R82" t="str">
         <v>TRUE</v>
@@ -4999,7 +4999,7 @@
         <v>Armadio Profile/ Solid</v>
       </c>
       <c r="C83" t="str">
-        <v>armarios</v>
+        <v>armadi</v>
       </c>
       <c r="D83" t="str">
         <v>Solidità e design si incontrano nell’anta Profile Solid, per armadi battenti dal carattere moderno e di design.</v>
@@ -5011,7 +5011,7 @@
         <v/>
       </c>
       <c r="G83" t="str">
-        <v>armadio, profile/, solid, armarios, armario, closet, ropero, wardrobe, cabina armadio, vestidor, design, solidita, incontrano, nell, anta, profile, armadi, battenti, carattere, moderno</v>
+        <v>armadio, profile/, solid, armadi, armario, armarios, closet, ropero, wardrobe, cabina armadio, vestidor, design, solidita, incontrano, nell, anta, profile, battenti, carattere, moderno</v>
       </c>
       <c r="H83" t="str">
         <v/>
@@ -5041,7 +5041,7 @@
         <v>https://www.febalcasa.com/it/tipologia/armadi/ante/battente/profile-solid/</v>
       </c>
       <c r="Q83" t="str">
-        <v>armarios</v>
+        <v>armadi</v>
       </c>
       <c r="R83" t="str">
         <v>TRUE</v>
@@ -5055,7 +5055,7 @@
         <v>Armadio Profile/ Reflex</v>
       </c>
       <c r="C84" t="str">
-        <v>armarios</v>
+        <v>armadi</v>
       </c>
       <c r="D84" t="str">
         <v>L'armadio con anta battente Profile Reflex riflette lo stile contemporaneo con finiture luminose e dettagli eleganti.</v>
@@ -5067,7 +5067,7 @@
         <v/>
       </c>
       <c r="G84" t="str">
-        <v>armadio, profile/, reflex, armarios, armario, closet, ropero, wardrobe, cabina armadio, vestidor, anta, battente, profile, riflette, stile, contemporaneo, finiture, luminose, dettagli, eleganti</v>
+        <v>armadio, profile/, reflex, armadi, armario, armarios, closet, ropero, wardrobe, cabina armadio, vestidor, anta, battente, profile, riflette, stile, contemporaneo, finiture, luminose, dettagli, eleganti</v>
       </c>
       <c r="H84" t="str">
         <v/>
@@ -5097,7 +5097,7 @@
         <v>https://www.febalcasa.com/it/tipologia/armadi/ante/battente/profile-reflex/</v>
       </c>
       <c r="Q84" t="str">
-        <v>armarios</v>
+        <v>armadi</v>
       </c>
       <c r="R84" t="str">
         <v>TRUE</v>
@@ -5111,7 +5111,7 @@
         <v>Armadio battente Aurora</v>
       </c>
       <c r="C85" t="str">
-        <v>armarios</v>
+        <v>armadi</v>
       </c>
       <c r="D85" t="str">
         <v>L'armadio con anta battente Aurora è disegnata con un profilo a doppia cornice in metallo Carbon grey e può accogliere un vetro Ombra fumé o Stop-sol.</v>
@@ -5123,7 +5123,7 @@
         <v/>
       </c>
       <c r="G85" t="str">
-        <v>armadio, battente, aurora, armarios, armario, closet, ropero, wardrobe, cabina armadio, vestidor, anta, disegnata, profilo, doppia, cornice, metallo, carbon, grey, accogliere</v>
+        <v>armadio, battente, aurora, armadi, armario, armarios, closet, ropero, wardrobe, cabina armadio, vestidor, anta, disegnata, profilo, doppia, cornice, metallo, carbon, grey, accogliere</v>
       </c>
       <c r="H85" t="str">
         <v/>
@@ -5153,7 +5153,7 @@
         <v>https://www.febalcasa.com/it/prodotti/aurora-porta-battente/</v>
       </c>
       <c r="Q85" t="str">
-        <v>armarios</v>
+        <v>armadi</v>
       </c>
       <c r="R85" t="str">
         <v>TRUE</v>
@@ -5167,7 +5167,7 @@
         <v>Cucina Anta Telaio Alluminio vetro</v>
       </c>
       <c r="C86" t="str">
-        <v>cocinas</v>
+        <v>cucine</v>
       </c>
       <c r="D86" t="str">
         <v>L’anta con telaio in alluminio offre molteplici possibilità di personalizzazione grazie alle numerose finiture e possibilità di apertura.</v>
@@ -5179,7 +5179,7 @@
         <v/>
       </c>
       <c r="G86" t="str">
-        <v>cucina, anta, telaio, alluminio, vetro, cocinas, cocina, kitchen, isla, possibilita, offre, molteplici, personalizzazione, grazie, numerose, finiture, apertura</v>
+        <v>cucina, anta, telaio, alluminio, vetro, cucine, cocina, cocinas, kitchen, isla, possibilita, offre, molteplici, personalizzazione, grazie, numerose, finiture, apertura</v>
       </c>
       <c r="H86" t="str">
         <v/>
@@ -5209,7 +5209,7 @@
         <v>https://www.febalcasa.com/it/prodotti/origina-anta-telaio-alluminio/</v>
       </c>
       <c r="Q86" t="str">
-        <v>cocinas</v>
+        <v>cucine</v>
       </c>
       <c r="R86" t="str">
         <v>TRUE</v>
@@ -5223,7 +5223,7 @@
         <v>Armadio Barret</v>
       </c>
       <c r="C87" t="str">
-        <v>armarios</v>
+        <v>armadi</v>
       </c>
       <c r="D87" t="str">
         <v>L'armadio con anta battente Barret è contraddistinta da una piacevole essenzialità formale personalizzabile grazie alla gamma di maniglie dedicate.</v>
@@ -5235,7 +5235,7 @@
         <v/>
       </c>
       <c r="G87" t="str">
-        <v>armadio, barret, armarios, armario, closet, ropero, wardrobe, cabina armadio, vestidor, anta, battente, contraddistinta, piacevole, essenzialita, formale, personalizzabile, grazie, gamma, maniglie</v>
+        <v>armadio, barret, armadi, armario, armarios, closet, ropero, wardrobe, cabina armadio, vestidor, anta, battente, contraddistinta, piacevole, essenzialita, formale, personalizzabile, grazie, gamma, maniglie</v>
       </c>
       <c r="H87" t="str">
         <v/>
@@ -5265,7 +5265,7 @@
         <v>https://www.febalcasa.com/it/prodotti/barret/</v>
       </c>
       <c r="Q87" t="str">
-        <v>armarios</v>
+        <v>armadi</v>
       </c>
       <c r="R87" t="str">
         <v>TRUE</v>
@@ -5279,10 +5279,10 @@
         <v>Sgabello Lola</v>
       </c>
       <c r="C88" t="str">
-        <v>taburetes</v>
+        <v>sgabelli</v>
       </c>
       <c r="D88" t="str">
-        <v>Disponibile con spalliera alta o bassa e in versione sgabello fisso o girevole, Lola presenta un design lineare ed estremo comfort. Accogliente e raffinata</v>
+        <v>Disponibile con spalliera alta o bassa e in versione sgabello fisso o girevole, Lola presenta un design lineare ed estremo comfort. Accogliente e raffinata Lola è adatta ad ogni contesto, anche il più sofisticato, grazie ai numerosi rivestimenti e alla forte ergonomia del modello. Lo schienale flessibile, offre una seduta estremamente comoda e piacevole che agevola l'appoggio della schiena assecondando il movimento del corpo. Le gambe sono disponibili in metallo verniciato nelle finiture Ottone scuro, nero, Antracite e Sabbia oppure rivestite in abbinamento alla seduta.</v>
       </c>
       <c r="E88" t="str">
         <v/>
@@ -5291,7 +5291,7 @@
         <v/>
       </c>
       <c r="G88" t="str">
-        <v>sgabello, lola, taburetes, taburete, banqueta, stool, bar, disponibile, spalliera, alta, bassa, versione, fisso, girevole, presenta, design, lineare</v>
+        <v>sgabello, lola, sgabelli, taburete, taburetes, banqueta, stool, bar, seduta, disponibile, spalliera, alta, bassa, versione, fisso, girevole, presenta, design</v>
       </c>
       <c r="H88" t="str">
         <v/>
@@ -5321,7 +5321,7 @@
         <v>https://www.febalcasa.com/it/prodotti/lola/</v>
       </c>
       <c r="Q88" t="str">
-        <v>taburetes</v>
+        <v>sgabelli</v>
       </c>
       <c r="R88" t="str">
         <v>TRUE</v>
@@ -5335,7 +5335,7 @@
         <v>Armadio Lumia</v>
       </c>
       <c r="C89" t="str">
-        <v>armarios</v>
+        <v>armadi</v>
       </c>
       <c r="D89" t="str">
         <v>L'armadio con anta battente Lumia è un classico senza tempo nell'arredo della zona notte. Lumia presenta l’esclusiva illuminazione led integrata.</v>
@@ -5347,7 +5347,7 @@
         <v/>
       </c>
       <c r="G89" t="str">
-        <v>armadio, lumia, armarios, armario, closet, ropero, wardrobe, cabina armadio, vestidor, anta, battente, classico, senza, tempo, nell, arredo, zona, notte, presenta</v>
+        <v>armadio, lumia, armadi, armario, armarios, closet, ropero, wardrobe, cabina armadio, vestidor, anta, battente, classico, senza, tempo, nell, arredo, zona, notte, presenta</v>
       </c>
       <c r="H89" t="str">
         <v/>
@@ -5377,7 +5377,7 @@
         <v>https://www.febalcasa.com/it/prodotti/lewitt-lumia/</v>
       </c>
       <c r="Q89" t="str">
-        <v>armarios</v>
+        <v>armadi</v>
       </c>
       <c r="R89" t="str">
         <v>TRUE</v>
@@ -5391,7 +5391,7 @@
         <v>Armadio Lumia</v>
       </c>
       <c r="C90" t="str">
-        <v>armarios</v>
+        <v>armadi</v>
       </c>
       <c r="D90" t="str">
         <v>L'armadio con anta battente Lumia è un classico senza tempo nell'arredo della zona notte. Lumia presenta l’esclusiva illuminazione led integrata.</v>
@@ -5403,7 +5403,7 @@
         <v/>
       </c>
       <c r="G90" t="str">
-        <v>armadio, lumia, armarios, armario, closet, ropero, wardrobe, cabina armadio, vestidor, anta, battente, classico, senza, tempo, nell, arredo, zona, notte, presenta</v>
+        <v>armadio, lumia, armadi, armario, armarios, closet, ropero, wardrobe, cabina armadio, vestidor, anta, battente, classico, senza, tempo, nell, arredo, zona, notte, presenta</v>
       </c>
       <c r="H90" t="str">
         <v/>
@@ -5433,7 +5433,7 @@
         <v>https://www.febalcasa.com/it/prodotti/lewitt-lumia/</v>
       </c>
       <c r="Q90" t="str">
-        <v>armarios</v>
+        <v>armadi</v>
       </c>
       <c r="R90" t="str">
         <v>TRUE</v>
@@ -5447,7 +5447,7 @@
         <v>Armadio Lewitt Plus</v>
       </c>
       <c r="C91" t="str">
-        <v>armarios</v>
+        <v>armadi</v>
       </c>
       <c r="D91" t="str">
         <v>L'armadio con anta battente Lewitt Plus con presa a gola continua unisce design e massima personalizzazione, ideale per ambienti contemporanei.</v>
@@ -5459,7 +5459,7 @@
         <v/>
       </c>
       <c r="G91" t="str">
-        <v>armadio, lewitt, plus, armarios, armario, closet, ropero, wardrobe, cabina armadio, vestidor, anta, battente, presa, gola, continua, unisce, design, massima, personalizzazione</v>
+        <v>armadio, lewitt, plus, armadi, armario, armarios, closet, ropero, wardrobe, cabina armadio, vestidor, anta, battente, presa, gola, continua, unisce, design, massima, personalizzazione</v>
       </c>
       <c r="H91" t="str">
         <v/>
@@ -5489,7 +5489,7 @@
         <v>https://www.febalcasa.com/it/prodotti/lewitt-plus/</v>
       </c>
       <c r="Q91" t="str">
-        <v>armarios</v>
+        <v>armadi</v>
       </c>
       <c r="R91" t="str">
         <v>TRUE</v>
@@ -5503,10 +5503,10 @@
         <v>Tavolo Madeira</v>
       </c>
       <c r="C92" t="str">
-        <v>mesas</v>
+        <v>tavoli</v>
       </c>
       <c r="D92" t="str">
-        <v>L’armonioso intreccio di archi definisce un tavolo unico, protagonista di ogni ambiente. Le gambe inclinate e sovrapposte formano un disegno geometrico di</v>
+        <v>L'armonioso intreccio di archi definisce un tavolo unico, protagonista di ogni ambiente. Le gambe inclinate e sovrapposte formano un disegno geometrico di grande impatto visivo che gioca con la tridimensionalità ottenendo un risultato perfetto nato dall'eleganza, dall'equilibrio e dalla leggerezza dei volumi. La base in metallo è disponibile in finitura Ottone Scuro, Nero, Antracite e Sabbia. Il piano è di forma rotonda, ovale fisso o allungabile ed è configurabile in Cristallo Lucido, Cristallo Velvet, Superceramica, Supermarmo opaco, Supermarmo lucido e legno Impiallacciato. La versione fissa può essere arricchita con il piano centrotavola girevole, un dispositivo rotante che permette di condividere facilmente cibi e oggetti con tutti i commensali.</v>
       </c>
       <c r="E92" t="str">
         <v/>
@@ -5515,7 +5515,7 @@
         <v/>
       </c>
       <c r="G92" t="str">
-        <v>tavolo, madeira, mesas, mesa, table, comedor, armonioso, intreccio, archi, definisce, unico, protagonista, ogni, ambiente, gambe, inclinate, sovrapposte</v>
+        <v>tavolo, madeira, tavoli, mesa, mesas, table, comedor, dall, piano, cristallo, lucido, supermarmo, armonioso, intreccio, archi, definisce, unico, protagonista</v>
       </c>
       <c r="H92" t="str">
         <v/>
@@ -5545,7 +5545,7 @@
         <v>https://www.febalcasa.com/it/prodotti/madeira/</v>
       </c>
       <c r="Q92" t="str">
-        <v>mesas</v>
+        <v>tavoli</v>
       </c>
       <c r="R92" t="str">
         <v>TRUE</v>
@@ -5559,10 +5559,10 @@
         <v>Sedia Dea</v>
       </c>
       <c r="C93" t="str">
-        <v>sillas</v>
+        <v>sedie</v>
       </c>
       <c r="D93" t="str">
-        <v>La sedia Dea è perfetta per progetti raffinati in ogni dettaglio. La linearità delle gambe in metallo verniciato disponibile nelle finiture Ottone scuro,</v>
+        <v>La sedia Dea è perfetta per progetti raffinati in ogni dettaglio. La linearità delle gambe in metallo verniciato disponibile nelle finiture Ottone scuro, Antracite, Nero e Sabbia è ammorbidita dalle forme curve e accoglienti della seduta e dello schienale, arricchite da un prezioso tocco sartoriale che si rivela con il grazioso movimento di pieghe che enfatizza i volumi e il senso di comfort. Dea è una sedia di valore che cattura inevitabilmente l'ammirazione di chiunque la osservi.</v>
       </c>
       <c r="E93" t="str">
         <v/>
@@ -5571,7 +5571,7 @@
         <v/>
       </c>
       <c r="G93" t="str">
-        <v>sedia, dea, sillas, silla, chair, asiento, perfetta, progetti, raffinati, ogni, dettaglio, linearita, gambe, metallo, verniciato, disponibile, nelle</v>
+        <v>sedia, dea, sedie, silla, sillas, chair, asiento, perfetta, progetti, raffinati, ogni, dettaglio, linearita, gambe, metallo, verniciato, disponibile, nelle</v>
       </c>
       <c r="H93" t="str">
         <v/>
@@ -5601,7 +5601,7 @@
         <v>https://www.febalcasa.com/it/prodotti/dea/</v>
       </c>
       <c r="Q93" t="str">
-        <v>sillas</v>
+        <v>sedie</v>
       </c>
       <c r="R93" t="str">
         <v>TRUE</v>
@@ -5615,10 +5615,10 @@
         <v>Tavolo Daniel</v>
       </c>
       <c r="C94" t="str">
-        <v>mesas</v>
+        <v>tavoli</v>
       </c>
       <c r="D94" t="str">
-        <v>Sinonimo di estrema eleganza, il tavolo Daniel con struttura ponte gamba rappresenta il punto centrale della sala da pranzo, il luogo dove si riuniscono</v>
+        <v>Sinonimo di estrema eleganza, il tavolo Daniel con struttura ponte gamba rappresenta il punto centrale della sala da pranzo, il luogo dove si riuniscono familiari e amici. Il suo piano personalizzabile in cristallo, superceramica e supermarmo accoglie comodamente i commensali garantendo qualità negli anni. Il modello è disponibile in forma quadrata, rettangolare e rettangolare allungabile.</v>
       </c>
       <c r="E94" t="str">
         <v/>
@@ -5627,7 +5627,7 @@
         <v/>
       </c>
       <c r="G94" t="str">
-        <v>tavolo, daniel, mesas, mesa, table, comedor, sinonimo, estrema, eleganza, struttura, ponte, gamba, rappresenta, punto, centrale, sala</v>
+        <v>tavolo, daniel, tavoli, mesa, mesas, table, comedor, rettangolare, sinonimo, estrema, eleganza, struttura, ponte, gamba, rappresenta, punto, centrale</v>
       </c>
       <c r="H94" t="str">
         <v/>
@@ -5657,7 +5657,7 @@
         <v>https://www.febalcasa.com/it/prodotti/daniel/</v>
       </c>
       <c r="Q94" t="str">
-        <v>mesas</v>
+        <v>tavoli</v>
       </c>
       <c r="R94" t="str">
         <v>TRUE</v>
@@ -5671,10 +5671,10 @@
         <v>Sedia Dea</v>
       </c>
       <c r="C95" t="str">
-        <v>sillas</v>
+        <v>sedie</v>
       </c>
       <c r="D95" t="str">
-        <v>La sedia Dea è perfetta per progetti raffinati in ogni dettaglio. La linearità delle gambe in metallo verniciato disponibile nelle finiture Ottone scuro,</v>
+        <v>La sedia Dea è perfetta per progetti raffinati in ogni dettaglio. La linearità delle gambe in metallo verniciato disponibile nelle finiture Ottone scuro, Antracite, Nero e Sabbia è ammorbidita dalle forme curve e accoglienti della seduta e dello schienale, arricchite da un prezioso tocco sartoriale che si rivela con il grazioso movimento di pieghe che enfatizza i volumi e il senso di comfort. Dea è una sedia di valore che cattura inevitabilmente l'ammirazione di chiunque la osservi.</v>
       </c>
       <c r="E95" t="str">
         <v/>
@@ -5683,7 +5683,7 @@
         <v/>
       </c>
       <c r="G95" t="str">
-        <v>sedia, dea, sillas, silla, chair, asiento, perfetta, progetti, raffinati, ogni, dettaglio, linearita, gambe, metallo, verniciato, disponibile, nelle</v>
+        <v>sedia, dea, sedie, silla, sillas, chair, asiento, perfetta, progetti, raffinati, ogni, dettaglio, linearita, gambe, metallo, verniciato, disponibile, nelle</v>
       </c>
       <c r="H95" t="str">
         <v/>
@@ -5713,7 +5713,7 @@
         <v>https://www.febalcasa.com/it/prodotti/dea/</v>
       </c>
       <c r="Q95" t="str">
-        <v>sillas</v>
+        <v>sedie</v>
       </c>
       <c r="R95" t="str">
         <v>TRUE</v>
@@ -5727,10 +5727,10 @@
         <v>Boiserie</v>
       </c>
       <c r="C96" t="str">
-        <v>paneles decorativos</v>
+        <v>boiserie</v>
       </c>
       <c r="D96" t="str">
-        <v>La parete attrezzata boiserie è concepita come un sistema in grado di dialogare con tutti gli altri arredi della gamma Febal Casa</v>
+        <v>La boiserie è concepita come un sistema in grado di dialogare con tutti gli altri arredi della gamma Febal Casa, un elemento versatile che si innesta con soluzione di continuità arrivando fino a terra.</v>
       </c>
       <c r="E96" t="str">
         <v/>
@@ -5739,7 +5739,7 @@
         <v/>
       </c>
       <c r="G96" t="str">
-        <v>boiserie, paneles decorativos, panel, revestimiento, pared, decorativo, columna, vertical, parete, attrezzata, concepita, sistema, grado, dialogare, tutti, altri, arredi, gamma, febal</v>
+        <v>boiserie, panel, paneles decorativos, revestimiento, pared, decorativo, columna, vertical, concepita, sistema, grado, dialogare, tutti, altri, arredi, gamma, febal, casa, elemento</v>
       </c>
       <c r="H96" t="str">
         <v/>
@@ -5769,7 +5769,7 @@
         <v>https://www.febalcasa.com/it/prodotti/boiserie/</v>
       </c>
       <c r="Q96" t="str">
-        <v>paneles-decorativos</v>
+        <v>boiserie</v>
       </c>
       <c r="R96" t="str">
         <v>TRUE</v>

</xml_diff>

<commit_message>
Baseline the uncommitted v1 chatbot work before the v2 refactor
Commits the working-tree state the v1 assistant has been running on:
catalog-engine matching/similarity/variants/color families, the Anthropic
and Claude Code orchestration paths, the Febal catalog pipeline and its
current catalog data, the CDP capture helpers, and the handoff notes.
Test outputs, experiment reports and the built tour export stay out.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/clients/febal-casa/catalog.xlsx
+++ b/clients/febal-casa/catalog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:T96"/>
+  <dimension ref="A1:U102"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -460,10 +460,13 @@
       <c r="T1" t="str">
         <v>style</v>
       </c>
+      <c r="U1" t="str">
+        <v>finish</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>box-100-b-103-boiserie-camino</v>
+        <v>FEB-001</v>
       </c>
       <c r="B2" t="str">
         <v>Boiserie camino</v>
@@ -475,10 +478,10 @@
         <v>La boiserie è concepita come un sistema in grado di dialogare con tutti gli altri arredi della gamma Febal Casa, un elemento versatile che si innesta con soluzione di continuità arrivando fino a terra.</v>
       </c>
       <c r="E2" t="str">
-        <v/>
+        <v>nero/grigio scuro venato</v>
       </c>
       <c r="F2" t="str">
-        <v/>
+        <v>pannello effetto pietra</v>
       </c>
       <c r="G2" t="str">
         <v>boiserie, camino, panel, paneles decorativos, revestimiento, pared, decorativo, columna, vertical, concepita, sistema, grado, dialogare, tutti, altri, arredi, gamma, febal, casa, elemento</v>
@@ -490,16 +493,16 @@
         <v>CASA 01 - AUTENTICA</v>
       </c>
       <c r="J2" t="str">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="K2">
-        <v>-81</v>
+        <v>-56.4</v>
       </c>
       <c r="L2">
-        <v>-4</v>
+        <v>-29.5</v>
       </c>
       <c r="M2">
-        <v>70</v>
+        <v>111.2</v>
       </c>
       <c r="N2" t="str">
         <v>BOX 100 - B_103</v>
@@ -517,15 +520,18 @@
         <v>TRUE</v>
       </c>
       <c r="S2" t="str">
-        <v/>
+        <v>boiserie modulare a tutta altezza</v>
       </c>
       <c r="T2" t="str">
-        <v/>
+        <v>Contemporaneo</v>
+      </c>
+      <c r="U2" t="str">
+        <v>Scenario</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>box-100-b-104-boiserie</v>
+        <v>FEB-002</v>
       </c>
       <c r="B3" t="str">
         <v>Boiserie</v>
@@ -537,10 +543,10 @@
         <v>La boiserie è concepita come un sistema in grado di dialogare con tutti gli altri arredi della gamma Febal Casa, un elemento versatile che si innesta con soluzione di continuità arrivando fino a terra.</v>
       </c>
       <c r="E3" t="str">
-        <v/>
+        <v>tortora/beige</v>
       </c>
       <c r="F3" t="str">
-        <v/>
+        <v>pannello laccato</v>
       </c>
       <c r="G3" t="str">
         <v>boiserie, panel, paneles decorativos, revestimiento, pared, decorativo, columna, vertical, concepita, sistema, grado, dialogare, tutti, altri, arredi, gamma, febal, casa, elemento</v>
@@ -555,13 +561,13 @@
         <v>14</v>
       </c>
       <c r="K3">
-        <v>46</v>
+        <v>39.6</v>
       </c>
       <c r="L3">
-        <v>7</v>
+        <v>5.1</v>
       </c>
       <c r="M3">
-        <v>70</v>
+        <v>110</v>
       </c>
       <c r="N3" t="str">
         <v>BOX 100 - B_104</v>
@@ -579,15 +585,18 @@
         <v>TRUE</v>
       </c>
       <c r="S3" t="str">
-        <v/>
+        <v>boiserie modulare a tutta altezza</v>
       </c>
       <c r="T3" t="str">
-        <v/>
+        <v>Contemporaneo</v>
+      </c>
+      <c r="U3" t="str">
+        <v>Laccato Opaco</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>box-100-b-106-divano-balmoral</v>
+        <v>FEB-003</v>
       </c>
       <c r="B4" t="str">
         <v>Divano Balmoral</v>
@@ -599,10 +608,10 @@
         <v>Un divano componibile pensato per interpretare le esigenze abitative contemporanee, coniugando estetica, ergonomia e versatilità. La scelta ideale per un soggiorno elegante, accogliente e su misura.</v>
       </c>
       <c r="E4" t="str">
-        <v/>
+        <v>verde oliva</v>
       </c>
       <c r="F4" t="str">
-        <v/>
+        <v>tessuto</v>
       </c>
       <c r="G4" t="str">
         <v>divano, balmoral, divani, sofa, sofá, sofás, couch, asiento, componibile, pensato, interpretare, esigenze, abitative, contemporanee, coniugando, estetica, ergonomia, versatilita, scelta</v>
@@ -617,13 +626,13 @@
         <v>11</v>
       </c>
       <c r="K4">
-        <v>-135</v>
+        <v>-152.7</v>
       </c>
       <c r="L4">
-        <v>-48</v>
+        <v>-52.8</v>
       </c>
       <c r="M4">
-        <v>70</v>
+        <v>101.4</v>
       </c>
       <c r="N4" t="str">
         <v>BOX 100 - B_106</v>
@@ -644,12 +653,15 @@
         <v>ad angolo</v>
       </c>
       <c r="T4" t="str">
+        <v>Contemporaneo, Classico elegante</v>
+      </c>
+      <c r="U4" t="str">
         <v/>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>box-100-b-109-tavolino-rio</v>
+        <v>FEB-004</v>
       </c>
       <c r="B5" t="str">
         <v>Tavolino Rio</v>
@@ -661,10 +673,10 @@
         <v>Il tavolino Rio è contraddistinto da una struttura in metallo che presenta la particolarità di poter accogliere riviste e giornali. Una funzione che lo rende il compagno ideale nei momenti di relax. Il piano può essere configurato a seconda del proprio gusto in finitura laccata opaca o impiallacciata.</v>
       </c>
       <c r="E5" t="str">
-        <v/>
+        <v>marrone scuro/nero venato</v>
       </c>
       <c r="F5" t="str">
-        <v/>
+        <v>marmo</v>
       </c>
       <c r="G5" t="str">
         <v>tavolino, rio, tavolini, mesa de centro, mesita, coffee table, contraddistinto, struttura, metallo, presenta, particolarita, poter, accogliere, riviste, giornali, funzione, rende</v>
@@ -679,13 +691,13 @@
         <v>11</v>
       </c>
       <c r="K5">
-        <v>89</v>
+        <v>98.1</v>
       </c>
       <c r="L5">
-        <v>-48</v>
+        <v>-50</v>
       </c>
       <c r="M5">
-        <v>70</v>
+        <v>75.8</v>
       </c>
       <c r="N5" t="str">
         <v>BOX 100 - B_109</v>
@@ -706,12 +718,15 @@
         <v/>
       </c>
       <c r="T5" t="str">
+        <v>Contemporaneo</v>
+      </c>
+      <c r="U5" t="str">
         <v/>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>box-100-b-110-tavolino-rio</v>
+        <v>FEB-005</v>
       </c>
       <c r="B6" t="str">
         <v>Tavolino Rio</v>
@@ -723,10 +738,10 @@
         <v>Il tavolino Rio è contraddistinto da una struttura in metallo che presenta la particolarità di poter accogliere riviste e giornali. Una funzione che lo rende il compagno ideale nei momenti di relax. Il piano può essere configurato a seconda del proprio gusto in finitura laccata opaca o impiallacciata.</v>
       </c>
       <c r="E6" t="str">
-        <v/>
+        <v>legno naturale</v>
       </c>
       <c r="F6" t="str">
-        <v/>
+        <v>legno</v>
       </c>
       <c r="G6" t="str">
         <v>tavolino, rio, tavolini, mesa de centro, mesita, coffee table, contraddistinto, struttura, metallo, presenta, particolarita, poter, accogliere, riviste, giornali, funzione, rende</v>
@@ -738,16 +753,16 @@
         <v>CASA 01 - AUTENTICA</v>
       </c>
       <c r="J6" t="str">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="K6">
-        <v>-44</v>
+        <v>95.3</v>
       </c>
       <c r="L6">
-        <v>-22</v>
+        <v>-38.5</v>
       </c>
       <c r="M6">
-        <v>70</v>
+        <v>93.9</v>
       </c>
       <c r="N6" t="str">
         <v>BOX 100 - B_110</v>
@@ -768,12 +783,15 @@
         <v/>
       </c>
       <c r="T6" t="str">
+        <v>Contemporaneo</v>
+      </c>
+      <c r="U6" t="str">
         <v/>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>box-100-b-125-boiserie</v>
+        <v>FEB-006</v>
       </c>
       <c r="B7" t="str">
         <v>Boiserie</v>
@@ -785,10 +803,10 @@
         <v>La boiserie è concepita come un sistema in grado di dialogare con tutti gli altri arredi della gamma Febal Casa, un elemento versatile che si innesta con soluzione di continuità arrivando fino a terra.</v>
       </c>
       <c r="E7" t="str">
-        <v/>
+        <v>nero venato bianco</v>
       </c>
       <c r="F7" t="str">
-        <v/>
+        <v>pannello effetto pietra</v>
       </c>
       <c r="G7" t="str">
         <v>boiserie, panel, paneles decorativos, revestimiento, pared, decorativo, columna, vertical, concepita, sistema, grado, dialogare, tutti, altri, arredi, gamma, febal, casa, elemento</v>
@@ -800,16 +818,16 @@
         <v>CASA 01 - AUTENTICA</v>
       </c>
       <c r="J7" t="str">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="K7">
-        <v>-63</v>
+        <v>35.7</v>
       </c>
       <c r="L7">
-        <v>-18</v>
+        <v>6.1</v>
       </c>
       <c r="M7">
-        <v>70</v>
+        <v>130</v>
       </c>
       <c r="N7" t="str">
         <v>BOX 100 - B_125</v>
@@ -827,15 +845,18 @@
         <v>TRUE</v>
       </c>
       <c r="S7" t="str">
-        <v/>
+        <v>boiserie modulare a tutta altezza</v>
       </c>
       <c r="T7" t="str">
-        <v/>
+        <v>Contemporaneo</v>
+      </c>
+      <c r="U7" t="str">
+        <v>Scenario</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>box-120-b-121-cucina-origina-anta-square-cannettato</v>
+        <v>FEB-007</v>
       </c>
       <c r="B8" t="str">
         <v>Cucina Origina Anta Square Cannettato</v>
@@ -844,16 +865,16 @@
         <v>cucine</v>
       </c>
       <c r="D8" t="str">
-        <v>Cucina Origina Anta Square Cannettato — pieza de la colección Febal Casa, sección CASA 01 - AUTENTICA.</v>
+        <v>Cucina Origina Anta Square Cannettato — elemento della collezione Febal Casa, sezione CASA 01 - AUTENTICA.</v>
       </c>
       <c r="E8" t="str">
-        <v/>
+        <v>rovere biondo, marmo marrone scuro venato</v>
       </c>
       <c r="F8" t="str">
-        <v/>
+        <v>legno, marmo</v>
       </c>
       <c r="G8" t="str">
-        <v>cucina, origina, anta, square, cannettato, cucine, cocina, cocinas, kitchen, isla, casa, pieza, coleccion, febal, seccion, autentica</v>
+        <v>cucina, origina, anta, square, cannettato, cucine, cocina, cocinas, kitchen, isla, casa, elemento, collezione, febal, sezione, autentica</v>
       </c>
       <c r="H8" t="str">
         <v/>
@@ -862,16 +883,16 @@
         <v>CASA 01 - AUTENTICA</v>
       </c>
       <c r="J8" t="str">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="K8">
-        <v>-6</v>
+        <v>52.7</v>
       </c>
       <c r="L8">
-        <v>-17</v>
+        <v>-36.9</v>
       </c>
       <c r="M8">
-        <v>70</v>
+        <v>110</v>
       </c>
       <c r="N8" t="str">
         <v>BOX 120 - B_121</v>
@@ -889,15 +910,18 @@
         <v>TRUE</v>
       </c>
       <c r="S8" t="str">
-        <v/>
+        <v>cucina componibile a isola</v>
       </c>
       <c r="T8" t="str">
-        <v/>
+        <v>Contemporaneo</v>
+      </c>
+      <c r="U8" t="str">
+        <v>Impiallacciato Opaco Cannettato</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>box-120-b-122-sistema-origina</v>
+        <v>FEB-008</v>
       </c>
       <c r="B9" t="str">
         <v>Sistema Origina</v>
@@ -906,16 +930,16 @@
         <v>sistemi modulari</v>
       </c>
       <c r="D9" t="str">
-        <v>Sistema Origina — pieza de la colección Febal Casa, sección CASA 01 - AUTENTICA.</v>
+        <v>Sistema Origina — elemento della collezione Febal Casa, sezione CASA 01 - AUTENTICA.</v>
       </c>
       <c r="E9" t="str">
-        <v/>
+        <v>rovere biondo, marmo marrone scuro venato</v>
       </c>
       <c r="F9" t="str">
-        <v/>
+        <v>legno, marmo</v>
       </c>
       <c r="G9" t="str">
-        <v>sistema, origina, sistemi modulari, sistema modular, sistemas modulares, modular, casa, pieza, coleccion, febal, seccion, autentica</v>
+        <v>sistema, origina, sistemi modulari, sistema modular, sistemas modulares, modular, casa, elemento, collezione, febal, sezione, autentica</v>
       </c>
       <c r="H9" t="str">
         <v/>
@@ -924,16 +948,16 @@
         <v>CASA 01 - AUTENTICA</v>
       </c>
       <c r="J9" t="str">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K9">
-        <v>10</v>
+        <v>7.3</v>
       </c>
       <c r="L9">
-        <v>-5</v>
+        <v>-3.4</v>
       </c>
       <c r="M9">
-        <v>70</v>
+        <v>130</v>
       </c>
       <c r="N9" t="str">
         <v>BOX 120 - B_122</v>
@@ -954,12 +978,15 @@
         <v/>
       </c>
       <c r="T9" t="str">
-        <v/>
+        <v>Contemporaneo</v>
+      </c>
+      <c r="U9" t="str">
+        <v>Impiallacciato Opaco Cannettato</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>box-120-b-123-sistema-origina</v>
+        <v>FEB-009</v>
       </c>
       <c r="B10" t="str">
         <v>Sistema Origina</v>
@@ -968,16 +995,16 @@
         <v>sistemi modulari</v>
       </c>
       <c r="D10" t="str">
-        <v>Sistema Origina — pieza de la colección Febal Casa, sección CASA 01 - AUTENTICA.</v>
+        <v>Sistema Origina — elemento della collezione Febal Casa, sezione CASA 01 - AUTENTICA.</v>
       </c>
       <c r="E10" t="str">
-        <v/>
+        <v>rovere biondo, marmo marrone scuro venato</v>
       </c>
       <c r="F10" t="str">
-        <v/>
+        <v>legno, marmo</v>
       </c>
       <c r="G10" t="str">
-        <v>sistema, origina, sistemi modulari, sistema modular, sistemas modulares, modular, casa, pieza, coleccion, febal, seccion, autentica</v>
+        <v>sistema, origina, sistemi modulari, sistema modular, sistemas modulares, modular, casa, elemento, collezione, febal, sezione, autentica</v>
       </c>
       <c r="H10" t="str">
         <v/>
@@ -989,13 +1016,13 @@
         <v>2</v>
       </c>
       <c r="K10">
-        <v>-7</v>
+        <v>136</v>
       </c>
       <c r="L10">
-        <v>4</v>
+        <v>-5.8</v>
       </c>
       <c r="M10">
-        <v>70</v>
+        <v>130</v>
       </c>
       <c r="N10" t="str">
         <v>BOX 120 - B_123</v>
@@ -1016,12 +1043,15 @@
         <v/>
       </c>
       <c r="T10" t="str">
-        <v/>
+        <v>Contemporaneo</v>
+      </c>
+      <c r="U10" t="str">
+        <v>Impiallacciato Opaco Cannettato</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>box-140-b-141-sistema-diciotto</v>
+        <v>FEB-010</v>
       </c>
       <c r="B11" t="str">
         <v>Sistema Diciotto</v>
@@ -1033,10 +1063,10 @@
         <v>Diciotto è una parete attrezzata per la zona living di design: pratico, versatile e funzionale permette una modularità altissima.</v>
       </c>
       <c r="E11" t="str">
-        <v/>
+        <v>antracite</v>
       </c>
       <c r="F11" t="str">
-        <v/>
+        <v>pannello laccato</v>
       </c>
       <c r="G11" t="str">
         <v>sistema, diciotto, sistemi modulari, sistema modular, sistemas modulares, modular, parete, attrezzata, zona, living, design, pratico, versatile, funzionale, permette, modularita, altissima</v>
@@ -1051,13 +1081,13 @@
         <v>19</v>
       </c>
       <c r="K11">
-        <v>-91</v>
+        <v>13.8</v>
       </c>
       <c r="L11">
-        <v>-3</v>
+        <v>-0.4</v>
       </c>
       <c r="M11">
-        <v>70</v>
+        <v>70.6</v>
       </c>
       <c r="N11" t="str">
         <v>BOX 140 - B_141</v>
@@ -1075,15 +1105,18 @@
         <v>TRUE</v>
       </c>
       <c r="S11" t="str">
-        <v/>
+        <v>parete attrezzata modulare</v>
       </c>
       <c r="T11" t="str">
-        <v/>
+        <v>Contemporaneo</v>
+      </c>
+      <c r="U11" t="str">
+        <v>Laccato Opaco</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>box-140-b-142-libreria-trenta</v>
+        <v>FEB-011</v>
       </c>
       <c r="B12" t="str">
         <v>Libreria Trenta</v>
@@ -1095,10 +1128,10 @@
         <v>Trenta è la libreria interpretata da Febal Casa come elemento chiave intorno cui viene progettata la zona giorno.</v>
       </c>
       <c r="E12" t="str">
-        <v/>
+        <v>antracite</v>
       </c>
       <c r="F12" t="str">
-        <v/>
+        <v>pannello laccato, vetro</v>
       </c>
       <c r="G12" t="str">
         <v>libreria, trenta, librerie, librería, librerías, estanteria, estantería, bookshelf, estante, interpretata, febal, casa, elemento, chiave, intorno, viene, progettata, zona, giorno</v>
@@ -1134,18 +1167,21 @@
         <v>librerie</v>
       </c>
       <c r="R12" t="str">
-        <v>TRUE</v>
+        <v>FALSE</v>
       </c>
       <c r="S12" t="str">
-        <v/>
+        <v>libreria modulare</v>
       </c>
       <c r="T12" t="str">
-        <v/>
+        <v>Contemporaneo</v>
+      </c>
+      <c r="U12" t="str">
+        <v>Laccato Opaco</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>box-140-b-143-libreria-trenta</v>
+        <v>FEB-012</v>
       </c>
       <c r="B13" t="str">
         <v>Libreria Trenta</v>
@@ -1157,10 +1193,10 @@
         <v>Trenta è la libreria interpretata da Febal Casa come elemento chiave intorno cui viene progettata la zona giorno.</v>
       </c>
       <c r="E13" t="str">
-        <v/>
+        <v>antracite</v>
       </c>
       <c r="F13" t="str">
-        <v/>
+        <v>pannello laccato, vetro</v>
       </c>
       <c r="G13" t="str">
         <v>libreria, trenta, librerie, librería, librerías, estanteria, estantería, bookshelf, estante, interpretata, febal, casa, elemento, chiave, intorno, viene, progettata, zona, giorno</v>
@@ -1172,16 +1208,16 @@
         <v>CASA 01 - AUTENTICA</v>
       </c>
       <c r="J13" t="str">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="K13">
-        <v>22</v>
+        <v>149.6</v>
       </c>
       <c r="L13">
-        <v>2</v>
+        <v>0.2</v>
       </c>
       <c r="M13">
-        <v>70</v>
+        <v>105.2</v>
       </c>
       <c r="N13" t="str">
         <v>BOX 140 - B_143</v>
@@ -1199,15 +1235,18 @@
         <v>TRUE</v>
       </c>
       <c r="S13" t="str">
-        <v/>
+        <v>libreria modulare</v>
       </c>
       <c r="T13" t="str">
-        <v/>
+        <v>Contemporaneo</v>
+      </c>
+      <c r="U13" t="str">
+        <v>Laccato Opaco</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>box-140-b-146-madie-aurora</v>
+        <v>FEB-013</v>
       </c>
       <c r="B14" t="str">
         <v>Madie Aurora</v>
@@ -1219,10 +1258,10 @@
         <v>La madia Aurora si distingue per la leggerezza dei volumi e l’estetica ricercata. Arreda la tua Casa con Febal Casa.</v>
       </c>
       <c r="E14" t="str">
-        <v/>
+        <v>noce, carbon grey</v>
       </c>
       <c r="F14" t="str">
-        <v/>
+        <v>legno, metallo, vetro</v>
       </c>
       <c r="G14" t="str">
         <v>madie, aurora, aparador, aparadores, madia, credenza, sideboard, buffet, casa, distingue, leggerezza, volumi, estetica, ricercata, arreda, febal</v>
@@ -1234,16 +1273,16 @@
         <v>CASA 01 - AUTENTICA</v>
       </c>
       <c r="J14" t="str">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="K14">
-        <v>-173</v>
+        <v>76.5</v>
       </c>
       <c r="L14">
-        <v>-31</v>
+        <v>-14.4</v>
       </c>
       <c r="M14">
-        <v>70</v>
+        <v>90</v>
       </c>
       <c r="N14" t="str">
         <v>BOX 140 - B_146</v>
@@ -1264,12 +1303,15 @@
         <v/>
       </c>
       <c r="T14" t="str">
+        <v>Contemporaneo</v>
+      </c>
+      <c r="U14" t="str">
         <v/>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>box-140-b-148-tavolino-rio</v>
+        <v>FEB-014</v>
       </c>
       <c r="B15" t="str">
         <v>Tavolino Rio</v>
@@ -1281,10 +1323,10 @@
         <v>Il tavolino Rio è contraddistinto da una struttura in metallo che presenta la particolarità di poter accogliere riviste e giornali. Una funzione che lo rende il compagno ideale nei momenti di relax. Il piano può essere configurato a seconda del proprio gusto in finitura laccata opaca o impiallacciata.</v>
       </c>
       <c r="E15" t="str">
-        <v/>
+        <v>marrone scuro/nero venato</v>
       </c>
       <c r="F15" t="str">
-        <v/>
+        <v>marmo</v>
       </c>
       <c r="G15" t="str">
         <v>tavolino, rio, tavolini, mesa de centro, mesita, coffee table, contraddistinto, struttura, metallo, presenta, particolarita, poter, accogliere, riviste, giornali, funzione, rende</v>
@@ -1320,18 +1362,21 @@
         <v>tavolini</v>
       </c>
       <c r="R15" t="str">
-        <v>TRUE</v>
+        <v>FALSE</v>
       </c>
       <c r="S15" t="str">
         <v/>
       </c>
       <c r="T15" t="str">
+        <v>Contemporaneo</v>
+      </c>
+      <c r="U15" t="str">
         <v/>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>box-160-b-161-armadio-profile-block</v>
+        <v>FEB-015</v>
       </c>
       <c r="B16" t="str">
         <v>Armadio Profile/ Block</v>
@@ -1343,10 +1388,10 @@
         <v>L'armadio con anta battente Profile Block si distingue per le sue linee nette e moderne, perfetta per un armadio dal carattere deciso.</v>
       </c>
       <c r="E16" t="str">
-        <v/>
+        <v>bronzo/champagne metallizzato</v>
       </c>
       <c r="F16" t="str">
-        <v/>
+        <v>pannello metallico</v>
       </c>
       <c r="G16" t="str">
         <v>armadio, profile/, block, armadi, armario, armarios, closet, ropero, wardrobe, cabina armadio, vestidor, anta, battente, profile, distingue, linee, nette, moderne, perfetta, carattere, deciso</v>
@@ -1361,13 +1406,13 @@
         <v>17</v>
       </c>
       <c r="K16">
-        <v>-171</v>
+        <v>-167.7</v>
       </c>
       <c r="L16">
-        <v>-4</v>
+        <v>-2.2</v>
       </c>
       <c r="M16">
-        <v>70</v>
+        <v>99.4</v>
       </c>
       <c r="N16" t="str">
         <v>BOX 160 - B_161</v>
@@ -1388,12 +1433,15 @@
         <v/>
       </c>
       <c r="T16" t="str">
-        <v/>
+        <v>Contemporaneo</v>
+      </c>
+      <c r="U16" t="str">
+        <v>Telaio Alluminio</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>box-160-b-162-libreria-lapis</v>
+        <v>FEB-016</v>
       </c>
       <c r="B17" t="str">
         <v>Libreria Lapis</v>
@@ -1405,10 +1453,10 @@
         <v>Il sistema libreria Lapis, configurabile a parete e centro stanza, si adatta perfettamente anche ad ambienti giorno e notte regalando estremo rigore e contenimento. Il suo design inedito è personalizzabile grazie a diversi elementi compositivi: ripiani in vetro, in metallo o in pannello, pensili e basi in differenti modularità per soddisfare qualsiasi esigenza.</v>
       </c>
       <c r="E17" t="str">
-        <v/>
+        <v>antracite, legno naturale</v>
       </c>
       <c r="F17" t="str">
-        <v/>
+        <v>metallo, legno</v>
       </c>
       <c r="G17" t="str">
         <v>libreria, lapis, librerie, librería, librerías, estanteria, estantería, bookshelf, estante, sistema, configurabile, parete, centro, stanza, adatta, perfettamente, ambienti, giorno, notte</v>
@@ -1423,13 +1471,13 @@
         <v>17</v>
       </c>
       <c r="K17">
-        <v>110</v>
+        <v>126.6</v>
       </c>
       <c r="L17">
-        <v>4</v>
+        <v>-2.6</v>
       </c>
       <c r="M17">
-        <v>70</v>
+        <v>86.5</v>
       </c>
       <c r="N17" t="str">
         <v>BOX 160 - B_162</v>
@@ -1447,15 +1495,18 @@
         <v>TRUE</v>
       </c>
       <c r="S17" t="str">
-        <v/>
+        <v>libreria a parete o centro stanza</v>
       </c>
       <c r="T17" t="str">
+        <v>Minimal</v>
+      </c>
+      <c r="U17" t="str">
         <v/>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>box-160-b-166-pouff-windsor</v>
+        <v>FEB-017</v>
       </c>
       <c r="B18" t="str">
         <v>Pouff Windsor</v>
@@ -1467,10 +1518,10 @@
         <v>Il pouf Windsor completa la gamma dei pouf della collezione divani Febal Casa. Grazie alle dimensioni e ai rivestimenti in cui è disponibile, è un elemento estremamente versatile che risponde a qualsiasi esigenza. La sua leggerezza permette di offrire soluzioni dinamiche per ogni stile di vita.</v>
       </c>
       <c r="E18" t="str">
-        <v/>
+        <v>verde oliva scuro</v>
       </c>
       <c r="F18" t="str">
-        <v/>
+        <v>tessuto</v>
       </c>
       <c r="G18" t="str">
         <v>pouff, windsor, pouf, puff, puffs, puf, ottoman, reposapies, completa, gamma, collezione, divani, febal, casa, grazie, dimensioni, rivestimenti, disponibile</v>
@@ -1485,13 +1536,13 @@
         <v>17</v>
       </c>
       <c r="K18">
-        <v>32</v>
+        <v>35.9</v>
       </c>
       <c r="L18">
-        <v>-40</v>
+        <v>-38.8</v>
       </c>
       <c r="M18">
-        <v>70</v>
+        <v>75.7</v>
       </c>
       <c r="N18" t="str">
         <v>BOX 160 - B_166</v>
@@ -1512,12 +1563,15 @@
         <v/>
       </c>
       <c r="T18" t="str">
+        <v>Contemporaneo</v>
+      </c>
+      <c r="U18" t="str">
         <v/>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>box-160-b-167-boiserie-tv</v>
+        <v>FEB-018</v>
       </c>
       <c r="B19" t="str">
         <v>Boiserie TV</v>
@@ -1547,13 +1601,13 @@
         <v>17</v>
       </c>
       <c r="K19">
-        <v>38</v>
+        <v>49.4</v>
       </c>
       <c r="L19">
-        <v>14</v>
+        <v>8.1</v>
       </c>
       <c r="M19">
-        <v>70</v>
+        <v>90.2</v>
       </c>
       <c r="N19" t="str">
         <v>BOX 160 - B_167</v>
@@ -1574,12 +1628,15 @@
         <v/>
       </c>
       <c r="T19" t="str">
+        <v>Contemporaneo</v>
+      </c>
+      <c r="U19" t="str">
         <v/>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>box-170-b-172-sistema-origina</v>
+        <v>FEB-019</v>
       </c>
       <c r="B20" t="str">
         <v>Sistema Origina</v>
@@ -1591,10 +1648,10 @@
         <v>L’anta a telaio è simbolo di un uno stile classico che può essere abbinato a aperture a gola, a maniglie e a pomoli.</v>
       </c>
       <c r="E20" t="str">
-        <v/>
+        <v>greige/tortora, marmo nero venato oro</v>
       </c>
       <c r="F20" t="str">
-        <v/>
+        <v>legno laccato, marmo</v>
       </c>
       <c r="G20" t="str">
         <v>sistema, origina, sistemi modulari, sistema modular, sistemas modulares, modular, anta, telaio, simbolo, stile, classico, abbinato, aperture, gola, maniglie, pomoli</v>
@@ -1630,18 +1687,21 @@
         <v>sistemi-modulari</v>
       </c>
       <c r="R20" t="str">
-        <v>TRUE</v>
+        <v>FALSE</v>
       </c>
       <c r="S20" t="str">
-        <v/>
+        <v>cucina componibile a isola</v>
       </c>
       <c r="T20" t="str">
-        <v/>
+        <v>Classico elegante</v>
+      </c>
+      <c r="U20" t="str">
+        <v>Laccato Opaco</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>box-170-b-173-sistema-origina</v>
+        <v>FEB-020</v>
       </c>
       <c r="B21" t="str">
         <v>Sistema Origina</v>
@@ -1653,10 +1713,10 @@
         <v>L’anta a telaio è simbolo di un uno stile classico che può essere abbinato a aperture a gola, a maniglie e a pomoli.</v>
       </c>
       <c r="E21" t="str">
-        <v/>
+        <v>greige/tortora, marmo nero venato oro</v>
       </c>
       <c r="F21" t="str">
-        <v/>
+        <v>legno laccato, marmo</v>
       </c>
       <c r="G21" t="str">
         <v>sistema, origina, sistemi modulari, sistema modular, sistemas modulares, modular, anta, telaio, simbolo, stile, classico, abbinato, aperture, gola, maniglie, pomoli</v>
@@ -1668,16 +1728,16 @@
         <v>CASA 01 - AUTENTICA</v>
       </c>
       <c r="J21" t="str">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="K21">
-        <v>-76</v>
+        <v>-175.9</v>
       </c>
       <c r="L21">
-        <v>1</v>
+        <v>-2.4</v>
       </c>
       <c r="M21">
-        <v>70</v>
+        <v>130</v>
       </c>
       <c r="N21" t="str">
         <v>BOX 170 - B_173</v>
@@ -1698,12 +1758,15 @@
         <v/>
       </c>
       <c r="T21" t="str">
-        <v/>
+        <v>Classico elegante</v>
+      </c>
+      <c r="U21" t="str">
+        <v>Laccato Opaco</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>box-170-b-174-sistema-origina</v>
+        <v>FEB-021</v>
       </c>
       <c r="B22" t="str">
         <v>Sistema Origina</v>
@@ -1715,10 +1778,10 @@
         <v>L’anta a telaio è simbolo di un uno stile classico che può essere abbinato a aperture a gola, a maniglie e a pomoli.</v>
       </c>
       <c r="E22" t="str">
-        <v/>
+        <v>greige/tortora, marmo nero venato oro</v>
       </c>
       <c r="F22" t="str">
-        <v/>
+        <v>legno laccato, marmo</v>
       </c>
       <c r="G22" t="str">
         <v>sistema, origina, sistemi modulari, sistema modular, sistemas modulares, modular, anta, telaio, simbolo, stile, classico, abbinato, aperture, gola, maniglie, pomoli</v>
@@ -1730,16 +1793,16 @@
         <v>CASA 01 - AUTENTICA</v>
       </c>
       <c r="J22" t="str">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="K22">
-        <v>126</v>
+        <v>-162.4</v>
       </c>
       <c r="L22">
-        <v>5</v>
+        <v>-3.9</v>
       </c>
       <c r="M22">
-        <v>70</v>
+        <v>117.3</v>
       </c>
       <c r="N22" t="str">
         <v>BOX 170 - B_174</v>
@@ -1760,12 +1823,15 @@
         <v/>
       </c>
       <c r="T22" t="str">
-        <v/>
+        <v>Classico elegante</v>
+      </c>
+      <c r="U22" t="str">
+        <v>Laccato Opaco</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>box-180-b-181-armadio-barret-con-portale</v>
+        <v>FEB-022</v>
       </c>
       <c r="B23" t="str">
         <v>Armadio Barret con Portale</v>
@@ -1777,10 +1843,10 @@
         <v>Scopri gli armadi a ponte con passaggio Febal Casa: soluzioni architettoniche che ottimizzano lo spazio con stile e funzionalità.</v>
       </c>
       <c r="E23" t="str">
-        <v/>
+        <v>wenge/marrone scurissimo</v>
       </c>
       <c r="F23" t="str">
-        <v/>
+        <v>pannello impiallacciato</v>
       </c>
       <c r="G23" t="str">
         <v>armadio, barret, portale, armadi, armario, armarios, closet, ropero, wardrobe, cabina armadio, vestidor, scopri, ponte, passaggio, febal, casa, soluzioni, architettoniche, ottimizzano, spazio, stile, funzionalita</v>
@@ -1816,18 +1882,21 @@
         <v>armadi</v>
       </c>
       <c r="R23" t="str">
-        <v>TRUE</v>
+        <v>FALSE</v>
       </c>
       <c r="S23" t="str">
-        <v/>
+        <v>armadio con passaggio a ponte</v>
       </c>
       <c r="T23" t="str">
+        <v>Contemporaneo</v>
+      </c>
+      <c r="U23" t="str">
         <v/>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>box-180-b-182-libreria-trenta</v>
+        <v>FEB-023</v>
       </c>
       <c r="B24" t="str">
         <v>Libreria Trenta</v>
@@ -1854,16 +1923,16 @@
         <v>CASA 01 - AUTENTICA</v>
       </c>
       <c r="J24" t="str">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="K24">
-        <v>75</v>
+        <v>-51.2</v>
       </c>
       <c r="L24">
-        <v>-6</v>
+        <v>-8.1</v>
       </c>
       <c r="M24">
-        <v>70</v>
+        <v>109.2</v>
       </c>
       <c r="N24" t="str">
         <v>BOX 180 - B_182</v>
@@ -1884,12 +1953,15 @@
         <v/>
       </c>
       <c r="T24" t="str">
+        <v>Contemporaneo</v>
+      </c>
+      <c r="U24" t="str">
         <v/>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>box-180-b-186-boiserie</v>
+        <v>FEB-024</v>
       </c>
       <c r="B25" t="str">
         <v>Boiserie</v>
@@ -1901,10 +1973,10 @@
         <v>La boiserie è concepita come un sistema in grado di dialogare con tutti gli altri arredi della gamma Febal Casa, un elemento versatile che si innesta con soluzione di continuità arrivando fino a terra.</v>
       </c>
       <c r="E25" t="str">
-        <v/>
+        <v>beige chiaro venato</v>
       </c>
       <c r="F25" t="str">
-        <v/>
+        <v>pannello effetto pietra</v>
       </c>
       <c r="G25" t="str">
         <v>boiserie, panel, paneles decorativos, revestimiento, pared, decorativo, columna, vertical, concepita, sistema, grado, dialogare, tutti, altri, arredi, gamma, febal, casa, elemento</v>
@@ -1916,16 +1988,16 @@
         <v>CASA 01 - AUTENTICA</v>
       </c>
       <c r="J25" t="str">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="K25">
-        <v>-163.96</v>
+        <v>-178.1</v>
       </c>
       <c r="L25">
-        <v>-0.17</v>
+        <v>-7.5</v>
       </c>
       <c r="M25">
-        <v>70</v>
+        <v>101.9</v>
       </c>
       <c r="N25" t="str">
         <v>BOX 180 - B_186</v>
@@ -1943,15 +2015,18 @@
         <v>TRUE</v>
       </c>
       <c r="S25" t="str">
-        <v/>
+        <v>boiserie modulare a tutta altezza</v>
       </c>
       <c r="T25" t="str">
-        <v/>
+        <v>Contemporaneo</v>
+      </c>
+      <c r="U25" t="str">
+        <v>Scenario</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>box-200-b-201-libreria-trenta-anta-libeskind022</v>
+        <v>FEB-025</v>
       </c>
       <c r="B26" t="str">
         <v>Libreria Trenta Anta Libeskind022</v>
@@ -1978,16 +2053,16 @@
         <v>CASA 02 - PERFETTA</v>
       </c>
       <c r="J26" t="str">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="K26">
-        <v>-117</v>
+        <v>147.5</v>
       </c>
       <c r="L26">
-        <v>2</v>
+        <v>-0.2</v>
       </c>
       <c r="M26">
-        <v>70</v>
+        <v>118.2</v>
       </c>
       <c r="N26" t="str">
         <v>BOX 200 - B_201</v>
@@ -2008,12 +2083,15 @@
         <v/>
       </c>
       <c r="T26" t="str">
+        <v>Contemporaneo</v>
+      </c>
+      <c r="U26" t="str">
         <v/>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>box-200-b-202-divano-camden</v>
+        <v>FEB-026</v>
       </c>
       <c r="B27" t="str">
         <v>Divano Camden</v>
@@ -2025,7 +2103,7 @@
         <v>Camden unisce eleganza e comfort in un design armonioso e avvolgente. Personalizzabile nei rivestimenti, si adatta a spazi classici e moderni, offrendo stile, calore e funzionalità a ogni ambiente living.</v>
       </c>
       <c r="E27" t="str">
-        <v/>
+        <v>verde</v>
       </c>
       <c r="F27" t="str">
         <v/>
@@ -2064,18 +2142,21 @@
         <v>divani</v>
       </c>
       <c r="R27" t="str">
-        <v>TRUE</v>
+        <v>FALSE</v>
       </c>
       <c r="S27" t="str">
-        <v/>
+        <v>modulare con isola</v>
       </c>
       <c r="T27" t="str">
-        <v/>
+        <v>Caldo accogliente, Classico elegante</v>
+      </c>
+      <c r="U27" t="str">
+        <v>Velvet</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>box-200-b-203-divano-camden</v>
+        <v>FEB-027</v>
       </c>
       <c r="B28" t="str">
         <v>Divano Camden</v>
@@ -2087,7 +2168,7 @@
         <v>Camden unisce eleganza e comfort in un design armonioso e avvolgente. Personalizzabile nei rivestimenti, si adatta a spazi classici e moderni, offrendo stile, calore e funzionalità a ogni ambiente living.</v>
       </c>
       <c r="E28" t="str">
-        <v/>
+        <v>cognac</v>
       </c>
       <c r="F28" t="str">
         <v/>
@@ -2102,16 +2183,16 @@
         <v>CASA 02 - PERFETTA</v>
       </c>
       <c r="J28" t="str">
-        <v>62</v>
+        <v>52</v>
       </c>
       <c r="K28">
-        <v>32</v>
+        <v>-128</v>
       </c>
       <c r="L28">
-        <v>-10</v>
+        <v>-41.6</v>
       </c>
       <c r="M28">
-        <v>70</v>
+        <v>87.8</v>
       </c>
       <c r="N28" t="str">
         <v>BOX 200 - B_203</v>
@@ -2129,15 +2210,18 @@
         <v>TRUE</v>
       </c>
       <c r="S28" t="str">
-        <v/>
+        <v>modulare curvo</v>
       </c>
       <c r="T28" t="str">
-        <v/>
+        <v>Caldo accogliente, Classico elegante</v>
+      </c>
+      <c r="U28" t="str">
+        <v>Boston</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>box-200-b-204-poltrone-astor</v>
+        <v>FEB-028</v>
       </c>
       <c r="B29" t="str">
         <v>Poltrone Astor</v>
@@ -2164,16 +2248,16 @@
         <v>CASA 02 - PERFETTA</v>
       </c>
       <c r="J29" t="str">
-        <v>62</v>
+        <v>52</v>
       </c>
       <c r="K29">
-        <v>-9</v>
+        <v>-34.5</v>
       </c>
       <c r="L29">
-        <v>-20</v>
+        <v>-26.4</v>
       </c>
       <c r="M29">
-        <v>70</v>
+        <v>67.9</v>
       </c>
       <c r="N29" t="str">
         <v>BOX 200 - B_204</v>
@@ -2194,12 +2278,15 @@
         <v/>
       </c>
       <c r="T29" t="str">
+        <v>Caldo accogliente, Contemporaneo</v>
+      </c>
+      <c r="U29" t="str">
         <v/>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>box-200-b-205-tavolini-ink</v>
+        <v>FEB-029</v>
       </c>
       <c r="B30" t="str">
         <v>Tavolini Ink</v>
@@ -2229,13 +2316,13 @@
         <v>52</v>
       </c>
       <c r="K30">
-        <v>-12</v>
+        <v>-12.8</v>
       </c>
       <c r="L30">
-        <v>-28</v>
+        <v>-28.5</v>
       </c>
       <c r="M30">
-        <v>70</v>
+        <v>49.8</v>
       </c>
       <c r="N30" t="str">
         <v>BOX 200 - B_205</v>
@@ -2256,12 +2343,15 @@
         <v/>
       </c>
       <c r="T30" t="str">
+        <v>Classico elegante</v>
+      </c>
+      <c r="U30" t="str">
         <v/>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>box-220-b-221-cucina-origina-anta-libeskind022</v>
+        <v>FEB-030</v>
       </c>
       <c r="B31" t="str">
         <v>Cucina Origina Anta Libeskind022</v>
@@ -2270,7 +2360,7 @@
         <v>cucine</v>
       </c>
       <c r="D31" t="str">
-        <v>Cucina Origina Anta Libeskind022 — pieza de la colección Febal Casa, sección CASA 02 - PERFETTA.</v>
+        <v>Cucina Origina Anta Libeskind022 — elemento della collezione Febal Casa, sezione CASA 02 - PERFETTA.</v>
       </c>
       <c r="E31" t="str">
         <v/>
@@ -2279,7 +2369,7 @@
         <v/>
       </c>
       <c r="G31" t="str">
-        <v>cucina, origina, anta, libeskind022, cucine, cocina, cocinas, kitchen, isla, casa, libeskind, pieza, coleccion, febal, seccion, perfetta</v>
+        <v>cucina, origina, anta, libeskind022, cucine, cocina, cocinas, kitchen, isla, casa, libeskind, elemento, collezione, febal, sezione, perfetta</v>
       </c>
       <c r="H31" t="str">
         <v/>
@@ -2291,13 +2381,13 @@
         <v>61</v>
       </c>
       <c r="K31">
-        <v>-140</v>
+        <v>-120.5</v>
       </c>
       <c r="L31">
-        <v>-30</v>
+        <v>-34.9</v>
       </c>
       <c r="M31">
-        <v>70</v>
+        <v>93.4</v>
       </c>
       <c r="N31" t="str">
         <v>BOX 220 - B_221</v>
@@ -2318,12 +2408,15 @@
         <v/>
       </c>
       <c r="T31" t="str">
+        <v>Contemporaneo</v>
+      </c>
+      <c r="U31" t="str">
         <v/>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>box-220-b-222-sistema-origina</v>
+        <v>FEB-031</v>
       </c>
       <c r="B32" t="str">
         <v>Sistema Origina</v>
@@ -2332,7 +2425,7 @@
         <v>sistemi modulari</v>
       </c>
       <c r="D32" t="str">
-        <v>Sistema Origina — pieza de la colección Febal Casa, sección CASA 02 - PERFETTA.</v>
+        <v>Sistema Origina — elemento della collezione Febal Casa, sezione CASA 02 - PERFETTA.</v>
       </c>
       <c r="E32" t="str">
         <v/>
@@ -2341,7 +2434,7 @@
         <v/>
       </c>
       <c r="G32" t="str">
-        <v>sistema, origina, sistemi modulari, sistema modular, sistemas modulares, modular, casa, pieza, coleccion, febal, seccion, perfetta</v>
+        <v>sistema, origina, sistemi modulari, sistema modular, sistemas modulares, modular, casa, elemento, collezione, febal, sezione, perfetta</v>
       </c>
       <c r="H32" t="str">
         <v/>
@@ -2353,13 +2446,13 @@
         <v>61</v>
       </c>
       <c r="K32">
-        <v>-143</v>
+        <v>-123.7</v>
       </c>
       <c r="L32">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="M32">
-        <v>70</v>
+        <v>69.4</v>
       </c>
       <c r="N32" t="str">
         <v>BOX 220 - B_222</v>
@@ -2380,12 +2473,15 @@
         <v/>
       </c>
       <c r="T32" t="str">
+        <v>Contemporaneo</v>
+      </c>
+      <c r="U32" t="str">
         <v/>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>box-220-b-223-pouff-windsor</v>
+        <v>FEB-032</v>
       </c>
       <c r="B33" t="str">
         <v>Pouff Windsor</v>
@@ -2415,13 +2511,13 @@
         <v>61</v>
       </c>
       <c r="K33">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="L33">
-        <v>-40</v>
+        <v>-35.4</v>
       </c>
       <c r="M33">
-        <v>70</v>
+        <v>84.9</v>
       </c>
       <c r="N33" t="str">
         <v>BOX 220 - B_223</v>
@@ -2442,12 +2538,15 @@
         <v/>
       </c>
       <c r="T33" t="str">
+        <v>Contemporaneo</v>
+      </c>
+      <c r="U33" t="str">
         <v/>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>box-240-b-241-libreria-trenta</v>
+        <v>FEB-033</v>
       </c>
       <c r="B34" t="str">
         <v>Libreria Trenta</v>
@@ -2474,16 +2573,16 @@
         <v>CASA 02 - PERFETTA</v>
       </c>
       <c r="J34" t="str">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="K34">
-        <v>47</v>
+        <v>50.8</v>
       </c>
       <c r="L34">
-        <v>2</v>
+        <v>-3.1</v>
       </c>
       <c r="M34">
-        <v>70</v>
+        <v>97.9</v>
       </c>
       <c r="N34" t="str">
         <v>BOX 240 - B_241</v>
@@ -2504,12 +2603,15 @@
         <v/>
       </c>
       <c r="T34" t="str">
+        <v>Contemporaneo</v>
+      </c>
+      <c r="U34" t="str">
         <v/>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>box-240-b-242-tavolo-phoenix</v>
+        <v>FEB-034</v>
       </c>
       <c r="B35" t="str">
         <v>Tavolo Phoenix</v>
@@ -2536,16 +2638,16 @@
         <v>CASA 02 - PERFETTA</v>
       </c>
       <c r="J35" t="str">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="K35">
-        <v>-18</v>
+        <v>-3.1</v>
       </c>
       <c r="L35">
-        <v>-38</v>
+        <v>-34.9</v>
       </c>
       <c r="M35">
-        <v>70</v>
+        <v>97.9</v>
       </c>
       <c r="N35" t="str">
         <v>BOX 240 - B_242</v>
@@ -2566,12 +2668,15 @@
         <v/>
       </c>
       <c r="T35" t="str">
+        <v>Contemporaneo</v>
+      </c>
+      <c r="U35" t="str">
         <v/>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>box-240-b-244-madia-libeskind022</v>
+        <v>FEB-035</v>
       </c>
       <c r="B36" t="str">
         <v>Madia Libeskind022</v>
@@ -2601,13 +2706,13 @@
         <v>55</v>
       </c>
       <c r="K36">
-        <v>158</v>
+        <v>170.7</v>
       </c>
       <c r="L36">
-        <v>-45</v>
+        <v>-31.6</v>
       </c>
       <c r="M36">
-        <v>70</v>
+        <v>98.8</v>
       </c>
       <c r="N36" t="str">
         <v>BOX 240 - B_244</v>
@@ -2628,12 +2733,15 @@
         <v/>
       </c>
       <c r="T36" t="str">
+        <v>Minimal, Contemporaneo</v>
+      </c>
+      <c r="U36" t="str">
         <v/>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>box-240-b-245-poltrona-vivienne</v>
+        <v>FEB-036</v>
       </c>
       <c r="B37" t="str">
         <v>Poltrona Vivienne</v>
@@ -2660,16 +2768,16 @@
         <v>CASA 02 - PERFETTA</v>
       </c>
       <c r="J37" t="str">
-        <v>56</v>
+        <v>49</v>
       </c>
       <c r="K37">
-        <v>101</v>
+        <v>-83.5</v>
       </c>
       <c r="L37">
-        <v>-12</v>
+        <v>-28.8</v>
       </c>
       <c r="M37">
-        <v>70</v>
+        <v>93.5</v>
       </c>
       <c r="N37" t="str">
         <v>BOX 240 - B_245</v>
@@ -2690,12 +2798,15 @@
         <v/>
       </c>
       <c r="T37" t="str">
+        <v>Classico elegante, Contemporaneo</v>
+      </c>
+      <c r="U37" t="str">
         <v/>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>box-260-b-261-armadio-collezione-momenti</v>
+        <v>FEB-037</v>
       </c>
       <c r="B38" t="str">
         <v>Armadio Collezione Momenti.</v>
@@ -2725,13 +2836,13 @@
         <v>66</v>
       </c>
       <c r="K38">
-        <v>-147</v>
+        <v>-112.5</v>
       </c>
       <c r="L38">
-        <v>-2</v>
+        <v>-6.8</v>
       </c>
       <c r="M38">
-        <v>70</v>
+        <v>123.6</v>
       </c>
       <c r="N38" t="str">
         <v>BOX 260 - B_261</v>
@@ -2752,12 +2863,15 @@
         <v/>
       </c>
       <c r="T38" t="str">
+        <v>Contemporaneo</v>
+      </c>
+      <c r="U38" t="str">
         <v/>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>box-260-b-264-boiserie</v>
+        <v>FEB-038</v>
       </c>
       <c r="B39" t="str">
         <v>Boiserie</v>
@@ -2787,13 +2901,13 @@
         <v>65</v>
       </c>
       <c r="K39">
-        <v>85</v>
+        <v>85.4</v>
       </c>
       <c r="L39">
-        <v>10</v>
+        <v>-1</v>
       </c>
       <c r="M39">
-        <v>70</v>
+        <v>109.7</v>
       </c>
       <c r="N39" t="str">
         <v>BOX 260 - B_264</v>
@@ -2814,12 +2928,15 @@
         <v/>
       </c>
       <c r="T39" t="str">
+        <v>Contemporaneo</v>
+      </c>
+      <c r="U39" t="str">
         <v/>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>box-280-b-281-letto-couple</v>
+        <v>FEB-039</v>
       </c>
       <c r="B40" t="str">
         <v>Letto Couple</v>
@@ -2828,7 +2945,7 @@
         <v>camera da letto</v>
       </c>
       <c r="D40" t="str">
-        <v>Letto Couple — pieza de la colección Febal Casa, sección CASA 02 - PERFETTA.</v>
+        <v>Letto Couple — elemento della collezione Febal Casa, sezione CASA 02 - PERFETTA.</v>
       </c>
       <c r="E40" t="str">
         <v/>
@@ -2837,7 +2954,7 @@
         <v/>
       </c>
       <c r="G40" t="str">
-        <v>letto, couple, camera da letto, cama, dormitorio, bed, recamara, recámara, habitacion, gruppo notte, casa, pieza, coleccion, febal, seccion, perfetta</v>
+        <v>letto, couple, camera da letto, cama, dormitorio, bed, recamara, recámara, habitacion, gruppo notte, casa, elemento, collezione, febal, sezione, perfetta</v>
       </c>
       <c r="H40" t="str">
         <v/>
@@ -2846,16 +2963,16 @@
         <v>CASA 02 - PERFETTA</v>
       </c>
       <c r="J40" t="str">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="K40">
-        <v>68</v>
+        <v>3.4</v>
       </c>
       <c r="L40">
-        <v>-29</v>
+        <v>-34</v>
       </c>
       <c r="M40">
-        <v>70</v>
+        <v>115.9</v>
       </c>
       <c r="N40" t="str">
         <v>BOX 280 - B_281</v>
@@ -2876,12 +2993,15 @@
         <v/>
       </c>
       <c r="T40" t="str">
+        <v>Contemporaneo</v>
+      </c>
+      <c r="U40" t="str">
         <v/>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>box-280-b-284-poltrona-isabelle</v>
+        <v>FEB-040</v>
       </c>
       <c r="B41" t="str">
         <v>Poltrona Isabelle</v>
@@ -2908,16 +3028,16 @@
         <v>CASA 02 - PERFETTA</v>
       </c>
       <c r="J41" t="str">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="K41">
-        <v>89</v>
+        <v>-81.5</v>
       </c>
       <c r="L41">
-        <v>-34</v>
+        <v>-40.1</v>
       </c>
       <c r="M41">
-        <v>70</v>
+        <v>89.3</v>
       </c>
       <c r="N41" t="str">
         <v>BOX 280 - B_284</v>
@@ -2938,12 +3058,15 @@
         <v/>
       </c>
       <c r="T41" t="str">
+        <v>Classico elegante, Contemporaneo</v>
+      </c>
+      <c r="U41" t="str">
         <v/>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>box-280-b-285-specchio-polar</v>
+        <v>FEB-041</v>
       </c>
       <c r="B42" t="str">
         <v>Specchio Polar</v>
@@ -2973,13 +3096,13 @@
         <v>58</v>
       </c>
       <c r="K42">
-        <v>123</v>
+        <v>136.7</v>
       </c>
       <c r="L42">
-        <v>-10</v>
+        <v>-6.8</v>
       </c>
       <c r="M42">
-        <v>70</v>
+        <v>96.4</v>
       </c>
       <c r="N42" t="str">
         <v>BOX 280 - B_285</v>
@@ -3000,12 +3123,15 @@
         <v/>
       </c>
       <c r="T42" t="str">
+        <v>Contemporaneo</v>
+      </c>
+      <c r="U42" t="str">
         <v/>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>box-290-b-291-boiserie</v>
+        <v>FEB-042</v>
       </c>
       <c r="B43" t="str">
         <v>Boiserie</v>
@@ -3032,16 +3158,16 @@
         <v>CASA 02 - PERFETTA</v>
       </c>
       <c r="J43" t="str">
-        <v>59a</v>
+        <v>59b</v>
       </c>
       <c r="K43">
-        <v>-100</v>
+        <v>-17.1</v>
       </c>
       <c r="L43">
-        <v>2</v>
+        <v>2.2</v>
       </c>
       <c r="M43">
-        <v>70</v>
+        <v>121.6</v>
       </c>
       <c r="N43" t="str">
         <v>BOX 290 - B_291</v>
@@ -3062,12 +3188,15 @@
         <v/>
       </c>
       <c r="T43" t="str">
+        <v>Contemporaneo</v>
+      </c>
+      <c r="U43" t="str">
         <v/>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>box-290-b-293-cabina-armadio-lapis</v>
+        <v>FEB-043</v>
       </c>
       <c r="B44" t="str">
         <v>Cabina Armadio Lapis</v>
@@ -3094,16 +3223,16 @@
         <v>CASA 02 - PERFETTA</v>
       </c>
       <c r="J44" t="str">
-        <v>59a</v>
+        <v>59b</v>
       </c>
       <c r="K44">
-        <v>-128</v>
+        <v>-14.1</v>
       </c>
       <c r="L44">
-        <v>-10</v>
+        <v>-14.6</v>
       </c>
       <c r="M44">
-        <v>70</v>
+        <v>121.6</v>
       </c>
       <c r="N44" t="str">
         <v>BOX 290 - B_293</v>
@@ -3124,12 +3253,15 @@
         <v/>
       </c>
       <c r="T44" t="str">
+        <v>Contemporaneo</v>
+      </c>
+      <c r="U44" t="str">
         <v/>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>box-290-b-294-boiserie</v>
+        <v>FEB-044</v>
       </c>
       <c r="B45" t="str">
         <v>Boiserie</v>
@@ -3180,18 +3312,21 @@
         <v>boiserie</v>
       </c>
       <c r="R45" t="str">
-        <v>TRUE</v>
+        <v>FALSE</v>
       </c>
       <c r="S45" t="str">
         <v/>
       </c>
       <c r="T45" t="str">
+        <v>Contemporaneo</v>
+      </c>
+      <c r="U45" t="str">
         <v/>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>box-290-b-295-armadio-lewitt-plus</v>
+        <v>FEB-045</v>
       </c>
       <c r="B46" t="str">
         <v>Armadio Lewitt Plus</v>
@@ -3221,13 +3356,13 @@
         <v>59a</v>
       </c>
       <c r="K46">
-        <v>136</v>
+        <v>133.2</v>
       </c>
       <c r="L46">
-        <v>-2</v>
+        <v>-5.3</v>
       </c>
       <c r="M46">
-        <v>70</v>
+        <v>121.6</v>
       </c>
       <c r="N46" t="str">
         <v>BOX 290 - B_295</v>
@@ -3248,12 +3383,15 @@
         <v/>
       </c>
       <c r="T46" t="str">
+        <v>Contemporaneo</v>
+      </c>
+      <c r="U46" t="str">
         <v/>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>box-300-b-301-sistema-diciotto</v>
+        <v>FEB-046</v>
       </c>
       <c r="B47" t="str">
         <v>Sistema Diciotto</v>
@@ -3280,16 +3418,16 @@
         <v>CASA 03 - AUDACE</v>
       </c>
       <c r="J47" t="str">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="K47">
-        <v>-120</v>
+        <v>-179.3</v>
       </c>
       <c r="L47">
-        <v>-1</v>
+        <v>-6.2</v>
       </c>
       <c r="M47">
-        <v>70</v>
+        <v>86.7</v>
       </c>
       <c r="N47" t="str">
         <v>BOX 300 - B_301</v>
@@ -3310,12 +3448,15 @@
         <v/>
       </c>
       <c r="T47" t="str">
+        <v>Contemporaneo</v>
+      </c>
+      <c r="U47" t="str">
         <v/>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>box-300-b-302-libreria-trenta</v>
+        <v>FEB-047</v>
       </c>
       <c r="B48" t="str">
         <v>Libreria Trenta</v>
@@ -3342,16 +3483,16 @@
         <v>CASA 03 - AUDACE</v>
       </c>
       <c r="J48" t="str">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="K48">
-        <v>160</v>
+        <v>10.2</v>
       </c>
       <c r="L48">
-        <v>13</v>
+        <v>2.8</v>
       </c>
       <c r="M48">
-        <v>70</v>
+        <v>98.3</v>
       </c>
       <c r="N48" t="str">
         <v>BOX 300 - B_302</v>
@@ -3372,12 +3513,15 @@
         <v/>
       </c>
       <c r="T48" t="str">
+        <v>Contemporaneo</v>
+      </c>
+      <c r="U48" t="str">
         <v/>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>box-300-b-303-divano-melrose</v>
+        <v>FEB-048</v>
       </c>
       <c r="B49" t="str">
         <v>Divano Melrose</v>
@@ -3404,16 +3548,16 @@
         <v>CASA 03 - AUDACE</v>
       </c>
       <c r="J49" t="str">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="K49">
-        <v>130</v>
+        <v>38.3</v>
       </c>
       <c r="L49">
-        <v>-15</v>
+        <v>-36.5</v>
       </c>
       <c r="M49">
-        <v>70</v>
+        <v>86.9</v>
       </c>
       <c r="N49" t="str">
         <v>BOX 300 - B_303</v>
@@ -3434,12 +3578,15 @@
         <v>ad angolo</v>
       </c>
       <c r="T49" t="str">
+        <v>Caldo accogliente, Contemporaneo</v>
+      </c>
+      <c r="U49" t="str">
         <v/>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>box-300-b-304-poltrona-andy</v>
+        <v>FEB-049</v>
       </c>
       <c r="B50" t="str">
         <v>Poltrona Andy</v>
@@ -3469,13 +3616,13 @@
         <v>42</v>
       </c>
       <c r="K50">
-        <v>-154</v>
+        <v>-172.5</v>
       </c>
       <c r="L50">
-        <v>-31</v>
+        <v>-44.8</v>
       </c>
       <c r="M50">
-        <v>70</v>
+        <v>86.1</v>
       </c>
       <c r="N50" t="str">
         <v>BOX 300 - B_304</v>
@@ -3496,12 +3643,15 @@
         <v/>
       </c>
       <c r="T50" t="str">
+        <v>Contemporaneo, Caldo accogliente</v>
+      </c>
+      <c r="U50" t="str">
         <v/>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>box-300-b-308-gruppo-notte-marlene</v>
+        <v>FEB-050</v>
       </c>
       <c r="B51" t="str">
         <v>Gruppo Notte Marlene</v>
@@ -3528,16 +3678,16 @@
         <v>CASA 03 - AUDACE</v>
       </c>
       <c r="J51" t="str">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="K51">
-        <v>-55</v>
+        <v>-69.7</v>
       </c>
       <c r="L51">
-        <v>-30</v>
+        <v>-22.3</v>
       </c>
       <c r="M51">
-        <v>70</v>
+        <v>78.2</v>
       </c>
       <c r="N51" t="str">
         <v>BOX 300 - B_308</v>
@@ -3558,12 +3708,15 @@
         <v/>
       </c>
       <c r="T51" t="str">
+        <v>Contemporaneo</v>
+      </c>
+      <c r="U51" t="str">
         <v/>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>box-320-b-321-cucina-modula-anta-square</v>
+        <v>FEB-051</v>
       </c>
       <c r="B52" t="str">
         <v>Cucina Modula anta Square</v>
@@ -3572,7 +3725,7 @@
         <v>cucine</v>
       </c>
       <c r="D52" t="str">
-        <v>Cucina Modula anta Square — pieza de la colección Febal Casa, sección CASA 03 - AUDACE.</v>
+        <v>Cucina Modula anta Square — elemento della collezione Febal Casa, sezione CASA 03 - AUDACE.</v>
       </c>
       <c r="E52" t="str">
         <v/>
@@ -3581,7 +3734,7 @@
         <v/>
       </c>
       <c r="G52" t="str">
-        <v>cucina, modula, anta, square, cucine, cocina, cocinas, kitchen, isla, casa, pieza, coleccion, febal, seccion, audace</v>
+        <v>cucina, modula, anta, square, cucine, cocina, cocinas, kitchen, isla, casa, elemento, collezione, febal, sezione, audace</v>
       </c>
       <c r="H52" t="str">
         <v/>
@@ -3590,16 +3743,16 @@
         <v>CASA 03 - AUDACE</v>
       </c>
       <c r="J52" t="str">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="K52">
-        <v>52</v>
+        <v>98.9</v>
       </c>
       <c r="L52">
-        <v>3</v>
+        <v>-8.3</v>
       </c>
       <c r="M52">
-        <v>70</v>
+        <v>114.7</v>
       </c>
       <c r="N52" t="str">
         <v>BOX 320 - B_321</v>
@@ -3620,12 +3773,15 @@
         <v/>
       </c>
       <c r="T52" t="str">
+        <v>Contemporaneo</v>
+      </c>
+      <c r="U52" t="str">
         <v/>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>box-320-b-322-tavolo-madeira</v>
+        <v>FEB-052</v>
       </c>
       <c r="B53" t="str">
         <v>Tavolo Madeira</v>
@@ -3634,16 +3790,16 @@
         <v>tavoli</v>
       </c>
       <c r="D53" t="str">
-        <v>Tavolo Madeira — pieza de la colección Febal Casa, sección CASA 03 - AUDACE.</v>
+        <v>L'armonioso intreccio di archi definisce un tavolo unico, protagonista di ogni ambiente. Le gambe inclinate e sovrapposte formano un disegno geometrico di grande impatto visivo che gioca con la tridimensionalità ottenendo un risultato perfetto nato dall'eleganza, dall'equilibrio e dalla leggerezza dei volumi. La base in metallo è disponibile in finitura Ottone Scuro, Nero, Antracite e Sabbia. Il piano è di forma rotonda, ovale fisso o allungabile ed è configurabile in Cristallo Lucido, Cristallo Velvet, Superceramica, Supermarmo opaco, Supermarmo lucido e legno Impiallacciato. La versione fissa può essere arricchita con il piano centrotavola girevole, un dispositivo rotante che permette di condividere facilmente cibi e oggetti con tutti i commensali.</v>
       </c>
       <c r="E53" t="str">
-        <v/>
+        <v>antracite</v>
       </c>
       <c r="F53" t="str">
-        <v/>
+        <v>supermarmo lucido, metallo</v>
       </c>
       <c r="G53" t="str">
-        <v>tavolo, madeira, tavoli, mesa, mesas, table, comedor, casa, pieza, coleccion, febal, seccion, audace</v>
+        <v>tavolo, madeira, tavoli, mesa, mesas, table, comedor, dall, piano, cristallo, lucido, supermarmo, armonioso, intreccio, archi, definisce, unico, protagonista</v>
       </c>
       <c r="H53" t="str">
         <v/>
@@ -3655,22 +3811,22 @@
         <v>97</v>
       </c>
       <c r="K53">
-        <v>100</v>
+        <v>89.6</v>
       </c>
       <c r="L53">
-        <v>-41</v>
+        <v>-38.4</v>
       </c>
       <c r="M53">
-        <v>70</v>
+        <v>75.3</v>
       </c>
       <c r="N53" t="str">
         <v>BOX 320 - B_322</v>
       </c>
       <c r="O53" t="str">
-        <v>assets/febal-casa/placeholder-product.png</v>
+        <v>assets/febal-casa/products/madeira.jpg</v>
       </c>
       <c r="P53" t="str">
-        <v xml:space="preserve">https://www.febalcasa.com/it/prodotti/madeira/ </v>
+        <v>https://www.febalcasa.com/it/prodotti/madeira/</v>
       </c>
       <c r="Q53" t="str">
         <v>tavoli</v>
@@ -3679,15 +3835,18 @@
         <v>TRUE</v>
       </c>
       <c r="S53" t="str">
-        <v/>
+        <v>rotondo o ovale, fisso o allungabile</v>
       </c>
       <c r="T53" t="str">
+        <v>Contemporaneo</v>
+      </c>
+      <c r="U53" t="str">
         <v/>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>box-320-b-323-sedia-nina</v>
+        <v>FEB-053</v>
       </c>
       <c r="B54" t="str">
         <v>Sedia Nina</v>
@@ -3717,13 +3876,13 @@
         <v>97</v>
       </c>
       <c r="K54">
-        <v>40</v>
+        <v>34.6</v>
       </c>
       <c r="L54">
-        <v>-40</v>
+        <v>-42.6</v>
       </c>
       <c r="M54">
-        <v>70</v>
+        <v>75.3</v>
       </c>
       <c r="N54" t="str">
         <v>BOX 320 - B_323</v>
@@ -3744,12 +3903,15 @@
         <v/>
       </c>
       <c r="T54" t="str">
+        <v>Caldo accogliente</v>
+      </c>
+      <c r="U54" t="str">
         <v/>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>box-320-b-324-madia-leaf</v>
+        <v>FEB-054</v>
       </c>
       <c r="B55" t="str">
         <v>Madia Leaf</v>
@@ -3776,16 +3938,16 @@
         <v>CASA 03 - AUDACE</v>
       </c>
       <c r="J55" t="str">
-        <v>97</v>
+        <v>40</v>
       </c>
       <c r="K55">
-        <v>-17.02</v>
+        <v>-109.2</v>
       </c>
       <c r="L55">
-        <v>-8.24</v>
+        <v>-41</v>
       </c>
       <c r="M55">
-        <v>70</v>
+        <v>98.4</v>
       </c>
       <c r="N55" t="str">
         <v>BOX 320 - B_324</v>
@@ -3806,12 +3968,15 @@
         <v/>
       </c>
       <c r="T55" t="str">
+        <v>Classico elegante</v>
+      </c>
+      <c r="U55" t="str">
         <v/>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>box-340-b-342-libreria-trenta</v>
+        <v>FEB-055</v>
       </c>
       <c r="B56" t="str">
         <v>Libreria Trenta</v>
@@ -3841,13 +4006,13 @@
         <v>47</v>
       </c>
       <c r="K56">
-        <v>-23</v>
+        <v>-36.4</v>
       </c>
       <c r="L56">
-        <v>-17</v>
+        <v>-5.4</v>
       </c>
       <c r="M56">
-        <v>70</v>
+        <v>110.2</v>
       </c>
       <c r="N56" t="str">
         <v>BOX 340 - B_342</v>
@@ -3868,12 +4033,15 @@
         <v/>
       </c>
       <c r="T56" t="str">
+        <v>Contemporaneo</v>
+      </c>
+      <c r="U56" t="str">
         <v/>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>box-340-b-344-gruppo-notte-marlene</v>
+        <v>FEB-056</v>
       </c>
       <c r="B57" t="str">
         <v>Gruppo Notte Marlene</v>
@@ -3900,16 +4068,16 @@
         <v>CASA 03 - AUDACE</v>
       </c>
       <c r="J57" t="str">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="K57">
-        <v>127</v>
+        <v>115.5</v>
       </c>
       <c r="L57">
-        <v>-37</v>
+        <v>-29.6</v>
       </c>
       <c r="M57">
-        <v>70</v>
+        <v>54.4</v>
       </c>
       <c r="N57" t="str">
         <v>BOX 340 - B_344</v>
@@ -3930,12 +4098,15 @@
         <v/>
       </c>
       <c r="T57" t="str">
+        <v>Contemporaneo, Classico elegante</v>
+      </c>
+      <c r="U57" t="str">
         <v/>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>box-340-b-345-boiserie</v>
+        <v>FEB-057</v>
       </c>
       <c r="B58" t="str">
         <v>Boiserie</v>
@@ -3962,16 +4133,16 @@
         <v>CASA 03 - AUDACE</v>
       </c>
       <c r="J58" t="str">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="K58">
-        <v>139</v>
+        <v>110.6</v>
       </c>
       <c r="L58">
-        <v>-21</v>
+        <v>-15.3</v>
       </c>
       <c r="M58">
-        <v>70</v>
+        <v>69.6</v>
       </c>
       <c r="N58" t="str">
         <v>BOX 340 - B_345</v>
@@ -3992,12 +4163,15 @@
         <v/>
       </c>
       <c r="T58" t="str">
+        <v>Contemporaneo</v>
+      </c>
+      <c r="U58" t="str">
         <v/>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>box-360-b-361-armadio-collezione-momenti</v>
+        <v>FEB-058</v>
       </c>
       <c r="B59" t="str">
         <v>Armadio Collezione Momenti.</v>
@@ -4006,7 +4180,7 @@
         <v>armadi</v>
       </c>
       <c r="D59" t="str">
-        <v>Armadio Collezione Momenti. — pieza de la colección Febal Casa, sección CASA 03 - AUDACE.</v>
+        <v>Armadio Collezione Momenti. — elemento della collezione Febal Casa, sezione CASA 03 - AUDACE.</v>
       </c>
       <c r="E59" t="str">
         <v/>
@@ -4015,7 +4189,7 @@
         <v/>
       </c>
       <c r="G59" t="str">
-        <v>armadio, collezione, momenti., armadi, armario, armarios, closet, ropero, wardrobe, cabina armadio, vestidor, casa, momenti, pieza, coleccion, febal, seccion, audace</v>
+        <v>armadio, collezione, momenti., armadi, armario, armarios, closet, ropero, wardrobe, cabina armadio, vestidor, casa, momenti, elemento, febal, sezione, audace</v>
       </c>
       <c r="H59" t="str">
         <v/>
@@ -4027,13 +4201,13 @@
         <v>92</v>
       </c>
       <c r="K59">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="L59">
-        <v>2</v>
+        <v>-2.2</v>
       </c>
       <c r="M59">
-        <v>70</v>
+        <v>74.5</v>
       </c>
       <c r="N59" t="str">
         <v>BOX 360 - B_361</v>
@@ -4054,12 +4228,15 @@
         <v/>
       </c>
       <c r="T59" t="str">
+        <v>Contemporaneo</v>
+      </c>
+      <c r="U59" t="str">
         <v/>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>box-360-b-362-letto-collezione-momenti</v>
+        <v>FEB-059</v>
       </c>
       <c r="B60" t="str">
         <v>Letto Collezione Momenti.</v>
@@ -4068,7 +4245,7 @@
         <v>camera da letto</v>
       </c>
       <c r="D60" t="str">
-        <v>Letto Collezione Momenti. — pieza de la colección Febal Casa, sección CASA 03 - AUDACE.</v>
+        <v>Letto Collezione Momenti. — elemento della collezione Febal Casa, sezione CASA 03 - AUDACE.</v>
       </c>
       <c r="E60" t="str">
         <v/>
@@ -4077,7 +4254,7 @@
         <v/>
       </c>
       <c r="G60" t="str">
-        <v>letto, collezione, momenti., camera da letto, cama, dormitorio, bed, recamara, recámara, habitacion, gruppo notte, casa, momenti, pieza, coleccion, febal, seccion, audace</v>
+        <v>letto, collezione, momenti., camera da letto, cama, dormitorio, bed, recamara, recámara, habitacion, gruppo notte, casa, momenti, elemento, febal, sezione, audace</v>
       </c>
       <c r="H60" t="str">
         <v/>
@@ -4089,13 +4266,13 @@
         <v>92</v>
       </c>
       <c r="K60">
-        <v>165</v>
+        <v>173.8</v>
       </c>
       <c r="L60">
-        <v>-28</v>
+        <v>-22.7</v>
       </c>
       <c r="M60">
-        <v>70</v>
+        <v>91.7</v>
       </c>
       <c r="N60" t="str">
         <v>BOX 360 - B_362</v>
@@ -4116,12 +4293,15 @@
         <v/>
       </c>
       <c r="T60" t="str">
+        <v>Contemporaneo</v>
+      </c>
+      <c r="U60" t="str">
         <v/>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>box-360-b-363-libreria-collezione-momenti</v>
+        <v>FEB-060</v>
       </c>
       <c r="B61" t="str">
         <v>Libreria Collezione Momenti.</v>
@@ -4130,7 +4310,7 @@
         <v>librerie</v>
       </c>
       <c r="D61" t="str">
-        <v>Libreria Collezione Momenti. — pieza de la colección Febal Casa, sección CASA 03 - AUDACE.</v>
+        <v>Libreria Collezione Momenti. — elemento della collezione Febal Casa, sezione CASA 03 - AUDACE.</v>
       </c>
       <c r="E61" t="str">
         <v/>
@@ -4139,7 +4319,7 @@
         <v/>
       </c>
       <c r="G61" t="str">
-        <v>libreria, collezione, momenti., librerie, librería, librerías, estanteria, estantería, bookshelf, estante, casa, momenti, pieza, coleccion, febal, seccion, audace</v>
+        <v>libreria, collezione, momenti., librerie, librería, librerías, estanteria, estantería, bookshelf, estante, casa, momenti, elemento, febal, sezione, audace</v>
       </c>
       <c r="H61" t="str">
         <v/>
@@ -4151,13 +4331,13 @@
         <v>92</v>
       </c>
       <c r="K61">
-        <v>35</v>
+        <v>7.4</v>
       </c>
       <c r="L61">
-        <v>10</v>
+        <v>-3.8</v>
       </c>
       <c r="M61">
-        <v>70</v>
+        <v>130</v>
       </c>
       <c r="N61" t="str">
         <v>BOX 360 - B_363</v>
@@ -4178,12 +4358,15 @@
         <v/>
       </c>
       <c r="T61" t="str">
+        <v>Contemporaneo</v>
+      </c>
+      <c r="U61" t="str">
         <v/>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>box-360-b-364-pouff-windsor</v>
+        <v>FEB-061</v>
       </c>
       <c r="B62" t="str">
         <v>Pouff Windsor</v>
@@ -4213,13 +4396,13 @@
         <v>92</v>
       </c>
       <c r="K62">
-        <v>132</v>
+        <v>127.6</v>
       </c>
       <c r="L62">
-        <v>-22</v>
+        <v>-23.3</v>
       </c>
       <c r="M62">
-        <v>70</v>
+        <v>53.8</v>
       </c>
       <c r="N62" t="str">
         <v>BOX 360 - B_364</v>
@@ -4240,21 +4423,24 @@
         <v/>
       </c>
       <c r="T62" t="str">
+        <v>Contemporaneo</v>
+      </c>
+      <c r="U62" t="str">
         <v/>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>box-360-b-365-armadio-collezione-momenti</v>
+        <v>FEB-062</v>
       </c>
       <c r="B63" t="str">
-        <v>Armadio  Collezione Momenti.</v>
+        <v>Armadio Collezione Momenti.</v>
       </c>
       <c r="C63" t="str">
         <v>armadi</v>
       </c>
       <c r="D63" t="str">
-        <v>Armadio  Collezione Momenti. — pieza de la colección Febal Casa, sección CASA 03 - AUDACE.</v>
+        <v>Armadio Collezione Momenti. — elemento della collezione Febal Casa, sezione CASA 03 - AUDACE.</v>
       </c>
       <c r="E63" t="str">
         <v/>
@@ -4263,7 +4449,7 @@
         <v/>
       </c>
       <c r="G63" t="str">
-        <v>armadio, collezione, momenti., armadi, armario, armarios, closet, ropero, wardrobe, cabina armadio, vestidor, casa, momenti, pieza, coleccion, febal, seccion, audace</v>
+        <v>armadio, collezione, momenti., armadi, armario, armarios, closet, ropero, wardrobe, cabina armadio, vestidor, casa, momenti, elemento, febal, sezione, audace</v>
       </c>
       <c r="H63" t="str">
         <v/>
@@ -4296,18 +4482,21 @@
         <v>armadi</v>
       </c>
       <c r="R63" t="str">
-        <v>TRUE</v>
+        <v>FALSE</v>
       </c>
       <c r="S63" t="str">
         <v/>
       </c>
       <c r="T63" t="str">
+        <v>Contemporaneo</v>
+      </c>
+      <c r="U63" t="str">
         <v/>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>box-400-b-401-boiserie</v>
+        <v>FEB-063</v>
       </c>
       <c r="B64" t="str">
         <v>Boiserie</v>
@@ -4337,13 +4526,13 @@
         <v>76</v>
       </c>
       <c r="K64">
-        <v>22</v>
+        <v>23.5</v>
       </c>
       <c r="L64">
-        <v>18</v>
+        <v>17.2</v>
       </c>
       <c r="M64">
-        <v>70</v>
+        <v>80.4</v>
       </c>
       <c r="N64" t="str">
         <v>BOX 400 - B_401</v>
@@ -4364,12 +4553,15 @@
         <v/>
       </c>
       <c r="T64" t="str">
+        <v>Contemporaneo</v>
+      </c>
+      <c r="U64" t="str">
         <v/>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>box-400-b-401-libreria-trenta</v>
+        <v>FEB-064</v>
       </c>
       <c r="B65" t="str">
         <v>Libreria Trenta</v>
@@ -4396,16 +4588,16 @@
         <v>CASA 04 - A-MARE</v>
       </c>
       <c r="J65" t="str">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="K65">
-        <v>-58</v>
+        <v>43.8</v>
       </c>
       <c r="L65">
-        <v>6</v>
+        <v>-2.9</v>
       </c>
       <c r="M65">
-        <v>70</v>
+        <v>102.7</v>
       </c>
       <c r="N65" t="str">
         <v>BOX 400 - B_401</v>
@@ -4426,12 +4618,15 @@
         <v/>
       </c>
       <c r="T65" t="str">
+        <v>Contemporaneo</v>
+      </c>
+      <c r="U65" t="str">
         <v/>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>box-400-b-402-madia-onda-zaha-hadid-architects</v>
+        <v>FEB-065</v>
       </c>
       <c r="B66" t="str">
         <v>Madia Onda - Zaha Hadid Architects</v>
@@ -4440,7 +4635,7 @@
         <v>madie</v>
       </c>
       <c r="D66" t="str">
-        <v>Madia Onda - Zaha Hadid Architects — pieza de la colección Febal Casa, sección CASA 04 - A-MARE.</v>
+        <v>Madia Onda - Zaha Hadid Architects — elemento della collezione Febal Casa, sezione CASA 04 - A-MARE.</v>
       </c>
       <c r="E66" t="str">
         <v/>
@@ -4449,7 +4644,7 @@
         <v/>
       </c>
       <c r="G66" t="str">
-        <v>madia, onda, zaha, hadid, architects, madie, aparador, aparadores, credenza, sideboard, buffet, casa, pieza, coleccion, febal, seccion, mare</v>
+        <v>madia, onda, zaha, hadid, architects, madie, aparador, aparadores, credenza, sideboard, buffet, casa, elemento, collezione, febal, sezione, mare</v>
       </c>
       <c r="H66" t="str">
         <v/>
@@ -4458,16 +4653,16 @@
         <v>CASA 04 - A-MARE</v>
       </c>
       <c r="J66" t="str">
-        <v>72</v>
+        <v>74a</v>
       </c>
       <c r="K66">
-        <v>-115</v>
+        <v>50.9</v>
       </c>
       <c r="L66">
-        <v>-23</v>
+        <v>-11</v>
       </c>
       <c r="M66">
-        <v>70</v>
+        <v>47.4</v>
       </c>
       <c r="N66" t="str">
         <v>BOX 400 - B_402</v>
@@ -4488,12 +4683,15 @@
         <v/>
       </c>
       <c r="T66" t="str">
+        <v>Contemporaneo</v>
+      </c>
+      <c r="U66" t="str">
         <v/>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>box-400-b-403-divano-navigli</v>
+        <v>FEB-066</v>
       </c>
       <c r="B67" t="str">
         <v>Divano Navigli</v>
@@ -4520,16 +4718,16 @@
         <v>CASA 04 - A-MARE</v>
       </c>
       <c r="J67" t="str">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="K67">
-        <v>-105</v>
+        <v>-75.9</v>
       </c>
       <c r="L67">
-        <v>-30</v>
+        <v>-38.7</v>
       </c>
       <c r="M67">
-        <v>70</v>
+        <v>95.4</v>
       </c>
       <c r="N67" t="str">
         <v>BOX 400 - B_403</v>
@@ -4550,12 +4748,15 @@
         <v/>
       </c>
       <c r="T67" t="str">
+        <v>Contemporaneo</v>
+      </c>
+      <c r="U67" t="str">
         <v/>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>box-420-b-421-libreria-lapis</v>
+        <v>FEB-067</v>
       </c>
       <c r="B68" t="str">
         <v>Libreria Lapis</v>
@@ -4582,16 +4783,16 @@
         <v>CASA 04 - A-MARE</v>
       </c>
       <c r="J68" t="str">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="K68">
-        <v>50</v>
+        <v>-18.4</v>
       </c>
       <c r="L68">
-        <v>5</v>
+        <v>-6.3</v>
       </c>
       <c r="M68">
-        <v>70</v>
+        <v>99.6</v>
       </c>
       <c r="N68" t="str">
         <v>BOX 420 - B_421</v>
@@ -4612,12 +4813,15 @@
         <v/>
       </c>
       <c r="T68" t="str">
+        <v>Minimal</v>
+      </c>
+      <c r="U68" t="str">
         <v/>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>box-420-b-422-sistema-origina</v>
+        <v>FEB-068</v>
       </c>
       <c r="B69" t="str">
         <v>Sistema Origina</v>
@@ -4644,16 +4848,16 @@
         <v>CASA 04 - A-MARE</v>
       </c>
       <c r="J69" t="str">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="K69">
-        <v>112</v>
+        <v>-112</v>
       </c>
       <c r="L69">
-        <v>-2</v>
+        <v>-8.3</v>
       </c>
       <c r="M69">
-        <v>70</v>
+        <v>88</v>
       </c>
       <c r="N69" t="str">
         <v>BOX 420 - B_422</v>
@@ -4674,12 +4878,15 @@
         <v/>
       </c>
       <c r="T69" t="str">
+        <v>Contemporaneo</v>
+      </c>
+      <c r="U69" t="str">
         <v/>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>box-420-b-423-cucina-origina-anta-sagoma-37</v>
+        <v>FEB-069</v>
       </c>
       <c r="B70" t="str">
         <v>Cucina Origina Anta Sagoma 37</v>
@@ -4706,16 +4913,16 @@
         <v>CASA 04 - A-MARE</v>
       </c>
       <c r="J70" t="str">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="K70">
-        <v>115</v>
+        <v>-118.3</v>
       </c>
       <c r="L70">
-        <v>-22</v>
+        <v>-34.9</v>
       </c>
       <c r="M70">
-        <v>70</v>
+        <v>90.6</v>
       </c>
       <c r="N70" t="str">
         <v>BOX 420 - B_423</v>
@@ -4736,12 +4943,15 @@
         <v/>
       </c>
       <c r="T70" t="str">
+        <v>Contemporaneo</v>
+      </c>
+      <c r="U70" t="str">
         <v/>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>box-420-b-424-cucina-origina-anta-sagoma-37</v>
+        <v>FEB-070</v>
       </c>
       <c r="B71" t="str">
         <v>Cucina Origina Anta Sagoma 37</v>
@@ -4792,18 +5002,21 @@
         <v>cucine</v>
       </c>
       <c r="R71" t="str">
-        <v>TRUE</v>
+        <v>FALSE</v>
       </c>
       <c r="S71" t="str">
         <v/>
       </c>
       <c r="T71" t="str">
+        <v>Contemporaneo</v>
+      </c>
+      <c r="U71" t="str">
         <v/>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>box-440-b-441-boiserie</v>
+        <v>FEB-071</v>
       </c>
       <c r="B72" t="str">
         <v>Boiserie</v>
@@ -4854,18 +5067,21 @@
         <v>boiserie</v>
       </c>
       <c r="R72" t="str">
-        <v>TRUE</v>
+        <v>FALSE</v>
       </c>
       <c r="S72" t="str">
         <v/>
       </c>
       <c r="T72" t="str">
+        <v>Contemporaneo</v>
+      </c>
+      <c r="U72" t="str">
         <v/>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>box-440-b-442-tavolo-leeds</v>
+        <v>FEB-072</v>
       </c>
       <c r="B73" t="str">
         <v>Tavolo Leeds</v>
@@ -4892,16 +5108,16 @@
         <v>CASA 04 - A-MARE</v>
       </c>
       <c r="J73" t="str">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="K73">
-        <v>146</v>
+        <v>-87.6</v>
       </c>
       <c r="L73">
-        <v>-12</v>
+        <v>-26.2</v>
       </c>
       <c r="M73">
-        <v>70</v>
+        <v>74.5</v>
       </c>
       <c r="N73" t="str">
         <v>BOX 440 - B_442</v>
@@ -4922,12 +5138,15 @@
         <v/>
       </c>
       <c r="T73" t="str">
+        <v>Contemporaneo</v>
+      </c>
+      <c r="U73" t="str">
         <v/>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>box-440-b-443-sedia-nives-con-braccioli</v>
+        <v>FEB-073</v>
       </c>
       <c r="B74" t="str">
         <v>Sedia Nives con braccioli</v>
@@ -4954,16 +5173,16 @@
         <v>CASA 04 - A-MARE</v>
       </c>
       <c r="J74" t="str">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="K74">
-        <v>138</v>
+        <v>-50.9</v>
       </c>
       <c r="L74">
-        <v>-19</v>
+        <v>-28.6</v>
       </c>
       <c r="M74">
-        <v>70</v>
+        <v>64.1</v>
       </c>
       <c r="N74" t="str">
         <v>BOX 440 - B_443</v>
@@ -4984,12 +5203,15 @@
         <v/>
       </c>
       <c r="T74" t="str">
+        <v>Classico elegante, Caldo accogliente</v>
+      </c>
+      <c r="U74" t="str">
         <v/>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>box-460-b-461-armadio-scorrevole-rodin</v>
+        <v>FEB-074</v>
       </c>
       <c r="B75" t="str">
         <v>Armadio Scorrevole Rodin</v>
@@ -5016,16 +5238,16 @@
         <v>CASA 04 - A-MARE</v>
       </c>
       <c r="J75" t="str">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="K75">
-        <v>-130</v>
+        <v>-8.6</v>
       </c>
       <c r="L75">
-        <v>2</v>
+        <v>-2.9</v>
       </c>
       <c r="M75">
-        <v>70</v>
+        <v>123.1</v>
       </c>
       <c r="N75" t="str">
         <v>BOX 460 - B_461</v>
@@ -5046,12 +5268,15 @@
         <v/>
       </c>
       <c r="T75" t="str">
+        <v>Contemporaneo</v>
+      </c>
+      <c r="U75" t="str">
         <v/>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>box-460-b-465-cabina-armadio-hype</v>
+        <v>FEB-075</v>
       </c>
       <c r="B76" t="str">
         <v>Cabina Armadio Hype</v>
@@ -5081,13 +5306,13 @@
         <v>74</v>
       </c>
       <c r="K76">
-        <v>43</v>
+        <v>37.4</v>
       </c>
       <c r="L76">
-        <v>-2</v>
+        <v>-6.4</v>
       </c>
       <c r="M76">
-        <v>70</v>
+        <v>114.1</v>
       </c>
       <c r="N76" t="str">
         <v>BOX 460 - B_465</v>
@@ -5108,12 +5333,15 @@
         <v/>
       </c>
       <c r="T76" t="str">
+        <v>Minimal</v>
+      </c>
+      <c r="U76" t="str">
         <v/>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>box-500-b-501-isola-onda-zaha-hadid-architects</v>
+        <v>FEB-076</v>
       </c>
       <c r="B77" t="str">
         <v>Isola Onda - Zaha Hadid Architects</v>
@@ -5122,7 +5350,7 @@
         <v>cucine</v>
       </c>
       <c r="D77" t="str">
-        <v>Isola Onda - Zaha Hadid Architects — pieza de la colección Febal Casa, sección CASA 04 - A-MARE.</v>
+        <v>Isola Onda - Zaha Hadid Architects — elemento della collezione Febal Casa, sezione CASA 04 - A-MARE.</v>
       </c>
       <c r="E77" t="str">
         <v/>
@@ -5131,7 +5359,7 @@
         <v/>
       </c>
       <c r="G77" t="str">
-        <v>isola, onda, zaha, hadid, architects, cucine, cocina, cocinas, cucina, kitchen, isla, casa, pieza, coleccion, febal, seccion, mare</v>
+        <v>isola, onda, zaha, hadid, architects, cucine, cocina, cocinas, cucina, kitchen, isla, casa, elemento, collezione, febal, sezione, mare</v>
       </c>
       <c r="H77" t="str">
         <v/>
@@ -5140,16 +5368,16 @@
         <v>CASA 04 - A-MARE</v>
       </c>
       <c r="J77" t="str">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="K77">
-        <v>92</v>
+        <v>5.5</v>
       </c>
       <c r="L77">
-        <v>-25</v>
+        <v>-17.7</v>
       </c>
       <c r="M77">
-        <v>70</v>
+        <v>57.6</v>
       </c>
       <c r="N77" t="str">
         <v>BOX 500 - B_501</v>
@@ -5170,12 +5398,15 @@
         <v/>
       </c>
       <c r="T77" t="str">
+        <v>Contemporaneo</v>
+      </c>
+      <c r="U77" t="str">
         <v/>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v>box-500-b-502-sistema-origina-anta-square</v>
+        <v>FEB-077</v>
       </c>
       <c r="B78" t="str">
         <v>Sistema Origina anta Square</v>
@@ -5202,16 +5433,16 @@
         <v>CASA 04 - A-MARE</v>
       </c>
       <c r="J78" t="str">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="K78">
-        <v>26</v>
+        <v>10.2</v>
       </c>
       <c r="L78">
-        <v>-15</v>
+        <v>0.2</v>
       </c>
       <c r="M78">
-        <v>70</v>
+        <v>83.6</v>
       </c>
       <c r="N78" t="str">
         <v>BOX 500 - B_502</v>
@@ -5232,12 +5463,15 @@
         <v/>
       </c>
       <c r="T78" t="str">
+        <v>Contemporaneo</v>
+      </c>
+      <c r="U78" t="str">
         <v/>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="str">
-        <v>box-500-b-503-sistema-origina-anta-square</v>
+        <v>FEB-078</v>
       </c>
       <c r="B79" t="str">
         <v>Sistema Origina anta Square</v>
@@ -5288,18 +5522,21 @@
         <v>sistemi-modulari</v>
       </c>
       <c r="R79" t="str">
-        <v>TRUE</v>
+        <v>FALSE</v>
       </c>
       <c r="S79" t="str">
         <v/>
       </c>
       <c r="T79" t="str">
+        <v>Contemporaneo</v>
+      </c>
+      <c r="U79" t="str">
         <v/>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="str">
-        <v>box-600-b-601-armadio-profile-leather</v>
+        <v>FEB-079</v>
       </c>
       <c r="B80" t="str">
         <v>Armadio Profile/ Leather</v>
@@ -5329,13 +5566,13 @@
         <v>26</v>
       </c>
       <c r="K80">
-        <v>-58</v>
+        <v>-64.3</v>
       </c>
       <c r="L80">
-        <v>6</v>
+        <v>-2.6</v>
       </c>
       <c r="M80">
-        <v>70</v>
+        <v>90.2</v>
       </c>
       <c r="N80" t="str">
         <v>BOX 600 - B_601</v>
@@ -5356,12 +5593,15 @@
         <v/>
       </c>
       <c r="T80" t="str">
+        <v>Classico elegante</v>
+      </c>
+      <c r="U80" t="str">
         <v/>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>box-600-b-602-armadio-profile-leather</v>
+        <v>FEB-080</v>
       </c>
       <c r="B81" t="str">
         <v>Armadio Profile/ Leather</v>
@@ -5412,18 +5652,21 @@
         <v>armadi</v>
       </c>
       <c r="R81" t="str">
-        <v>TRUE</v>
+        <v>FALSE</v>
       </c>
       <c r="S81" t="str">
         <v/>
       </c>
       <c r="T81" t="str">
+        <v>Classico elegante</v>
+      </c>
+      <c r="U81" t="str">
         <v/>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="str">
-        <v>box-600-b-603-armadio-profile-solid</v>
+        <v>FEB-081</v>
       </c>
       <c r="B82" t="str">
         <v>Armadio Profile/ Solid</v>
@@ -5450,16 +5693,16 @@
         <v>GALLERIA</v>
       </c>
       <c r="J82" t="str">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="K82">
-        <v>85</v>
+        <v>153.6</v>
       </c>
       <c r="L82">
-        <v>1</v>
+        <v>-1.7</v>
       </c>
       <c r="M82">
-        <v>70</v>
+        <v>130</v>
       </c>
       <c r="N82" t="str">
         <v>BOX 600 - B_603</v>
@@ -5480,12 +5723,15 @@
         <v/>
       </c>
       <c r="T82" t="str">
+        <v>Contemporaneo</v>
+      </c>
+      <c r="U82" t="str">
         <v/>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="str">
-        <v>box-600-b-604-armadio-profile-solid</v>
+        <v>FEB-082</v>
       </c>
       <c r="B83" t="str">
         <v>Armadio Profile/ Solid</v>
@@ -5536,18 +5782,21 @@
         <v>armadi</v>
       </c>
       <c r="R83" t="str">
-        <v>TRUE</v>
+        <v>FALSE</v>
       </c>
       <c r="S83" t="str">
         <v/>
       </c>
       <c r="T83" t="str">
+        <v>Contemporaneo</v>
+      </c>
+      <c r="U83" t="str">
         <v/>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="str">
-        <v>box-600-b-605-armadio-profile-reflex</v>
+        <v>FEB-083</v>
       </c>
       <c r="B84" t="str">
         <v>Armadio Profile/ Reflex</v>
@@ -5577,13 +5826,13 @@
         <v>31</v>
       </c>
       <c r="K84">
-        <v>-179</v>
+        <v>-177.3</v>
       </c>
       <c r="L84">
-        <v>-5</v>
+        <v>-3.6</v>
       </c>
       <c r="M84">
-        <v>70</v>
+        <v>63.7</v>
       </c>
       <c r="N84" t="str">
         <v>BOX 600 - B_605</v>
@@ -5604,12 +5853,15 @@
         <v/>
       </c>
       <c r="T84" t="str">
+        <v>Contemporaneo</v>
+      </c>
+      <c r="U84" t="str">
         <v/>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="str">
-        <v>box-600-b-607-armadio-battente-aurora</v>
+        <v>FEB-084</v>
       </c>
       <c r="B85" t="str">
         <v>Armadio battente Aurora</v>
@@ -5636,16 +5888,16 @@
         <v>GALLERIA</v>
       </c>
       <c r="J85" t="str">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="K85">
-        <v>-92</v>
+        <v>-5.6</v>
       </c>
       <c r="L85">
-        <v>3</v>
+        <v>-9.3</v>
       </c>
       <c r="M85">
-        <v>70</v>
+        <v>130</v>
       </c>
       <c r="N85" t="str">
         <v>BOX 600 - B_607</v>
@@ -5666,12 +5918,15 @@
         <v/>
       </c>
       <c r="T85" t="str">
+        <v>Contemporaneo</v>
+      </c>
+      <c r="U85" t="str">
         <v/>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="str">
-        <v>box-620-b-621-cucina-anta-telaio-alluminio-vetro</v>
+        <v>FEB-085</v>
       </c>
       <c r="B86" t="str">
         <v>Cucina Anta Telaio Alluminio vetro</v>
@@ -5698,16 +5953,16 @@
         <v>GALLERIA</v>
       </c>
       <c r="J86" t="str">
-        <v>31</v>
+        <v>80-opening</v>
       </c>
       <c r="K86">
-        <v>18</v>
+        <v>19.3</v>
       </c>
       <c r="L86">
-        <v>-15</v>
+        <v>-30.5</v>
       </c>
       <c r="M86">
-        <v>70</v>
+        <v>87.6</v>
       </c>
       <c r="N86" t="str">
         <v>BOX 620 - B_621</v>
@@ -5728,12 +5983,15 @@
         <v/>
       </c>
       <c r="T86" t="str">
+        <v>Contemporaneo</v>
+      </c>
+      <c r="U86" t="str">
         <v/>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="str">
-        <v>box-620-b-622-armadio-barret</v>
+        <v>FEB-086</v>
       </c>
       <c r="B87" t="str">
         <v>Armadio Barret</v>
@@ -5760,16 +6018,16 @@
         <v>GALLERIA</v>
       </c>
       <c r="J87" t="str">
-        <v>31</v>
+        <v>83</v>
       </c>
       <c r="K87">
-        <v>-27</v>
+        <v>31.4</v>
       </c>
       <c r="L87">
-        <v>2</v>
+        <v>-6.3</v>
       </c>
       <c r="M87">
-        <v>70</v>
+        <v>130</v>
       </c>
       <c r="N87" t="str">
         <v>BOX 620 - B_622</v>
@@ -5790,12 +6048,15 @@
         <v/>
       </c>
       <c r="T87" t="str">
+        <v>Minimal</v>
+      </c>
+      <c r="U87" t="str">
         <v/>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="str">
-        <v>box-620-b-623-sgabello-lola</v>
+        <v>FEB-087</v>
       </c>
       <c r="B88" t="str">
         <v>Sgabello Lola</v>
@@ -5825,13 +6086,13 @@
         <v>31</v>
       </c>
       <c r="K88">
-        <v>6</v>
+        <v>4.6</v>
       </c>
       <c r="L88">
-        <v>-29</v>
+        <v>-32.4</v>
       </c>
       <c r="M88">
-        <v>70</v>
+        <v>67.3</v>
       </c>
       <c r="N88" t="str">
         <v>BOX 620 - B_623</v>
@@ -5852,12 +6113,15 @@
         <v/>
       </c>
       <c r="T88" t="str">
+        <v>Caldo accogliente, Minimal</v>
+      </c>
+      <c r="U88" t="str">
         <v/>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="str">
-        <v>box-640-b-641-armadio-lumia</v>
+        <v>FEB-088</v>
       </c>
       <c r="B89" t="str">
         <v>Armadio Lumia</v>
@@ -5887,13 +6151,13 @@
         <v>88-open</v>
       </c>
       <c r="K89">
-        <v>55</v>
+        <v>-116.8</v>
       </c>
       <c r="L89">
-        <v>-2</v>
+        <v>0.4</v>
       </c>
       <c r="M89">
-        <v>70</v>
+        <v>130</v>
       </c>
       <c r="N89" t="str">
         <v>BOX 640 - B_641</v>
@@ -5914,12 +6178,15 @@
         <v/>
       </c>
       <c r="T89" t="str">
+        <v>Classico elegante</v>
+      </c>
+      <c r="U89" t="str">
         <v/>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="str">
-        <v>box-640-b-642-armadio-lumia</v>
+        <v>FEB-089</v>
       </c>
       <c r="B90" t="str">
         <v>Armadio Lumia</v>
@@ -5970,18 +6237,21 @@
         <v>armadi</v>
       </c>
       <c r="R90" t="str">
-        <v>TRUE</v>
+        <v>FALSE</v>
       </c>
       <c r="S90" t="str">
         <v/>
       </c>
       <c r="T90" t="str">
+        <v>Classico elegante</v>
+      </c>
+      <c r="U90" t="str">
         <v/>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="str">
-        <v>box-640-b-643-armadio-lewitt-plus</v>
+        <v>FEB-090</v>
       </c>
       <c r="B91" t="str">
         <v>Armadio Lewitt Plus</v>
@@ -6008,16 +6278,16 @@
         <v>GALLERIA</v>
       </c>
       <c r="J91" t="str">
-        <v>85</v>
+        <v>86-open</v>
       </c>
       <c r="K91">
-        <v>163</v>
+        <v>157.3</v>
       </c>
       <c r="L91">
-        <v>-4</v>
+        <v>-12.2</v>
       </c>
       <c r="M91">
-        <v>70</v>
+        <v>103.1</v>
       </c>
       <c r="N91" t="str">
         <v>BOX 640 - B_643</v>
@@ -6038,12 +6308,15 @@
         <v/>
       </c>
       <c r="T91" t="str">
+        <v>Contemporaneo</v>
+      </c>
+      <c r="U91" t="str">
         <v/>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="str">
-        <v>box-640-b-644-tavolo-madeira</v>
+        <v>FEB-091</v>
       </c>
       <c r="B92" t="str">
         <v>Tavolo Madeira</v>
@@ -6055,10 +6328,10 @@
         <v>L'armonioso intreccio di archi definisce un tavolo unico, protagonista di ogni ambiente. Le gambe inclinate e sovrapposte formano un disegno geometrico di grande impatto visivo che gioca con la tridimensionalità ottenendo un risultato perfetto nato dall'eleganza, dall'equilibrio e dalla leggerezza dei volumi. La base in metallo è disponibile in finitura Ottone Scuro, Nero, Antracite e Sabbia. Il piano è di forma rotonda, ovale fisso o allungabile ed è configurabile in Cristallo Lucido, Cristallo Velvet, Superceramica, Supermarmo opaco, Supermarmo lucido e legno Impiallacciato. La versione fissa può essere arricchita con il piano centrotavola girevole, un dispositivo rotante che permette di condividere facilmente cibi e oggetti con tutti i commensali.</v>
       </c>
       <c r="E92" t="str">
-        <v/>
+        <v>bianco/sabbia</v>
       </c>
       <c r="F92" t="str">
-        <v/>
+        <v>supermarmo opaco, metallo</v>
       </c>
       <c r="G92" t="str">
         <v>tavolo, madeira, tavoli, mesa, mesas, table, comedor, dall, piano, cristallo, lucido, supermarmo, armonioso, intreccio, archi, definisce, unico, protagonista</v>
@@ -6073,13 +6346,13 @@
         <v>88-open</v>
       </c>
       <c r="K92">
-        <v>62</v>
+        <v>61.4</v>
       </c>
       <c r="L92">
-        <v>-30</v>
+        <v>-28.6</v>
       </c>
       <c r="M92">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="N92" t="str">
         <v>BOX 640 - B_644</v>
@@ -6097,15 +6370,18 @@
         <v>TRUE</v>
       </c>
       <c r="S92" t="str">
-        <v/>
+        <v>rotondo o ovale, fisso o allungabile</v>
       </c>
       <c r="T92" t="str">
+        <v>Contemporaneo, Classico elegante</v>
+      </c>
+      <c r="U92" t="str">
         <v/>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="str">
-        <v>box-640-b-645-sedia-dea</v>
+        <v>FEB-092</v>
       </c>
       <c r="B93" t="str">
         <v>Sedia Dea</v>
@@ -6132,16 +6408,16 @@
         <v>GALLERIA</v>
       </c>
       <c r="J93" t="str">
-        <v>88-open</v>
+        <v>84</v>
       </c>
       <c r="K93">
-        <v>89</v>
+        <v>128.2</v>
       </c>
       <c r="L93">
-        <v>-47</v>
+        <v>-35.6</v>
       </c>
       <c r="M93">
-        <v>70</v>
+        <v>54.1</v>
       </c>
       <c r="N93" t="str">
         <v>BOX 640 - B_645</v>
@@ -6162,12 +6438,15 @@
         <v/>
       </c>
       <c r="T93" t="str">
+        <v>Classico elegante, Caldo accogliente</v>
+      </c>
+      <c r="U93" t="str">
         <v/>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="str">
-        <v>box-660-b-664-tavolo-daniel</v>
+        <v>FEB-093</v>
       </c>
       <c r="B94" t="str">
         <v>Tavolo Daniel</v>
@@ -6197,13 +6476,13 @@
         <v>91</v>
       </c>
       <c r="K94">
-        <v>69</v>
+        <v>74.8</v>
       </c>
       <c r="L94">
-        <v>-31</v>
+        <v>-29</v>
       </c>
       <c r="M94">
-        <v>70</v>
+        <v>95</v>
       </c>
       <c r="N94" t="str">
         <v>BOX 660 - B_664</v>
@@ -6224,12 +6503,15 @@
         <v/>
       </c>
       <c r="T94" t="str">
+        <v>Classico elegante</v>
+      </c>
+      <c r="U94" t="str">
         <v/>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="str">
-        <v>box-660-b-665-sedia-dea</v>
+        <v>FEB-094</v>
       </c>
       <c r="B95" t="str">
         <v>Sedia Dea</v>
@@ -6241,10 +6523,10 @@
         <v>La sedia Dea è perfetta per progetti raffinati in ogni dettaglio. La linearità delle gambe in metallo verniciato disponibile nelle finiture Ottone scuro, Antracite, Nero e Sabbia è ammorbidita dalle forme curve e accoglienti della seduta e dello schienale, arricchite da un prezioso tocco sartoriale che si rivela con il grazioso movimento di pieghe che enfatizza i volumi e il senso di comfort. Dea è una sedia di valore che cattura inevitabilmente l'ammirazione di chiunque la osservi.</v>
       </c>
       <c r="E95" t="str">
-        <v/>
+        <v>tortora</v>
       </c>
       <c r="F95" t="str">
-        <v/>
+        <v>tessuto</v>
       </c>
       <c r="G95" t="str">
         <v>sedia, dea, sedie, silla, sillas, chair, asiento, perfetta, progetti, raffinati, ogni, dettaglio, linearita, gambe, metallo, verniciato, disponibile, nelle</v>
@@ -6259,13 +6541,13 @@
         <v>91</v>
       </c>
       <c r="K95">
-        <v>121</v>
+        <v>131.4</v>
       </c>
       <c r="L95">
-        <v>-33</v>
+        <v>-4.6</v>
       </c>
       <c r="M95">
-        <v>70</v>
+        <v>82</v>
       </c>
       <c r="N95" t="str">
         <v>BOX 660 - B_665</v>
@@ -6286,12 +6568,15 @@
         <v/>
       </c>
       <c r="T95" t="str">
-        <v/>
+        <v>Classico elegante, Caldo accogliente</v>
+      </c>
+      <c r="U95" t="str">
+        <v>Nero</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="str">
-        <v>box-660-b-667-boiserie</v>
+        <v>FEB-095</v>
       </c>
       <c r="B96" t="str">
         <v>Boiserie</v>
@@ -6318,16 +6603,16 @@
         <v>GALLERIA</v>
       </c>
       <c r="J96" t="str">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="K96">
-        <v>25</v>
+        <v>132.6</v>
       </c>
       <c r="L96">
-        <v>10</v>
+        <v>-13.4</v>
       </c>
       <c r="M96">
-        <v>70</v>
+        <v>80.2</v>
       </c>
       <c r="N96" t="str">
         <v>BOX 660 - B_667</v>
@@ -6348,12 +6633,405 @@
         <v/>
       </c>
       <c r="T96" t="str">
+        <v>Contemporaneo</v>
+      </c>
+      <c r="U96" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="str">
+        <v>FEB-096</v>
+      </c>
+      <c r="B97" t="str">
+        <v>Armadio Profile/ Leather</v>
+      </c>
+      <c r="C97" t="str">
+        <v>armadi</v>
+      </c>
+      <c r="D97" t="str">
+        <v>L'armadio con anta battente Profile Leather di Febal Casa combina eleganza materica e funzionalità per un arredo raffinato.</v>
+      </c>
+      <c r="E97" t="str">
+        <v/>
+      </c>
+      <c r="F97" t="str">
+        <v/>
+      </c>
+      <c r="G97" t="str">
+        <v>armadio, profile/, leather, armadi, armario, armarios, closet, ropero, wardrobe, cabina armadio, vestidor, anta, battente, profile, febal, casa, combina, eleganza, materica, funzionalita, arredo</v>
+      </c>
+      <c r="H97" t="str">
+        <v/>
+      </c>
+      <c r="I97" t="str">
+        <v>CASA 01 - AUTENTICA</v>
+      </c>
+      <c r="J97" t="str">
+        <v>38</v>
+      </c>
+      <c r="K97">
+        <v>7</v>
+      </c>
+      <c r="L97">
+        <v>1.7</v>
+      </c>
+      <c r="M97">
+        <v>65.6</v>
+      </c>
+      <c r="N97" t="str">
+        <v>BOX 180 - B_192</v>
+      </c>
+      <c r="O97" t="str">
+        <v>assets/febal-casa/placeholder-product.png</v>
+      </c>
+      <c r="P97" t="str">
+        <v>https://www.febalcasa.com/it/tipologia/armadi/ante/battente/profile-leather/</v>
+      </c>
+      <c r="Q97" t="str">
+        <v>armadi</v>
+      </c>
+      <c r="R97" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="S97" t="str">
+        <v/>
+      </c>
+      <c r="T97" t="str">
+        <v/>
+      </c>
+      <c r="U97" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="str">
+        <v>FEB-097</v>
+      </c>
+      <c r="B98" t="str">
+        <v>Cabina Armadio Telaio</v>
+      </c>
+      <c r="C98" t="str">
+        <v>armadi</v>
+      </c>
+      <c r="D98" t="str">
+        <v>Una cabina armadio dal design architettonico, con struttura in metallo e pannelli in vetro per un guardaroba con effetto leggero e luminoso.</v>
+      </c>
+      <c r="E98" t="str">
+        <v/>
+      </c>
+      <c r="F98" t="str">
+        <v/>
+      </c>
+      <c r="G98" t="str">
+        <v>cabina, armadio, telaio, armadi, armario, armarios, closet, ropero, wardrobe, cabina armadio, vestidor, design, architettonico, struttura, metallo, pannelli, vetro, guardaroba, effetto, leggero, luminoso</v>
+      </c>
+      <c r="H98" t="str">
+        <v/>
+      </c>
+      <c r="I98" t="str">
+        <v>CASA 01 - AUTENTICA</v>
+      </c>
+      <c r="J98" t="str">
+        <v>38</v>
+      </c>
+      <c r="K98">
+        <v>83.8</v>
+      </c>
+      <c r="L98">
+        <v>-1.3</v>
+      </c>
+      <c r="M98">
+        <v>65.5</v>
+      </c>
+      <c r="N98" t="str">
+        <v>BOX 180 - B_193</v>
+      </c>
+      <c r="O98" t="str">
+        <v>assets/febal-casa/products/telaio.jpg</v>
+      </c>
+      <c r="P98" t="str">
+        <v>https://www.febalcasa.com/it/tipologia/cabine-armadio/telaio/</v>
+      </c>
+      <c r="Q98" t="str">
+        <v>armadi</v>
+      </c>
+      <c r="R98" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="S98" t="str">
+        <v/>
+      </c>
+      <c r="T98" t="str">
+        <v/>
+      </c>
+      <c r="U98" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="str">
+        <v>FEB-098</v>
+      </c>
+      <c r="B99" t="str">
+        <v>Cassettiera Square</v>
+      </c>
+      <c r="C99" t="str">
+        <v>cassettiere</v>
+      </c>
+      <c r="D99" t="str">
+        <v>Cassettiera Square — elemento della collezione Febal Casa, sezione CASA 01 - AUTENTICA.</v>
+      </c>
+      <c r="E99" t="str">
+        <v/>
+      </c>
+      <c r="F99" t="str">
+        <v/>
+      </c>
+      <c r="G99" t="str">
+        <v>cassettiera, square, cassettiere, comoda, cómoda, cómodas, cajonera, dresser, casa, elemento, collezione, febal, sezione, autentica</v>
+      </c>
+      <c r="H99" t="str">
+        <v/>
+      </c>
+      <c r="I99" t="str">
+        <v>CASA 01 - AUTENTICA</v>
+      </c>
+      <c r="J99" t="str">
+        <v>36</v>
+      </c>
+      <c r="K99">
+        <v>-14.1</v>
+      </c>
+      <c r="L99">
+        <v>-49</v>
+      </c>
+      <c r="M99">
+        <v>108.6</v>
+      </c>
+      <c r="N99" t="str">
+        <v>BOX 180 - B_194</v>
+      </c>
+      <c r="O99" t="str">
+        <v>assets/febal-casa/products/square.jpg</v>
+      </c>
+      <c r="P99" t="str">
+        <v>https://www.febalcasa.com/it/tipologia/armadi/cassettiere/square/</v>
+      </c>
+      <c r="Q99" t="str">
+        <v>cassettiere</v>
+      </c>
+      <c r="R99" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="S99" t="str">
+        <v/>
+      </c>
+      <c r="T99" t="str">
+        <v/>
+      </c>
+      <c r="U99" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="str">
+        <v>FEB-099</v>
+      </c>
+      <c r="B100" t="str">
+        <v>Armadio Barret con Portale</v>
+      </c>
+      <c r="C100" t="str">
+        <v>armadi</v>
+      </c>
+      <c r="D100" t="str">
+        <v>Scopri gli armadi a ponte con passaggio Febal Casa: soluzioni architettoniche che ottimizzano lo spazio con stile e funzionalità.</v>
+      </c>
+      <c r="E100" t="str">
+        <v/>
+      </c>
+      <c r="F100" t="str">
+        <v/>
+      </c>
+      <c r="G100" t="str">
+        <v>armadio, barret, portale, armadi, armario, armarios, closet, ropero, wardrobe, cabina armadio, vestidor, scopri, ponte, passaggio, febal, casa, soluzioni, architettoniche, ottimizzano, spazio, stile, funzionalita</v>
+      </c>
+      <c r="H100" t="str">
+        <v/>
+      </c>
+      <c r="I100" t="str">
+        <v>CASA 01 - AUTENTICA</v>
+      </c>
+      <c r="J100" t="str">
+        <v>33</v>
+      </c>
+      <c r="K100">
+        <v>38.1</v>
+      </c>
+      <c r="L100">
+        <v>-0.9</v>
+      </c>
+      <c r="M100">
+        <v>119.2</v>
+      </c>
+      <c r="N100" t="str">
+        <v>BOX 190 - B_191</v>
+      </c>
+      <c r="O100" t="str">
+        <v>assets/febal-casa/placeholder-product.png</v>
+      </c>
+      <c r="P100" t="str">
+        <v>https://www.febalcasa.com/it/tipologia/armadi/ispirazioni/armadio-con-passaggio-con-ponte/</v>
+      </c>
+      <c r="Q100" t="str">
+        <v>armadi</v>
+      </c>
+      <c r="R100" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="S100" t="str">
+        <v/>
+      </c>
+      <c r="T100" t="str">
+        <v/>
+      </c>
+      <c r="U100" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="str">
+        <v>FEB-100</v>
+      </c>
+      <c r="B101" t="str">
+        <v>Armadio Halley</v>
+      </c>
+      <c r="C101" t="str">
+        <v>armadi</v>
+      </c>
+      <c r="D101" t="str">
+        <v>L’armadio con anta scorrevole Halley gioca sui contrasti cromatici e materici esaltati dalla luce led integrata che unisce efficacia ed estetica.</v>
+      </c>
+      <c r="E101" t="str">
+        <v/>
+      </c>
+      <c r="F101" t="str">
+        <v/>
+      </c>
+      <c r="G101" t="str">
+        <v>armadio, halley, armadi, armario, armarios, closet, ropero, wardrobe, cabina armadio, vestidor, anta, scorrevole, gioca, contrasti, cromatici, materici, esaltati, luce, integrata, unisce</v>
+      </c>
+      <c r="H101" t="str">
+        <v/>
+      </c>
+      <c r="I101" t="str">
+        <v>CASA 03 - AUDACE</v>
+      </c>
+      <c r="J101" t="str">
+        <v>47</v>
+      </c>
+      <c r="K101">
+        <v>-151.8</v>
+      </c>
+      <c r="L101">
+        <v>-4.3</v>
+      </c>
+      <c r="M101">
+        <v>130</v>
+      </c>
+      <c r="N101" t="str">
+        <v>BOX 340 - B_341</v>
+      </c>
+      <c r="O101" t="str">
+        <v>assets/febal-casa/products/halley.jpg</v>
+      </c>
+      <c r="P101" t="str">
+        <v>https://www.febalcasa.com/it/prodotti/febal-notte-armadio-scorrevole-halley-01/</v>
+      </c>
+      <c r="Q101" t="str">
+        <v>armadi</v>
+      </c>
+      <c r="R101" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="S101" t="str">
+        <v/>
+      </c>
+      <c r="T101" t="str">
+        <v/>
+      </c>
+      <c r="U101" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="str">
+        <v>FEB-101</v>
+      </c>
+      <c r="B102" t="str">
+        <v>Letto Arden</v>
+      </c>
+      <c r="C102" t="str">
+        <v>camera da letto</v>
+      </c>
+      <c r="D102" t="str">
+        <v>Allure di Febal Casa: letto imbottito con testata dalle linee verticali che evocano il fusto di una colonna. Discrezione e carattere per la camera da letto matrimoniale.</v>
+      </c>
+      <c r="E102" t="str">
+        <v/>
+      </c>
+      <c r="F102" t="str">
+        <v/>
+      </c>
+      <c r="G102" t="str">
+        <v>letto, arden, camera da letto, cama, dormitorio, bed, recamara, recámara, habitacion, gruppo notte, allure, febal, casa, imbottito, testata, linee, verticali, evocano, fusto, colonna, discrezione</v>
+      </c>
+      <c r="H102" t="str">
+        <v/>
+      </c>
+      <c r="I102" t="str">
+        <v>CASA 03 - AUDACE</v>
+      </c>
+      <c r="J102" t="str">
+        <v>46</v>
+      </c>
+      <c r="K102">
+        <v>144.3</v>
+      </c>
+      <c r="L102">
+        <v>-36.6</v>
+      </c>
+      <c r="M102">
+        <v>91.6</v>
+      </c>
+      <c r="N102" t="str">
+        <v>BOX 340 - B_343</v>
+      </c>
+      <c r="O102" t="str">
+        <v>assets/febal-casa/products/allure.jpg</v>
+      </c>
+      <c r="P102" t="str">
+        <v>https://www.febalcasa.com/it/prodotti/allure/</v>
+      </c>
+      <c r="Q102" t="str">
+        <v>camera-da-letto</v>
+      </c>
+      <c r="R102" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="S102" t="str">
+        <v/>
+      </c>
+      <c r="T102" t="str">
+        <v/>
+      </c>
+      <c r="U102" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:T96"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:U102"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>